<commit_message>
chore(data): daily ingest 2026-09-12
NORMAL/SLOWING · GDPNow 4.42 · NY 2.26
</commit_message>
<xml_diff>
--- a/data/cache/nyfed_nowcast_raw.xlsx
+++ b/data/cache/nyfed_nowcast_raw.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\SHARE\drf\TimeSeries\products\Nowcast\automated_nowcast\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C142E9D-8DAB-4E9A-A6FB-776E4380DBAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B10012E2-17FB-4AA7-95D1-F92A85E7D170}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{ABCE1506-5AF9-4A77-93FF-F8162337FD42}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{ABCE1506-5AF9-4A77-93FF-F8162337FD42}"/>
   </bookViews>
   <sheets>
     <sheet name="New York Fed Nowcast" sheetId="3" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="62">
   <si>
     <t>Forecast Date</t>
   </si>
@@ -1841,7 +1841,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1670CA3-538E-42E7-9E1F-A6A72E94A86A}">
-  <dimension ref="A1:Q203"/>
+  <dimension ref="A1:Q204"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.140625" customWidth="1"/>
@@ -4223,6 +4223,17 @@
         <v>2.2599999999999998</v>
       </c>
       <c r="Q203">
+        <v>2.5099999999999998</v>
+      </c>
+    </row>
+    <row r="204" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A204" s="2">
+        <v>46276</v>
+      </c>
+      <c r="P204">
+        <v>2.2599999999999998</v>
+      </c>
+      <c r="Q204">
         <v>2.5099999999999998</v>
       </c>
     </row>
@@ -4247,7 +4258,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{596092BD-1EF6-4EC0-96F0-3BB4B0DA037F}">
-  <dimension ref="A1:I203"/>
+  <dimension ref="A1:I204"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.42578125" customWidth="1"/>
@@ -7039,6 +7050,20 @@
         <v>2.2599999999999998</v>
       </c>
       <c r="E203">
+        <v>2.5099999999999998</v>
+      </c>
+    </row>
+    <row r="204" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A204" s="2">
+        <v>46276</v>
+      </c>
+      <c r="B204" t="s">
+        <v>61</v>
+      </c>
+      <c r="D204">
+        <v>2.2599999999999998</v>
+      </c>
+      <c r="E204">
         <v>2.5099999999999998</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): daily ingest 2026-09-19
NORMAL/SLOWING · GDPNow 5.08 · NY 2.33
</commit_message>
<xml_diff>
--- a/data/cache/nyfed_nowcast_raw.xlsx
+++ b/data/cache/nyfed_nowcast_raw.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\SHARE\drf\TimeSeries\products\Nowcast\automated_nowcast\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B10012E2-17FB-4AA7-95D1-F92A85E7D170}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A24D6A5-3236-47E9-B4DD-75AEAE1BBBB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{ABCE1506-5AF9-4A77-93FF-F8162337FD42}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="62">
   <si>
     <t>Forecast Date</t>
   </si>
@@ -1841,7 +1841,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1670CA3-538E-42E7-9E1F-A6A72E94A86A}">
-  <dimension ref="A1:Q204"/>
+  <dimension ref="A1:Q205"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.140625" customWidth="1"/>
@@ -4235,6 +4235,17 @@
       </c>
       <c r="Q204">
         <v>2.5099999999999998</v>
+      </c>
+    </row>
+    <row r="205" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A205" s="2">
+        <v>46283</v>
+      </c>
+      <c r="P205">
+        <v>2.33</v>
+      </c>
+      <c r="Q205">
+        <v>2.6</v>
       </c>
     </row>
   </sheetData>
@@ -4258,7 +4269,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{596092BD-1EF6-4EC0-96F0-3BB4B0DA037F}">
-  <dimension ref="A1:I204"/>
+  <dimension ref="A1:I205"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.42578125" customWidth="1"/>
@@ -7065,6 +7076,20 @@
       </c>
       <c r="E204">
         <v>2.5099999999999998</v>
+      </c>
+    </row>
+    <row r="205" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A205" s="2">
+        <v>46283</v>
+      </c>
+      <c r="B205" t="s">
+        <v>61</v>
+      </c>
+      <c r="D205">
+        <v>2.33</v>
+      </c>
+      <c r="E205">
+        <v>2.6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data): daily ingest 2026-10-05
NORMAL/SLOWING · GDPNow 3.68 · NY 2.46
</commit_message>
<xml_diff>
--- a/data/cache/nyfed_nowcast_raw.xlsx
+++ b/data/cache/nyfed_nowcast_raw.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\SHARE\drf\TimeSeries\products\Nowcast\automated_nowcast\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A24D6A5-3236-47E9-B4DD-75AEAE1BBBB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{386C3A18-A0EE-49C5-9E14-E30951C56DC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{ABCE1506-5AF9-4A77-93FF-F8162337FD42}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="51840" windowHeight="21120" activeTab="2" xr2:uid="{ABCE1506-5AF9-4A77-93FF-F8162337FD42}"/>
   </bookViews>
   <sheets>
     <sheet name="New York Fed Nowcast" sheetId="3" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="62">
   <si>
     <t>Forecast Date</t>
   </si>
@@ -1604,15 +1604,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4E1EDB4-3E22-4B96-9108-06AEDE165285}">
   <dimension ref="B1:I42"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="24.85546875" style="5" customWidth="1"/>
-    <col min="2" max="2" width="129.42578125" style="5" customWidth="1"/>
-    <col min="3" max="16384" width="9.140625" style="5"/>
+    <col min="1" max="1" width="24.81640625" style="5" customWidth="1"/>
+    <col min="2" max="2" width="129.453125" style="5" customWidth="1"/>
+    <col min="3" max="16384" width="9.1796875" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="2:9" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="2" spans="2:9" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B2" s="33" t="s">
         <v>13</v>
       </c>
@@ -1624,7 +1624,7 @@
       <c r="H2" s="33"/>
       <c r="I2" s="33"/>
     </row>
-    <row r="3" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B3" s="33"/>
       <c r="C3" s="33"/>
       <c r="D3" s="33"/>
@@ -1634,67 +1634,67 @@
       <c r="H3" s="33"/>
       <c r="I3" s="33"/>
     </row>
-    <row r="4" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B4" s="4" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="2:9" ht="31.5" x14ac:dyDescent="0.5">
+    <row r="8" spans="2:9" ht="31" x14ac:dyDescent="0.7">
       <c r="B8" s="24" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="2:9" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:9" ht="18.5" x14ac:dyDescent="0.45">
       <c r="B9" s="25" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B10" s="6"/>
     </row>
-    <row r="11" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B11" s="20" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="12" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B12" s="7" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="13" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B13" s="9" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="14" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B14" s="9" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="15" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B15" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B17" s="22" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B18" s="23" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="19" spans="2:7" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:7" ht="10.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C19" s="16"/>
       <c r="D19" s="16"/>
       <c r="E19" s="16"/>
       <c r="F19" s="16"/>
       <c r="G19" s="16"/>
     </row>
-    <row r="20" spans="2:7" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B20" s="19" t="s">
         <v>27</v>
       </c>
@@ -1703,7 +1703,7 @@
       <c r="E20" s="8"/>
       <c r="F20" s="8"/>
     </row>
-    <row r="21" spans="2:7" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B21" s="10" t="s">
         <v>28</v>
       </c>
@@ -1712,14 +1712,14 @@
       <c r="E21" s="8"/>
       <c r="F21" s="8"/>
     </row>
-    <row r="22" spans="2:7" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B22" s="10"/>
       <c r="C22" s="8"/>
       <c r="D22" s="8"/>
       <c r="E22" s="8"/>
       <c r="F22" s="8"/>
     </row>
-    <row r="23" spans="2:7" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B23" s="19" t="s">
         <v>29</v>
       </c>
@@ -1728,7 +1728,7 @@
       <c r="E23" s="8"/>
       <c r="F23" s="8"/>
     </row>
-    <row r="24" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B24" s="10" t="s">
         <v>36</v>
       </c>
@@ -1737,55 +1737,55 @@
       <c r="E24" s="8"/>
       <c r="F24" s="8"/>
     </row>
-    <row r="25" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B25" s="10"/>
       <c r="C25" s="8"/>
       <c r="D25" s="8"/>
       <c r="E25" s="8"/>
       <c r="F25" s="8"/>
     </row>
-    <row r="26" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B26" s="19" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="27" spans="2:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:7" ht="29" x14ac:dyDescent="0.35">
       <c r="B27" s="21" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="28" spans="2:7" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B28" s="21"/>
     </row>
-    <row r="29" spans="2:7" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:7" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B29" s="11" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="30" spans="2:7" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:7" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B30" s="13" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="31" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B31" s="18" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="32" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B32" s="18" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="33" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B33" s="17" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="34" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B34" s="13"/>
     </row>
-    <row r="35" spans="2:6" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:6" ht="13" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B35" s="14" t="s">
         <v>23</v>
       </c>
@@ -1794,7 +1794,7 @@
       <c r="E35" s="11"/>
       <c r="F35" s="11"/>
     </row>
-    <row r="36" spans="2:6" ht="16.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:6" ht="16.399999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B36" s="6" t="s">
         <v>24</v>
       </c>
@@ -1803,13 +1803,13 @@
       <c r="E36" s="12"/>
       <c r="F36" s="12"/>
     </row>
-    <row r="38" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C38" s="11"/>
       <c r="D38" s="11"/>
       <c r="E38" s="11"/>
       <c r="F38" s="11"/>
     </row>
-    <row r="42" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:6" x14ac:dyDescent="0.35">
       <c r="C42" s="15"/>
       <c r="D42" s="15"/>
     </row>
@@ -1841,14 +1841,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1670CA3-538E-42E7-9E1F-A6A72E94A86A}">
-  <dimension ref="A1:Q205"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:Q207"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="27.140625" customWidth="1"/>
+    <col min="1" max="1" width="27.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="2" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B2" s="29"/>
       <c r="C2" s="29"/>
       <c r="D2" s="29"/>
@@ -1857,7 +1857,7 @@
       <c r="G2" s="29"/>
       <c r="H2" s="29"/>
     </row>
-    <row r="3" spans="1:16" s="3" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:16" s="3" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B3" s="30" t="s">
         <v>25</v>
       </c>
@@ -1869,16 +1869,16 @@
       <c r="H3" s="31"/>
       <c r="I3" s="31"/>
     </row>
-    <row r="4" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="C4" s="32" t="s">
         <v>14</v>
       </c>
       <c r="D4" s="32"/>
     </row>
-    <row r="5" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A5"/>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>0</v>
       </c>
@@ -1928,7 +1928,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A7" s="2">
         <v>44897</v>
       </c>
@@ -1936,7 +1936,7 @@
         <v>1.79</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A8" s="2">
         <v>44904</v>
       </c>
@@ -1944,7 +1944,7 @@
         <v>1.76</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A9" s="2">
         <v>44911</v>
       </c>
@@ -1952,7 +1952,7 @@
         <v>1.58</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A10" s="2">
         <v>44918</v>
       </c>
@@ -1960,7 +1960,7 @@
         <v>1.33</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A11" s="2">
         <v>44925</v>
       </c>
@@ -1968,7 +1968,7 @@
         <v>1.31</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A12" s="2">
         <v>44932</v>
       </c>
@@ -1976,7 +1976,7 @@
         <v>1.57</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A13" s="2">
         <v>44939</v>
       </c>
@@ -1984,7 +1984,7 @@
         <v>1.64</v>
       </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A14" s="2">
         <v>44946</v>
       </c>
@@ -1992,7 +1992,7 @@
         <v>0.79</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A15" s="2">
         <v>44953</v>
       </c>
@@ -2000,7 +2000,7 @@
         <v>1.2</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A16" s="2">
         <v>44960</v>
       </c>
@@ -2008,7 +2008,7 @@
         <v>1.59</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" s="2">
         <v>44967</v>
       </c>
@@ -2016,7 +2016,7 @@
         <v>1.48</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" s="2">
         <v>44974</v>
       </c>
@@ -2024,7 +2024,7 @@
         <v>1.1399999999999999</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" s="2">
         <v>44981</v>
       </c>
@@ -2035,7 +2035,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" s="2">
         <v>44988</v>
       </c>
@@ -2046,7 +2046,7 @@
         <v>1.45</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" s="2">
         <v>44995</v>
       </c>
@@ -2057,7 +2057,7 @@
         <v>1.53</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" s="2">
         <v>45002</v>
       </c>
@@ -2068,7 +2068,7 @@
         <v>1.3</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" s="2">
         <v>45009</v>
       </c>
@@ -2079,7 +2079,7 @@
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A24" s="2">
         <v>45016</v>
       </c>
@@ -2090,7 +2090,7 @@
         <v>1.08</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A25" s="2">
         <v>45023</v>
       </c>
@@ -2101,7 +2101,7 @@
         <v>0.67</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A26" s="2">
         <v>45030</v>
       </c>
@@ -2112,7 +2112,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A27" s="2">
         <v>45037</v>
       </c>
@@ -2123,7 +2123,7 @@
         <v>1.1200000000000001</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A28" s="2">
         <v>45044</v>
       </c>
@@ -2134,7 +2134,7 @@
         <v>0.52</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A29" s="2">
         <v>45051</v>
       </c>
@@ -2142,7 +2142,7 @@
         <v>1.28</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A30" s="2">
         <v>45058</v>
       </c>
@@ -2150,7 +2150,7 @@
         <v>1.19</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A31" s="2">
         <v>45065</v>
       </c>
@@ -2158,7 +2158,7 @@
         <v>1.44</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A32" s="2">
         <v>45072</v>
       </c>
@@ -2169,7 +2169,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" s="2">
         <v>45079</v>
       </c>
@@ -2180,7 +2180,7 @@
         <v>1.96</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" s="2">
         <v>45086</v>
       </c>
@@ -2191,7 +2191,7 @@
         <v>1.9</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" s="2">
         <v>45093</v>
       </c>
@@ -2202,7 +2202,7 @@
         <v>1.81</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" s="2">
         <v>45100</v>
       </c>
@@ -2213,7 +2213,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" s="2">
         <v>45107</v>
       </c>
@@ -2224,7 +2224,7 @@
         <v>2.0699999999999998</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" s="2">
         <v>45114</v>
       </c>
@@ -2235,7 +2235,7 @@
         <v>1.53</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" s="2">
         <v>45121</v>
       </c>
@@ -2246,7 +2246,7 @@
         <v>1.51</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" s="2">
         <v>45128</v>
       </c>
@@ -2257,7 +2257,7 @@
         <v>1.25</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" s="2">
         <v>45135</v>
       </c>
@@ -2268,7 +2268,7 @@
         <v>1.93</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" s="2">
         <v>45142</v>
       </c>
@@ -2276,7 +2276,7 @@
         <v>1.81</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43" s="2">
         <v>45149</v>
       </c>
@@ -2284,7 +2284,7 @@
         <v>1.7</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" s="2">
         <v>45156</v>
       </c>
@@ -2292,7 +2292,7 @@
         <v>2.34</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" s="2">
         <v>45163</v>
       </c>
@@ -2300,7 +2300,7 @@
         <v>2.12</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A46" s="2">
         <v>45170</v>
       </c>
@@ -2311,7 +2311,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" s="2">
         <v>45177</v>
       </c>
@@ -2322,7 +2322,7 @@
         <v>2.29</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48" s="2">
         <v>45184</v>
       </c>
@@ -2333,7 +2333,7 @@
         <v>2.35</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A49" s="2">
         <v>45191</v>
       </c>
@@ -2344,7 +2344,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A50" s="2">
         <v>45198</v>
       </c>
@@ -2355,7 +2355,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A51" s="2">
         <v>45205</v>
       </c>
@@ -2366,7 +2366,7 @@
         <v>2.4039999999999999</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A52" s="2">
         <v>45212</v>
       </c>
@@ -2377,7 +2377,7 @@
         <v>2.34</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A53" s="2">
         <v>45219</v>
       </c>
@@ -2388,7 +2388,7 @@
         <v>2.27</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A54" s="2">
         <v>45226</v>
       </c>
@@ -2399,7 +2399,7 @@
         <v>2.79</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A55" s="2">
         <v>45233</v>
       </c>
@@ -2407,7 +2407,7 @@
         <v>2.41</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A56" s="2">
         <v>45240</v>
       </c>
@@ -2415,7 +2415,7 @@
         <v>2.5099999999999998</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A57" s="2">
         <v>45247</v>
       </c>
@@ -2423,7 +2423,7 @@
         <v>2.4500000000000002</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A58" s="2">
         <v>45254</v>
       </c>
@@ -2431,7 +2431,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A59" s="2">
         <v>45261</v>
       </c>
@@ -2442,7 +2442,7 @@
         <v>2.0499999999999998</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A60" s="2">
         <v>45268</v>
       </c>
@@ -2453,7 +2453,7 @@
         <v>2.13</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A61" s="2">
         <v>45275</v>
       </c>
@@ -2464,7 +2464,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A62" s="2">
         <v>45282</v>
       </c>
@@ -2475,7 +2475,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A63" s="2">
         <v>45289</v>
       </c>
@@ -2486,7 +2486,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A64" s="2">
         <v>45296</v>
       </c>
@@ -2497,7 +2497,7 @@
         <v>2.68</v>
       </c>
     </row>
-    <row r="65" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A65" s="2">
         <v>45303</v>
       </c>
@@ -2508,7 +2508,7 @@
         <v>2.4500000000000002</v>
       </c>
     </row>
-    <row r="66" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A66" s="2">
         <v>45310</v>
       </c>
@@ -2529,7 +2529,7 @@
       <c r="O66" s="26"/>
       <c r="P66" s="26"/>
     </row>
-    <row r="67" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A67" s="2">
         <v>45317</v>
       </c>
@@ -2550,7 +2550,7 @@
       <c r="O67" s="26"/>
       <c r="P67" s="26"/>
     </row>
-    <row r="68" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A68" s="2">
         <v>45324</v>
       </c>
@@ -2569,7 +2569,7 @@
       <c r="O68" s="26"/>
       <c r="P68" s="26"/>
     </row>
-    <row r="69" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A69" s="2">
         <v>45331</v>
       </c>
@@ -2588,7 +2588,7 @@
       <c r="O69" s="26"/>
       <c r="P69" s="26"/>
     </row>
-    <row r="70" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A70" s="2">
         <v>45338</v>
       </c>
@@ -2607,7 +2607,7 @@
       <c r="O70" s="26"/>
       <c r="P70" s="26"/>
     </row>
-    <row r="71" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A71" s="2">
         <v>45345</v>
       </c>
@@ -2626,7 +2626,7 @@
       <c r="O71" s="26"/>
       <c r="P71" s="26"/>
     </row>
-    <row r="72" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A72" s="2">
         <v>45352</v>
       </c>
@@ -2647,7 +2647,7 @@
       <c r="O72" s="26"/>
       <c r="P72" s="26"/>
     </row>
-    <row r="73" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A73" s="2">
         <v>45359</v>
       </c>
@@ -2668,7 +2668,7 @@
       <c r="O73" s="26"/>
       <c r="P73" s="26"/>
     </row>
-    <row r="74" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A74" s="2">
         <v>45366</v>
       </c>
@@ -2689,7 +2689,7 @@
       <c r="O74" s="26"/>
       <c r="P74" s="26"/>
     </row>
-    <row r="75" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A75" s="2">
         <v>45373</v>
       </c>
@@ -2710,7 +2710,7 @@
       <c r="O75" s="26"/>
       <c r="P75" s="26"/>
     </row>
-    <row r="76" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A76" s="2">
         <v>45380</v>
       </c>
@@ -2731,7 +2731,7 @@
       <c r="O76" s="26"/>
       <c r="P76" s="26"/>
     </row>
-    <row r="77" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A77" s="2">
         <v>45387</v>
       </c>
@@ -2752,7 +2752,7 @@
       <c r="O77" s="26"/>
       <c r="P77" s="26"/>
     </row>
-    <row r="78" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A78" s="2">
         <v>45394</v>
       </c>
@@ -2773,7 +2773,7 @@
       <c r="O78" s="26"/>
       <c r="P78" s="26"/>
     </row>
-    <row r="79" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A79" s="2">
         <v>45401</v>
       </c>
@@ -2794,7 +2794,7 @@
       <c r="O79" s="26"/>
       <c r="P79" s="26"/>
     </row>
-    <row r="80" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A80" s="2">
         <v>45408</v>
       </c>
@@ -2815,7 +2815,7 @@
       <c r="O80" s="26"/>
       <c r="P80" s="26"/>
     </row>
-    <row r="81" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A81" s="2">
         <v>45415</v>
       </c>
@@ -2834,7 +2834,7 @@
       <c r="O81" s="26"/>
       <c r="P81" s="26"/>
     </row>
-    <row r="82" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A82" s="2">
         <v>45422</v>
       </c>
@@ -2853,7 +2853,7 @@
       <c r="O82" s="26"/>
       <c r="P82" s="26"/>
     </row>
-    <row r="83" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A83" s="2">
         <v>45429</v>
       </c>
@@ -2872,7 +2872,7 @@
       <c r="O83" s="26"/>
       <c r="P83" s="26"/>
     </row>
-    <row r="84" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A84" s="2">
         <v>45436</v>
       </c>
@@ -2891,7 +2891,7 @@
       <c r="O84" s="26"/>
       <c r="P84" s="26"/>
     </row>
-    <row r="85" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A85" s="2">
         <v>45443</v>
       </c>
@@ -2912,7 +2912,7 @@
       <c r="O85" s="26"/>
       <c r="P85" s="26"/>
     </row>
-    <row r="86" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A86" s="2">
         <v>45450</v>
       </c>
@@ -2933,7 +2933,7 @@
       <c r="O86" s="26"/>
       <c r="P86" s="26"/>
     </row>
-    <row r="87" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A87" s="2">
         <v>45457</v>
       </c>
@@ -2954,7 +2954,7 @@
       <c r="O87" s="26"/>
       <c r="P87" s="26"/>
     </row>
-    <row r="88" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A88" s="2">
         <v>45464</v>
       </c>
@@ -2975,7 +2975,7 @@
       <c r="O88" s="26"/>
       <c r="P88" s="26"/>
     </row>
-    <row r="89" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A89" s="2">
         <v>45471</v>
       </c>
@@ -2996,7 +2996,7 @@
       <c r="O89" s="26"/>
       <c r="P89" s="26"/>
     </row>
-    <row r="90" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A90" s="2">
         <v>45478</v>
       </c>
@@ -3017,7 +3017,7 @@
       <c r="O90" s="26"/>
       <c r="P90" s="26"/>
     </row>
-    <row r="91" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A91" s="2">
         <v>45485</v>
       </c>
@@ -3038,7 +3038,7 @@
       <c r="O91" s="26"/>
       <c r="P91" s="26"/>
     </row>
-    <row r="92" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A92" s="2">
         <v>45492</v>
       </c>
@@ -3059,7 +3059,7 @@
       <c r="O92" s="26"/>
       <c r="P92" s="26"/>
     </row>
-    <row r="93" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A93" s="2">
         <v>45499</v>
       </c>
@@ -3080,7 +3080,7 @@
       <c r="O93" s="26"/>
       <c r="P93" s="26"/>
     </row>
-    <row r="94" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A94" s="2">
         <v>45506</v>
       </c>
@@ -3099,7 +3099,7 @@
       <c r="O94" s="26"/>
       <c r="P94" s="26"/>
     </row>
-    <row r="95" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A95" s="2">
         <v>45513</v>
       </c>
@@ -3107,7 +3107,7 @@
         <v>2.238</v>
       </c>
     </row>
-    <row r="96" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A96" s="2">
         <v>45520</v>
       </c>
@@ -3115,7 +3115,7 @@
         <v>1.84</v>
       </c>
     </row>
-    <row r="97" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A97" s="2">
         <v>45527</v>
       </c>
@@ -3123,7 +3123,7 @@
         <v>1.9410000000000001</v>
       </c>
     </row>
-    <row r="98" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A98" s="2">
         <v>45534</v>
       </c>
@@ -3134,7 +3134,7 @@
         <v>2.1160000000000001</v>
       </c>
     </row>
-    <row r="99" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A99" s="2">
         <v>45541</v>
       </c>
@@ -3145,7 +3145,7 @@
         <v>2.2130000000000001</v>
       </c>
     </row>
-    <row r="100" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A100" s="2">
         <v>45548</v>
       </c>
@@ -3156,7 +3156,7 @@
         <v>2.1749999999999998</v>
       </c>
     </row>
-    <row r="101" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A101" s="2">
         <v>45555</v>
       </c>
@@ -3167,7 +3167,7 @@
         <v>2.74</v>
       </c>
     </row>
-    <row r="102" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A102" s="2">
         <v>45562</v>
       </c>
@@ -3178,7 +3178,7 @@
         <v>2.7970000000000002</v>
       </c>
     </row>
-    <row r="103" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A103" s="2">
         <v>45569</v>
       </c>
@@ -3189,7 +3189,7 @@
         <v>2.7629999999999999</v>
       </c>
     </row>
-    <row r="104" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A104" s="2">
         <v>45576</v>
       </c>
@@ -3200,7 +3200,7 @@
         <v>2.7530000000000001</v>
       </c>
     </row>
-    <row r="105" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A105" s="2">
         <v>45583</v>
       </c>
@@ -3211,7 +3211,7 @@
         <v>2.6070000000000002</v>
       </c>
     </row>
-    <row r="106" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A106" s="2">
         <v>45590</v>
       </c>
@@ -3222,7 +3222,7 @@
         <v>2.4649999999999999</v>
       </c>
     </row>
-    <row r="107" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A107" s="2">
         <v>45597</v>
       </c>
@@ -3233,7 +3233,7 @@
         <v>2.0070000000000001</v>
       </c>
     </row>
-    <row r="108" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A108" s="2">
         <v>45604</v>
       </c>
@@ -3241,7 +3241,7 @@
         <v>2.0590000000000002</v>
       </c>
     </row>
-    <row r="109" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A109" s="2">
         <v>45611</v>
       </c>
@@ -3249,7 +3249,7 @@
         <v>2.0640000000000001</v>
       </c>
     </row>
-    <row r="110" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A110" s="2">
         <v>45618</v>
       </c>
@@ -3257,7 +3257,7 @@
         <v>1.909</v>
       </c>
     </row>
-    <row r="111" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A111" s="2">
         <v>45625</v>
       </c>
@@ -3265,7 +3265,7 @@
         <v>1.8049999999999999</v>
       </c>
     </row>
-    <row r="112" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A112" s="2">
         <v>45632</v>
       </c>
@@ -3276,7 +3276,7 @@
         <v>2.3769999999999998</v>
       </c>
     </row>
-    <row r="113" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A113" s="2">
         <v>45639</v>
       </c>
@@ -3287,7 +3287,7 @@
         <v>2.2909999999999999</v>
       </c>
     </row>
-    <row r="114" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A114" s="2">
         <v>45646</v>
       </c>
@@ -3298,7 +3298,7 @@
         <v>2.1269999999999998</v>
       </c>
     </row>
-    <row r="115" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A115" s="2">
         <v>45653</v>
       </c>
@@ -3309,7 +3309,7 @@
         <v>2.0819999999999999</v>
       </c>
     </row>
-    <row r="116" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A116" s="2">
         <v>45660</v>
       </c>
@@ -3320,7 +3320,7 @@
         <v>2.2080000000000002</v>
       </c>
     </row>
-    <row r="117" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A117" s="2">
         <v>45667</v>
       </c>
@@ -3331,7 +3331,7 @@
         <v>2.738</v>
       </c>
     </row>
-    <row r="118" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A118" s="2">
         <v>45674</v>
       </c>
@@ -3342,7 +3342,7 @@
         <v>2.9994999999999998</v>
       </c>
     </row>
-    <row r="119" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A119" s="2">
         <v>45681</v>
       </c>
@@ -3353,7 +3353,7 @@
         <v>2.9994999999999998</v>
       </c>
     </row>
-    <row r="120" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A120" s="2">
         <v>45688</v>
       </c>
@@ -3364,7 +3364,7 @@
         <v>2.915</v>
       </c>
     </row>
-    <row r="121" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A121" s="2">
         <v>45695</v>
       </c>
@@ -3372,7 +3372,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="122" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A122" s="2">
         <v>45702</v>
       </c>
@@ -3380,7 +3380,7 @@
         <v>3.0150000000000001</v>
       </c>
     </row>
-    <row r="123" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A123" s="2">
         <v>45709</v>
       </c>
@@ -3388,7 +3388,7 @@
         <v>2.9460000000000002</v>
       </c>
     </row>
-    <row r="124" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A124" s="2">
         <v>45716</v>
       </c>
@@ -3399,7 +3399,7 @@
         <v>2.8490000000000002</v>
       </c>
     </row>
-    <row r="125" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A125" s="2">
         <v>45723</v>
       </c>
@@ -3410,7 +3410,7 @@
         <v>2.5750000000000002</v>
       </c>
     </row>
-    <row r="126" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A126" s="2">
         <v>45730</v>
       </c>
@@ -3421,7 +3421,7 @@
         <v>2.6579999999999999</v>
       </c>
     </row>
-    <row r="127" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A127" s="2">
         <v>45737</v>
       </c>
@@ -3432,7 +3432,7 @@
         <v>2.641</v>
       </c>
     </row>
-    <row r="128" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A128" s="2">
         <v>45744</v>
       </c>
@@ -3443,7 +3443,7 @@
         <v>2.629</v>
       </c>
     </row>
-    <row r="129" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A129" s="2">
         <v>45751</v>
       </c>
@@ -3454,7 +3454,7 @@
         <v>2.4380000000000002</v>
       </c>
     </row>
-    <row r="130" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A130" s="2">
         <v>45758</v>
       </c>
@@ -3465,7 +3465,7 @@
         <v>2.6179999999999999</v>
       </c>
     </row>
-    <row r="131" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A131" s="2">
         <v>45765</v>
       </c>
@@ -3476,7 +3476,7 @@
         <v>2.605</v>
       </c>
     </row>
-    <row r="132" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A132" s="2">
         <v>45772</v>
       </c>
@@ -3487,7 +3487,7 @@
         <v>2.7149999999999999</v>
       </c>
     </row>
-    <row r="133" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A133" s="2">
         <v>45779</v>
       </c>
@@ -3498,7 +3498,7 @@
         <v>2.335</v>
       </c>
     </row>
-    <row r="134" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A134" s="2">
         <v>45786</v>
       </c>
@@ -3506,7 +3506,7 @@
         <v>2.4249999999999998</v>
       </c>
     </row>
-    <row r="135" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A135" s="2">
         <v>45793</v>
       </c>
@@ -3514,7 +3514,7 @@
         <v>2.3460000000000001</v>
       </c>
     </row>
-    <row r="136" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A136" s="2">
         <v>45800</v>
       </c>
@@ -3522,7 +3522,7 @@
         <v>2.4289999999999998</v>
       </c>
     </row>
-    <row r="137" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A137" s="2">
         <v>45807</v>
       </c>
@@ -3533,7 +3533,7 @@
         <v>2.5379999999999998</v>
       </c>
     </row>
-    <row r="138" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A138" s="2">
         <v>45814</v>
       </c>
@@ -3544,7 +3544,7 @@
         <v>2.3980000000000001</v>
       </c>
     </row>
-    <row r="139" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A139" s="2">
         <v>45821</v>
       </c>
@@ -3555,7 +3555,7 @@
         <v>2.504</v>
       </c>
     </row>
-    <row r="140" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A140" s="2">
         <v>45828</v>
       </c>
@@ -3566,7 +3566,7 @@
         <v>2.0609999999999999</v>
       </c>
     </row>
-    <row r="141" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A141" s="2">
         <v>45835</v>
       </c>
@@ -3577,7 +3577,7 @@
         <v>1.917</v>
       </c>
     </row>
-    <row r="142" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A142" s="2">
         <v>45842</v>
       </c>
@@ -3588,7 +3588,7 @@
         <v>1.7809999999999999</v>
       </c>
     </row>
-    <row r="143" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A143" s="2">
         <v>45849</v>
       </c>
@@ -3599,7 +3599,7 @@
         <v>1.78</v>
       </c>
     </row>
-    <row r="144" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A144" s="2">
         <v>45856</v>
       </c>
@@ -3610,7 +3610,7 @@
         <v>2.44</v>
       </c>
     </row>
-    <row r="145" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A145" s="2">
         <v>45863</v>
       </c>
@@ -3621,7 +3621,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="146" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A146" s="2">
         <v>45870</v>
       </c>
@@ -3632,7 +3632,7 @@
         <v>2.12</v>
       </c>
     </row>
-    <row r="147" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A147" s="2">
         <v>45877</v>
       </c>
@@ -3640,7 +3640,7 @@
         <v>2.02</v>
       </c>
     </row>
-    <row r="148" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A148" s="2">
         <v>45884</v>
       </c>
@@ -3648,7 +3648,7 @@
         <v>2.06</v>
       </c>
     </row>
-    <row r="149" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A149" s="2">
         <v>45891</v>
       </c>
@@ -3656,7 +3656,7 @@
         <v>2.0099999999999998</v>
       </c>
     </row>
-    <row r="150" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A150" s="2">
         <v>45898</v>
       </c>
@@ -3667,7 +3667,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="151" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A151" s="2">
         <v>45905</v>
       </c>
@@ -3678,7 +3678,7 @@
         <v>2.2799999999999998</v>
       </c>
     </row>
-    <row r="152" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A152" s="2">
         <v>45912</v>
       </c>
@@ -3689,7 +3689,7 @@
         <v>2.16</v>
       </c>
     </row>
-    <row r="153" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A153" s="2">
         <v>45919</v>
       </c>
@@ -3700,7 +3700,7 @@
         <v>2.1800000000000002</v>
       </c>
     </row>
-    <row r="154" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A154" s="2">
         <v>45926</v>
       </c>
@@ -3711,7 +3711,7 @@
         <v>2.46</v>
       </c>
     </row>
-    <row r="155" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A155" s="2">
         <v>45933</v>
       </c>
@@ -3722,7 +3722,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="156" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A156" s="2">
         <v>45940</v>
       </c>
@@ -3733,7 +3733,7 @@
         <v>2.23</v>
       </c>
     </row>
-    <row r="157" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A157" s="2">
         <v>45947</v>
       </c>
@@ -3744,7 +3744,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="158" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A158" s="2">
         <v>45954</v>
       </c>
@@ -3755,7 +3755,7 @@
         <v>2.2599999999999998</v>
       </c>
     </row>
-    <row r="159" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A159" s="2">
         <v>45961</v>
       </c>
@@ -3766,7 +3766,7 @@
         <v>2.2599999999999998</v>
       </c>
     </row>
-    <row r="160" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A160" s="2">
         <v>45968</v>
       </c>
@@ -3777,7 +3777,7 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="161" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A161" s="2">
         <v>45975</v>
       </c>
@@ -3788,7 +3788,7 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="162" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A162" s="2">
         <v>45982</v>
       </c>
@@ -3799,7 +3799,7 @@
         <v>2.31</v>
       </c>
     </row>
-    <row r="163" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A163" s="2">
         <v>45989</v>
       </c>
@@ -3813,7 +3813,7 @@
         <v>2.66</v>
       </c>
     </row>
-    <row r="164" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A164" s="2">
         <v>45996</v>
       </c>
@@ -3824,7 +3824,7 @@
         <v>2.2200000000000002</v>
       </c>
     </row>
-    <row r="165" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A165" s="2">
         <v>46003</v>
       </c>
@@ -3835,7 +3835,7 @@
         <v>2.2400000000000002</v>
       </c>
     </row>
-    <row r="166" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A166" s="2">
         <v>46010</v>
       </c>
@@ -3846,7 +3846,7 @@
         <v>2.11</v>
       </c>
     </row>
-    <row r="167" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A167" s="2">
         <v>46017</v>
       </c>
@@ -3857,7 +3857,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="168" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A168" s="2">
         <v>46024</v>
       </c>
@@ -3868,7 +3868,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="169" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A169" s="2">
         <v>46031</v>
       </c>
@@ -3879,7 +3879,7 @@
         <v>2.61</v>
       </c>
     </row>
-    <row r="170" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A170" s="2">
         <v>46038</v>
       </c>
@@ -3890,7 +3890,7 @@
         <v>2.75</v>
       </c>
     </row>
-    <row r="171" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A171" s="2">
         <v>46045</v>
       </c>
@@ -3901,7 +3901,7 @@
         <v>2.73</v>
       </c>
     </row>
-    <row r="172" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A172" s="2">
         <v>46052</v>
       </c>
@@ -3912,7 +3912,7 @@
         <v>2.73</v>
       </c>
     </row>
-    <row r="173" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A173" s="2">
         <v>46059</v>
       </c>
@@ -3923,7 +3923,7 @@
         <v>2.59</v>
       </c>
     </row>
-    <row r="174" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A174" s="2">
         <v>46066</v>
       </c>
@@ -3934,7 +3934,7 @@
         <v>2.63</v>
       </c>
     </row>
-    <row r="175" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A175" s="2">
         <v>46073</v>
       </c>
@@ -3945,7 +3945,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="176" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A176" s="2">
         <v>46080</v>
       </c>
@@ -3953,7 +3953,7 @@
         <v>2.38</v>
       </c>
     </row>
-    <row r="177" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A177" s="2">
         <v>46087</v>
       </c>
@@ -3961,7 +3961,7 @@
         <v>2.23</v>
       </c>
     </row>
-    <row r="178" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A178" s="2">
         <v>46094</v>
       </c>
@@ -3972,7 +3972,7 @@
         <v>2.68</v>
       </c>
     </row>
-    <row r="179" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A179" s="2">
         <v>46101</v>
       </c>
@@ -3983,7 +3983,7 @@
         <v>2.67</v>
       </c>
     </row>
-    <row r="180" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A180" s="2">
         <v>46108</v>
       </c>
@@ -3994,7 +3994,7 @@
         <v>2.68</v>
       </c>
     </row>
-    <row r="181" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A181" s="2">
         <v>46115</v>
       </c>
@@ -4005,7 +4005,7 @@
         <v>2.82</v>
       </c>
     </row>
-    <row r="182" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A182" s="2">
         <v>46122</v>
       </c>
@@ -4016,7 +4016,7 @@
         <v>2.6</v>
       </c>
     </row>
-    <row r="183" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A183" s="2">
         <v>46129</v>
       </c>
@@ -4027,7 +4027,7 @@
         <v>2.75</v>
       </c>
     </row>
-    <row r="184" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A184" s="2">
         <v>46136</v>
       </c>
@@ -4038,7 +4038,7 @@
         <v>2.81</v>
       </c>
     </row>
-    <row r="185" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A185" s="2">
         <v>46143</v>
       </c>
@@ -4049,7 +4049,7 @@
         <v>2.52</v>
       </c>
     </row>
-    <row r="186" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A186" s="2">
         <v>46150</v>
       </c>
@@ -4057,7 +4057,7 @@
         <v>2.59</v>
       </c>
     </row>
-    <row r="187" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A187" s="2">
         <v>46157</v>
       </c>
@@ -4065,7 +4065,7 @@
         <v>2.61</v>
       </c>
     </row>
-    <row r="188" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A188" s="2">
         <v>46164</v>
       </c>
@@ -4073,7 +4073,7 @@
         <v>2.61</v>
       </c>
     </row>
-    <row r="189" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A189" s="2">
         <v>46171</v>
       </c>
@@ -4084,7 +4084,7 @@
         <v>2.36</v>
       </c>
     </row>
-    <row r="190" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A190" s="2">
         <v>46178</v>
       </c>
@@ -4095,7 +4095,7 @@
         <v>2.4700000000000002</v>
       </c>
     </row>
-    <row r="191" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A191" s="2">
         <v>46185</v>
       </c>
@@ -4106,7 +4106,7 @@
         <v>2.46</v>
       </c>
     </row>
-    <row r="192" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A192" s="2">
         <v>46192</v>
       </c>
@@ -4117,7 +4117,7 @@
         <v>2.4500000000000002</v>
       </c>
     </row>
-    <row r="193" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A193" s="2">
         <v>46199</v>
       </c>
@@ -4128,7 +4128,7 @@
         <v>2.42</v>
       </c>
     </row>
-    <row r="194" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A194" s="2">
         <v>46206</v>
       </c>
@@ -4139,7 +4139,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="195" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A195" s="2">
         <v>46213</v>
       </c>
@@ -4150,7 +4150,7 @@
         <v>2.36</v>
       </c>
     </row>
-    <row r="196" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A196" s="2">
         <v>46220</v>
       </c>
@@ -4161,7 +4161,7 @@
         <v>2.6</v>
       </c>
     </row>
-    <row r="197" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A197" s="2">
         <v>46227</v>
       </c>
@@ -4172,7 +4172,7 @@
         <v>2.62</v>
       </c>
     </row>
-    <row r="198" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A198" s="2">
         <v>46234</v>
       </c>
@@ -4183,7 +4183,7 @@
         <v>2.52</v>
       </c>
     </row>
-    <row r="199" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A199" s="2">
         <v>46241</v>
       </c>
@@ -4191,7 +4191,7 @@
         <v>2.2400000000000002</v>
       </c>
     </row>
-    <row r="200" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A200" s="2">
         <v>46248</v>
       </c>
@@ -4199,7 +4199,7 @@
         <v>2.14</v>
       </c>
     </row>
-    <row r="201" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A201" s="2">
         <v>46255</v>
       </c>
@@ -4207,7 +4207,7 @@
         <v>2.27</v>
       </c>
     </row>
-    <row r="202" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A202" s="2">
         <v>46262</v>
       </c>
@@ -4215,7 +4215,7 @@
         <v>2.2200000000000002</v>
       </c>
     </row>
-    <row r="203" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A203" s="2">
         <v>46269</v>
       </c>
@@ -4226,7 +4226,7 @@
         <v>2.5099999999999998</v>
       </c>
     </row>
-    <row r="204" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A204" s="2">
         <v>46276</v>
       </c>
@@ -4237,7 +4237,7 @@
         <v>2.5099999999999998</v>
       </c>
     </row>
-    <row r="205" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A205" s="2">
         <v>46283</v>
       </c>
@@ -4246,6 +4246,28 @@
       </c>
       <c r="Q205">
         <v>2.6</v>
+      </c>
+    </row>
+    <row r="206" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A206" s="2">
+        <v>46290</v>
+      </c>
+      <c r="P206">
+        <v>2.33</v>
+      </c>
+      <c r="Q206">
+        <v>2.6</v>
+      </c>
+    </row>
+    <row r="207" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A207" s="2">
+        <v>46297</v>
+      </c>
+      <c r="P207">
+        <v>2.46</v>
+      </c>
+      <c r="Q207">
+        <v>2.54</v>
       </c>
     </row>
   </sheetData>
@@ -4269,18 +4291,18 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{596092BD-1EF6-4EC0-96F0-3BB4B0DA037F}">
-  <dimension ref="A1:I205"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:I207"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="23.42578125" customWidth="1"/>
-    <col min="2" max="2" width="18.85546875" customWidth="1"/>
-    <col min="3" max="3" width="24.85546875" customWidth="1"/>
-    <col min="4" max="4" width="25.140625" customWidth="1"/>
-    <col min="5" max="5" width="23.42578125" customWidth="1"/>
+    <col min="1" max="1" width="23.453125" customWidth="1"/>
+    <col min="2" max="2" width="18.81640625" customWidth="1"/>
+    <col min="3" max="3" width="24.81640625" customWidth="1"/>
+    <col min="4" max="4" width="25.1796875" customWidth="1"/>
+    <col min="5" max="5" width="23.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="2" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B2" s="29"/>
       <c r="C2" s="29"/>
       <c r="D2" s="29"/>
@@ -4289,7 +4311,7 @@
       <c r="G2" s="29"/>
       <c r="H2" s="29"/>
     </row>
-    <row r="3" spans="1:9" s="3" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" s="3" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B3" s="30" t="s">
         <v>25</v>
       </c>
@@ -4301,16 +4323,16 @@
       <c r="H3" s="31"/>
       <c r="I3" s="31"/>
     </row>
-    <row r="4" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="C4" s="32" t="s">
         <v>14</v>
       </c>
       <c r="D4" s="32"/>
     </row>
-    <row r="5" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A5"/>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -4327,7 +4349,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" s="2">
         <v>44897</v>
       </c>
@@ -4338,7 +4360,7 @@
         <v>1.79</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" s="2">
         <v>44904</v>
       </c>
@@ -4349,7 +4371,7 @@
         <v>1.76</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" s="2">
         <v>44911</v>
       </c>
@@ -4360,7 +4382,7 @@
         <v>1.58</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" s="2">
         <v>44918</v>
       </c>
@@ -4371,7 +4393,7 @@
         <v>1.33</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" s="2">
         <v>44925</v>
       </c>
@@ -4382,7 +4404,7 @@
         <v>1.31</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" s="2">
         <v>44932</v>
       </c>
@@ -4393,7 +4415,7 @@
         <v>1.57</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" s="2">
         <v>44939</v>
       </c>
@@ -4404,7 +4426,7 @@
         <v>1.64</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" s="2">
         <v>44946</v>
       </c>
@@ -4415,7 +4437,7 @@
         <v>0.79</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" s="2">
         <v>44953</v>
       </c>
@@ -4426,7 +4448,7 @@
         <v>1.2</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" s="2">
         <v>44960</v>
       </c>
@@ -4437,7 +4459,7 @@
         <v>1.59</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" s="2">
         <v>44967</v>
       </c>
@@ -4448,7 +4470,7 @@
         <v>1.48</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" s="2">
         <v>44974</v>
       </c>
@@ -4459,7 +4481,7 @@
         <v>1.1399999999999999</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" s="2">
         <v>44981</v>
       </c>
@@ -4473,7 +4495,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" s="2">
         <v>44988</v>
       </c>
@@ -4487,7 +4509,7 @@
         <v>1.45</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" s="2">
         <v>44995</v>
       </c>
@@ -4501,7 +4523,7 @@
         <v>1.53</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" s="2">
         <v>45002</v>
       </c>
@@ -4515,7 +4537,7 @@
         <v>1.3</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" s="2">
         <v>45009</v>
       </c>
@@ -4529,7 +4551,7 @@
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" s="2">
         <v>45016</v>
       </c>
@@ -4543,7 +4565,7 @@
         <v>1.08</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" s="2">
         <v>45023</v>
       </c>
@@ -4557,7 +4579,7 @@
         <v>0.67</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" s="2">
         <v>45030</v>
       </c>
@@ -4571,7 +4593,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" s="2">
         <v>45037</v>
       </c>
@@ -4585,7 +4607,7 @@
         <v>1.1200000000000001</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" s="2">
         <v>45044</v>
       </c>
@@ -4599,7 +4621,7 @@
         <v>0.52</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" s="2">
         <v>45051</v>
       </c>
@@ -4610,7 +4632,7 @@
         <v>1.28</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" s="2">
         <v>45058</v>
       </c>
@@ -4621,7 +4643,7 @@
         <v>1.19</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" s="2">
         <v>45065</v>
       </c>
@@ -4632,7 +4654,7 @@
         <v>1.44</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" s="2">
         <v>45072</v>
       </c>
@@ -4646,7 +4668,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" s="2">
         <v>45079</v>
       </c>
@@ -4660,7 +4682,7 @@
         <v>1.96</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" s="2">
         <v>45086</v>
       </c>
@@ -4674,7 +4696,7 @@
         <v>1.9</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" s="2">
         <v>45093</v>
       </c>
@@ -4688,7 +4710,7 @@
         <v>1.81</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" s="2">
         <v>45100</v>
       </c>
@@ -4702,7 +4724,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" s="2">
         <v>45107</v>
       </c>
@@ -4716,7 +4738,7 @@
         <v>2.0699999999999998</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" s="2">
         <v>45114</v>
       </c>
@@ -4730,7 +4752,7 @@
         <v>1.53</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" s="2">
         <v>45121</v>
       </c>
@@ -4744,7 +4766,7 @@
         <v>1.51</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" s="2">
         <v>45128</v>
       </c>
@@ -4758,7 +4780,7 @@
         <v>1.25</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" s="2">
         <v>45135</v>
       </c>
@@ -4772,7 +4794,7 @@
         <v>1.93</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" s="2">
         <v>45142</v>
       </c>
@@ -4783,7 +4805,7 @@
         <v>1.81</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43" s="2">
         <v>45149</v>
       </c>
@@ -4794,7 +4816,7 @@
         <v>1.7</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" s="2">
         <v>45156</v>
       </c>
@@ -4805,7 +4827,7 @@
         <v>2.34</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" s="2">
         <v>45163</v>
       </c>
@@ -4816,7 +4838,7 @@
         <v>2.12</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A46" s="2">
         <v>45170</v>
       </c>
@@ -4830,7 +4852,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" s="2">
         <v>45177</v>
       </c>
@@ -4844,7 +4866,7 @@
         <v>2.29</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48" s="2">
         <v>45184</v>
       </c>
@@ -4858,7 +4880,7 @@
         <v>2.35</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A49" s="2">
         <v>45191</v>
       </c>
@@ -4872,7 +4894,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A50" s="2">
         <v>45198</v>
       </c>
@@ -4886,7 +4908,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A51" s="2">
         <v>45205</v>
       </c>
@@ -4900,7 +4922,7 @@
         <v>2.4039999999999999</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A52" s="2">
         <v>45212</v>
       </c>
@@ -4914,7 +4936,7 @@
         <v>2.34</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A53" s="2">
         <v>45219</v>
       </c>
@@ -4928,7 +4950,7 @@
         <v>2.27</v>
       </c>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A54" s="2">
         <v>45226</v>
       </c>
@@ -4942,7 +4964,7 @@
         <v>2.79</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A55" s="2">
         <v>45233</v>
       </c>
@@ -4953,7 +4975,7 @@
         <v>2.41</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A56" s="2">
         <v>45240</v>
       </c>
@@ -4964,7 +4986,7 @@
         <v>2.5099999999999998</v>
       </c>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A57" s="2">
         <v>45247</v>
       </c>
@@ -4975,7 +4997,7 @@
         <v>2.4500000000000002</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A58" s="2">
         <v>45254</v>
       </c>
@@ -4986,7 +5008,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A59" s="2">
         <v>45261</v>
       </c>
@@ -5000,7 +5022,7 @@
         <v>2.0499999999999998</v>
       </c>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A60" s="2">
         <v>45268</v>
       </c>
@@ -5014,7 +5036,7 @@
         <v>2.13</v>
       </c>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A61" s="2">
         <v>45275</v>
       </c>
@@ -5028,7 +5050,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A62" s="2">
         <v>45282</v>
       </c>
@@ -5042,7 +5064,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A63" s="2">
         <v>45289</v>
       </c>
@@ -5056,7 +5078,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A64" s="2">
         <v>45296</v>
       </c>
@@ -5073,7 +5095,7 @@
       <c r="F64" s="26"/>
       <c r="G64" s="26"/>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A65" s="2">
         <v>45303</v>
       </c>
@@ -5090,7 +5112,7 @@
       <c r="F65" s="26"/>
       <c r="G65" s="26"/>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A66" s="2">
         <v>45310</v>
       </c>
@@ -5107,7 +5129,7 @@
       <c r="F66" s="26"/>
       <c r="G66" s="26"/>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A67" s="2">
         <v>45317</v>
       </c>
@@ -5124,7 +5146,7 @@
       <c r="F67" s="26"/>
       <c r="G67" s="26"/>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A68" s="2">
         <v>45324</v>
       </c>
@@ -5139,7 +5161,7 @@
       <c r="F68" s="26"/>
       <c r="G68" s="26"/>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A69" s="2">
         <v>45331</v>
       </c>
@@ -5154,7 +5176,7 @@
       <c r="F69" s="26"/>
       <c r="G69" s="26"/>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A70" s="2">
         <v>45338</v>
       </c>
@@ -5169,7 +5191,7 @@
       <c r="F70" s="26"/>
       <c r="G70" s="26"/>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A71" s="2">
         <v>45345</v>
       </c>
@@ -5184,7 +5206,7 @@
       <c r="F71" s="26"/>
       <c r="G71" s="26"/>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A72" s="2">
         <v>45352</v>
       </c>
@@ -5201,7 +5223,7 @@
       <c r="F72" s="26"/>
       <c r="G72" s="26"/>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A73" s="2">
         <v>45359</v>
       </c>
@@ -5218,7 +5240,7 @@
       <c r="F73" s="26"/>
       <c r="G73" s="26"/>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A74" s="2">
         <v>45366</v>
       </c>
@@ -5232,7 +5254,7 @@
         <v>2.09</v>
       </c>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A75" s="2">
         <v>45373</v>
       </c>
@@ -5246,7 +5268,7 @@
         <v>2.19</v>
       </c>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A76" s="2">
         <v>45380</v>
       </c>
@@ -5263,7 +5285,7 @@
       <c r="F76" s="26"/>
       <c r="G76" s="26"/>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A77" s="2">
         <v>45387</v>
       </c>
@@ -5280,7 +5302,7 @@
       <c r="F77" s="26"/>
       <c r="G77" s="26"/>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A78" s="2">
         <v>45394</v>
       </c>
@@ -5297,7 +5319,7 @@
       <c r="F78" s="26"/>
       <c r="G78" s="26"/>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A79" s="2">
         <v>45401</v>
       </c>
@@ -5314,7 +5336,7 @@
       <c r="F79" s="26"/>
       <c r="G79" s="26"/>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A80" s="2">
         <v>45408</v>
       </c>
@@ -5331,7 +5353,7 @@
       <c r="F80" s="26"/>
       <c r="G80" s="26"/>
     </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A81" s="2">
         <v>45415</v>
       </c>
@@ -5346,7 +5368,7 @@
       <c r="F81" s="26"/>
       <c r="G81" s="26"/>
     </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A82" s="2">
         <v>45422</v>
       </c>
@@ -5361,7 +5383,7 @@
       <c r="F82" s="26"/>
       <c r="G82" s="26"/>
     </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A83" s="2">
         <v>45429</v>
       </c>
@@ -5376,7 +5398,7 @@
       <c r="F83" s="26"/>
       <c r="G83" s="26"/>
     </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A84" s="2">
         <v>45436</v>
       </c>
@@ -5391,7 +5413,7 @@
       <c r="F84" s="26"/>
       <c r="G84" s="26"/>
     </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A85" s="2">
         <v>45443</v>
       </c>
@@ -5408,7 +5430,7 @@
       <c r="F85" s="26"/>
       <c r="G85" s="26"/>
     </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A86" s="2">
         <v>45450</v>
       </c>
@@ -5425,7 +5447,7 @@
       <c r="F86" s="26"/>
       <c r="G86" s="26"/>
     </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A87" s="2">
         <v>45457</v>
       </c>
@@ -5442,7 +5464,7 @@
       <c r="F87" s="26"/>
       <c r="G87" s="26"/>
     </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A88" s="2">
         <v>45464</v>
       </c>
@@ -5459,7 +5481,7 @@
       <c r="F88" s="26"/>
       <c r="G88" s="26"/>
     </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A89" s="2">
         <v>45471</v>
       </c>
@@ -5476,7 +5498,7 @@
       <c r="F89" s="26"/>
       <c r="G89" s="26"/>
     </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A90" s="2">
         <v>45478</v>
       </c>
@@ -5493,7 +5515,7 @@
       <c r="F90" s="26"/>
       <c r="G90" s="26"/>
     </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A91" s="2">
         <v>45485</v>
       </c>
@@ -5510,7 +5532,7 @@
       <c r="F91" s="26"/>
       <c r="G91" s="26"/>
     </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A92" s="2">
         <v>45492</v>
       </c>
@@ -5527,7 +5549,7 @@
       <c r="F92" s="26"/>
       <c r="G92" s="26"/>
     </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A93" s="2">
         <v>45499</v>
       </c>
@@ -5544,7 +5566,7 @@
       <c r="F93" s="26"/>
       <c r="G93" s="26"/>
     </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A94" s="2">
         <v>45506</v>
       </c>
@@ -5559,7 +5581,7 @@
       <c r="F94" s="26"/>
       <c r="G94" s="26"/>
     </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A95" s="2">
         <v>45513</v>
       </c>
@@ -5574,7 +5596,7 @@
       <c r="F95" s="26"/>
       <c r="G95" s="26"/>
     </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A96" s="2">
         <v>45520</v>
       </c>
@@ -5589,7 +5611,7 @@
       <c r="F96" s="26"/>
       <c r="G96" s="26"/>
     </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A97" s="2">
         <v>45527</v>
       </c>
@@ -5604,7 +5626,7 @@
       <c r="F97" s="26"/>
       <c r="G97" s="26"/>
     </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A98" s="2">
         <v>45534</v>
       </c>
@@ -5621,7 +5643,7 @@
       <c r="F98" s="26"/>
       <c r="G98" s="26"/>
     </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A99" s="2">
         <v>45541</v>
       </c>
@@ -5638,7 +5660,7 @@
       <c r="F99" s="26"/>
       <c r="G99" s="26"/>
     </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A100" s="2">
         <v>45548</v>
       </c>
@@ -5655,7 +5677,7 @@
       <c r="F100" s="26"/>
       <c r="G100" s="26"/>
     </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A101" s="2">
         <v>45555</v>
       </c>
@@ -5669,7 +5691,7 @@
         <v>2.74</v>
       </c>
     </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A102" s="2">
         <v>45562</v>
       </c>
@@ -5683,7 +5705,7 @@
         <v>2.7970000000000002</v>
       </c>
     </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A103" s="2">
         <v>45569</v>
       </c>
@@ -5697,7 +5719,7 @@
         <v>2.7629999999999999</v>
       </c>
     </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A104" s="2">
         <v>45576</v>
       </c>
@@ -5711,7 +5733,7 @@
         <v>2.7530000000000001</v>
       </c>
     </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A105" s="2">
         <v>45583</v>
       </c>
@@ -5726,7 +5748,7 @@
       </c>
       <c r="E105" s="26"/>
     </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A106" s="2">
         <v>45590</v>
       </c>
@@ -5741,7 +5763,7 @@
       </c>
       <c r="E106" s="26"/>
     </row>
-    <row r="107" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A107" s="2">
         <v>45597</v>
       </c>
@@ -5756,7 +5778,7 @@
       </c>
       <c r="E107" s="26"/>
     </row>
-    <row r="108" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A108" s="2">
         <v>45604</v>
       </c>
@@ -5769,7 +5791,7 @@
       </c>
       <c r="E108" s="26"/>
     </row>
-    <row r="109" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A109" s="2">
         <v>45611</v>
       </c>
@@ -5782,7 +5804,7 @@
       </c>
       <c r="E109" s="26"/>
     </row>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A110" s="2">
         <v>45618</v>
       </c>
@@ -5795,7 +5817,7 @@
       </c>
       <c r="E110" s="26"/>
     </row>
-    <row r="111" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A111" s="2">
         <v>45625</v>
       </c>
@@ -5808,7 +5830,7 @@
       </c>
       <c r="E111" s="26"/>
     </row>
-    <row r="112" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A112" s="2">
         <v>45632</v>
       </c>
@@ -5823,7 +5845,7 @@
         <v>2.3769999999999998</v>
       </c>
     </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A113" s="2">
         <v>45639</v>
       </c>
@@ -5838,7 +5860,7 @@
         <v>2.2909999999999999</v>
       </c>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A114" s="2">
         <v>45646</v>
       </c>
@@ -5853,7 +5875,7 @@
         <v>2.1269999999999998</v>
       </c>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A115" s="2">
         <v>45653</v>
       </c>
@@ -5868,7 +5890,7 @@
         <v>2.0819999999999999</v>
       </c>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A116" s="2">
         <v>45660</v>
       </c>
@@ -5882,7 +5904,7 @@
         <v>2.2080000000000002</v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A117" s="2">
         <v>45667</v>
       </c>
@@ -5896,7 +5918,7 @@
         <v>2.738</v>
       </c>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A118" s="2">
         <v>45674</v>
       </c>
@@ -5910,7 +5932,7 @@
         <v>2.9994999999999998</v>
       </c>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A119" s="2">
         <v>45681</v>
       </c>
@@ -5924,7 +5946,7 @@
         <v>2.9994999999999998</v>
       </c>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A120" s="2">
         <v>45688</v>
       </c>
@@ -5938,7 +5960,7 @@
         <v>2.915</v>
       </c>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A121" s="2">
         <v>45695</v>
       </c>
@@ -5949,7 +5971,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A122" s="2">
         <v>45702</v>
       </c>
@@ -5960,7 +5982,7 @@
         <v>3.0150000000000001</v>
       </c>
     </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A123" s="2">
         <v>45709</v>
       </c>
@@ -5971,7 +5993,7 @@
         <v>2.9460000000000002</v>
       </c>
     </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A124" s="2">
         <v>45716</v>
       </c>
@@ -5985,7 +6007,7 @@
         <v>2.8490000000000002</v>
       </c>
     </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A125" s="2">
         <v>45723</v>
       </c>
@@ -5999,7 +6021,7 @@
         <v>2.5750000000000002</v>
       </c>
     </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A126" s="2">
         <v>45730</v>
       </c>
@@ -6013,7 +6035,7 @@
         <v>2.6579999999999999</v>
       </c>
     </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A127" s="2">
         <v>45737</v>
       </c>
@@ -6027,7 +6049,7 @@
         <v>2.641</v>
       </c>
     </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A128" s="2">
         <v>45744</v>
       </c>
@@ -6041,7 +6063,7 @@
         <v>2.629</v>
       </c>
     </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A129" s="2">
         <v>45751</v>
       </c>
@@ -6055,7 +6077,7 @@
         <v>2.4380000000000002</v>
       </c>
     </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A130" s="2">
         <v>45758</v>
       </c>
@@ -6069,7 +6091,7 @@
         <v>2.6179999999999999</v>
       </c>
     </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A131" s="2">
         <v>45765</v>
       </c>
@@ -6083,7 +6105,7 @@
         <v>2.605</v>
       </c>
     </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A132" s="2">
         <v>45772</v>
       </c>
@@ -6097,7 +6119,7 @@
         <v>2.7149999999999999</v>
       </c>
     </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A133" s="2">
         <v>45779</v>
       </c>
@@ -6111,7 +6133,7 @@
         <v>2.335</v>
       </c>
     </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A134" s="2">
         <v>45786</v>
       </c>
@@ -6122,7 +6144,7 @@
         <v>2.4249999999999998</v>
       </c>
     </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A135" s="2">
         <v>45793</v>
       </c>
@@ -6133,7 +6155,7 @@
         <v>2.3460000000000001</v>
       </c>
     </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A136" s="2">
         <v>45800</v>
       </c>
@@ -6144,7 +6166,7 @@
         <v>2.4289999999999998</v>
       </c>
     </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A137" s="2">
         <v>45807</v>
       </c>
@@ -6158,7 +6180,7 @@
         <v>2.5379999999999998</v>
       </c>
     </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A138" s="2">
         <v>45814</v>
       </c>
@@ -6172,7 +6194,7 @@
         <v>2.3980000000000001</v>
       </c>
     </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A139" s="2">
         <v>45821</v>
       </c>
@@ -6186,7 +6208,7 @@
         <v>2.504</v>
       </c>
     </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A140" s="2">
         <v>45828</v>
       </c>
@@ -6201,7 +6223,7 @@
         <v>2.0609999999999999</v>
       </c>
     </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A141" s="2">
         <v>45835</v>
       </c>
@@ -6216,7 +6238,7 @@
         <v>1.917</v>
       </c>
     </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A142" s="2">
         <v>45842</v>
       </c>
@@ -6230,7 +6252,7 @@
         <v>1.7809999999999999</v>
       </c>
     </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A143" s="2">
         <v>45849</v>
       </c>
@@ -6245,7 +6267,7 @@
       </c>
       <c r="E143" s="26"/>
     </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A144" s="2">
         <v>45856</v>
       </c>
@@ -6260,7 +6282,7 @@
       </c>
       <c r="E144" s="26"/>
     </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A145" s="2">
         <v>45863</v>
       </c>
@@ -6275,7 +6297,7 @@
       </c>
       <c r="E145" s="26"/>
     </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A146" s="2">
         <v>45870</v>
       </c>
@@ -6290,7 +6312,7 @@
       </c>
       <c r="E146" s="26"/>
     </row>
-    <row r="147" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A147" s="2">
         <v>45877</v>
       </c>
@@ -6303,7 +6325,7 @@
       </c>
       <c r="E147" s="26"/>
     </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A148" s="2">
         <v>45884</v>
       </c>
@@ -6316,7 +6338,7 @@
       </c>
       <c r="E148" s="26"/>
     </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A149" s="2">
         <v>45891</v>
       </c>
@@ -6329,7 +6351,7 @@
       </c>
       <c r="E149" s="26"/>
     </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A150" s="2">
         <v>45898</v>
       </c>
@@ -6344,7 +6366,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A151" s="2">
         <v>45905</v>
       </c>
@@ -6359,7 +6381,7 @@
         <v>2.2799999999999998</v>
       </c>
     </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A152" s="2">
         <v>45912</v>
       </c>
@@ -6374,7 +6396,7 @@
         <v>2.16</v>
       </c>
     </row>
-    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A153" s="2">
         <v>45919</v>
       </c>
@@ -6388,7 +6410,7 @@
         <v>2.1800000000000002</v>
       </c>
     </row>
-    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A154" s="2">
         <v>45926</v>
       </c>
@@ -6402,7 +6424,7 @@
         <v>2.46</v>
       </c>
     </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A155" s="2">
         <v>45933</v>
       </c>
@@ -6416,7 +6438,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A156" s="2">
         <v>45940</v>
       </c>
@@ -6430,7 +6452,7 @@
         <v>2.23</v>
       </c>
     </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A157" s="2">
         <v>45947</v>
       </c>
@@ -6444,7 +6466,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A158" s="2">
         <v>45954</v>
       </c>
@@ -6458,7 +6480,7 @@
         <v>2.2599999999999998</v>
       </c>
     </row>
-    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A159" s="2">
         <v>45961</v>
       </c>
@@ -6472,7 +6494,7 @@
         <v>2.2599999999999998</v>
       </c>
     </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A160" s="2">
         <v>45968</v>
       </c>
@@ -6486,7 +6508,7 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A161" s="2">
         <v>45975</v>
       </c>
@@ -6500,7 +6522,7 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A162" s="2">
         <v>45982</v>
       </c>
@@ -6514,7 +6536,7 @@
         <v>2.31</v>
       </c>
     </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A163" s="2">
         <v>45989</v>
       </c>
@@ -6531,7 +6553,7 @@
         <v>2.66</v>
       </c>
     </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A164" s="2">
         <v>45996</v>
       </c>
@@ -6545,7 +6567,7 @@
         <v>2.2200000000000002</v>
       </c>
     </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A165" s="2">
         <v>46003</v>
       </c>
@@ -6559,7 +6581,7 @@
         <v>2.2400000000000002</v>
       </c>
     </row>
-    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A166" s="2">
         <v>46010</v>
       </c>
@@ -6573,7 +6595,7 @@
         <v>2.11</v>
       </c>
     </row>
-    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A167" s="2">
         <v>46017</v>
       </c>
@@ -6587,7 +6609,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A168" s="2">
         <v>46024</v>
       </c>
@@ -6601,7 +6623,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A169" s="2">
         <v>46031</v>
       </c>
@@ -6615,7 +6637,7 @@
         <v>2.61</v>
       </c>
     </row>
-    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A170" s="2">
         <v>46038</v>
       </c>
@@ -6629,7 +6651,7 @@
         <v>2.75</v>
       </c>
     </row>
-    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A171" s="2">
         <v>46045</v>
       </c>
@@ -6643,7 +6665,7 @@
         <v>2.73</v>
       </c>
     </row>
-    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A172" s="2">
         <v>46052</v>
       </c>
@@ -6657,7 +6679,7 @@
         <v>2.73</v>
       </c>
     </row>
-    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A173" s="2">
         <v>46059</v>
       </c>
@@ -6671,7 +6693,7 @@
         <v>2.59</v>
       </c>
     </row>
-    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A174" s="2">
         <v>46066</v>
       </c>
@@ -6685,7 +6707,7 @@
         <v>2.63</v>
       </c>
     </row>
-    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A175" s="2">
         <v>46073</v>
       </c>
@@ -6699,7 +6721,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="176" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A176" s="2">
         <v>46080</v>
       </c>
@@ -6710,7 +6732,7 @@
         <v>2.38</v>
       </c>
     </row>
-    <row r="177" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A177" s="2">
         <v>46087</v>
       </c>
@@ -6721,7 +6743,7 @@
         <v>2.23</v>
       </c>
     </row>
-    <row r="178" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A178" s="2">
         <v>46094</v>
       </c>
@@ -6735,7 +6757,7 @@
         <v>2.68</v>
       </c>
     </row>
-    <row r="179" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A179" s="2">
         <v>46101</v>
       </c>
@@ -6749,7 +6771,7 @@
         <v>2.67</v>
       </c>
     </row>
-    <row r="180" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A180" s="2">
         <v>46108</v>
       </c>
@@ -6763,7 +6785,7 @@
         <v>2.68</v>
       </c>
     </row>
-    <row r="181" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A181" s="2">
         <v>46115</v>
       </c>
@@ -6777,7 +6799,7 @@
         <v>2.82</v>
       </c>
     </row>
-    <row r="182" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A182" s="2">
         <v>46122</v>
       </c>
@@ -6791,7 +6813,7 @@
         <v>2.6</v>
       </c>
     </row>
-    <row r="183" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A183" s="2">
         <v>46129</v>
       </c>
@@ -6805,7 +6827,7 @@
         <v>2.75</v>
       </c>
     </row>
-    <row r="184" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A184" s="2">
         <v>46136</v>
       </c>
@@ -6819,7 +6841,7 @@
         <v>2.81</v>
       </c>
     </row>
-    <row r="185" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A185" s="2">
         <v>46143</v>
       </c>
@@ -6833,7 +6855,7 @@
         <v>2.52</v>
       </c>
     </row>
-    <row r="186" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A186" s="2">
         <v>46150</v>
       </c>
@@ -6844,7 +6866,7 @@
         <v>2.59</v>
       </c>
     </row>
-    <row r="187" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A187" s="2">
         <v>46157</v>
       </c>
@@ -6855,7 +6877,7 @@
         <v>2.61</v>
       </c>
     </row>
-    <row r="188" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A188" s="2">
         <v>46164</v>
       </c>
@@ -6866,7 +6888,7 @@
         <v>2.61</v>
       </c>
     </row>
-    <row r="189" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A189" s="2">
         <v>46171</v>
       </c>
@@ -6880,7 +6902,7 @@
         <v>2.36</v>
       </c>
     </row>
-    <row r="190" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A190" s="2">
         <v>46178</v>
       </c>
@@ -6894,7 +6916,7 @@
         <v>2.4700000000000002</v>
       </c>
     </row>
-    <row r="191" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A191" s="2">
         <v>46185</v>
       </c>
@@ -6908,7 +6930,7 @@
         <v>2.46</v>
       </c>
     </row>
-    <row r="192" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A192" s="2">
         <v>46192</v>
       </c>
@@ -6922,7 +6944,7 @@
         <v>2.4500000000000002</v>
       </c>
     </row>
-    <row r="193" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A193" s="2">
         <v>46199</v>
       </c>
@@ -6936,7 +6958,7 @@
         <v>2.42</v>
       </c>
     </row>
-    <row r="194" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A194" s="2">
         <v>46206</v>
       </c>
@@ -6950,7 +6972,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="195" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A195" s="2">
         <v>46213</v>
       </c>
@@ -6964,7 +6986,7 @@
         <v>2.36</v>
       </c>
     </row>
-    <row r="196" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A196" s="2">
         <v>46220</v>
       </c>
@@ -6978,7 +7000,7 @@
         <v>2.6</v>
       </c>
     </row>
-    <row r="197" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A197" s="2">
         <v>46227</v>
       </c>
@@ -6992,7 +7014,7 @@
         <v>2.62</v>
       </c>
     </row>
-    <row r="198" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A198" s="2">
         <v>46234</v>
       </c>
@@ -7006,7 +7028,7 @@
         <v>2.52</v>
       </c>
     </row>
-    <row r="199" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A199" s="2">
         <v>46241</v>
       </c>
@@ -7017,7 +7039,7 @@
         <v>2.2400000000000002</v>
       </c>
     </row>
-    <row r="200" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A200" s="2">
         <v>46248</v>
       </c>
@@ -7028,7 +7050,7 @@
         <v>2.14</v>
       </c>
     </row>
-    <row r="201" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A201" s="2">
         <v>46255</v>
       </c>
@@ -7039,7 +7061,7 @@
         <v>2.27</v>
       </c>
     </row>
-    <row r="202" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A202" s="2">
         <v>46262</v>
       </c>
@@ -7050,7 +7072,7 @@
         <v>2.2200000000000002</v>
       </c>
     </row>
-    <row r="203" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A203" s="2">
         <v>46269</v>
       </c>
@@ -7064,7 +7086,7 @@
         <v>2.5099999999999998</v>
       </c>
     </row>
-    <row r="204" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A204" s="2">
         <v>46276</v>
       </c>
@@ -7078,7 +7100,7 @@
         <v>2.5099999999999998</v>
       </c>
     </row>
-    <row r="205" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A205" s="2">
         <v>46283</v>
       </c>
@@ -7090,6 +7112,34 @@
       </c>
       <c r="E205">
         <v>2.6</v>
+      </c>
+    </row>
+    <row r="206" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A206" s="2">
+        <v>46290</v>
+      </c>
+      <c r="B206" t="s">
+        <v>61</v>
+      </c>
+      <c r="D206">
+        <v>2.33</v>
+      </c>
+      <c r="E206">
+        <v>2.6</v>
+      </c>
+    </row>
+    <row r="207" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A207" s="2">
+        <v>46297</v>
+      </c>
+      <c r="B207" t="s">
+        <v>61</v>
+      </c>
+      <c r="D207">
+        <v>2.46</v>
+      </c>
+      <c r="E207">
+        <v>2.54</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data): daily ingest 2026-10-10
NORMAL/SLOWING · GDPNow 3.59 · NY 2.65
</commit_message>
<xml_diff>
--- a/data/cache/nyfed_nowcast_raw.xlsx
+++ b/data/cache/nyfed_nowcast_raw.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\SHARE\drf\TimeSeries\products\Nowcast\automated_nowcast\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{386C3A18-A0EE-49C5-9E14-E30951C56DC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70247AE9-CD4B-4378-91C4-F2EA8132CF27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="51840" windowHeight="21120" activeTab="2" xr2:uid="{ABCE1506-5AF9-4A77-93FF-F8162337FD42}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{ABCE1506-5AF9-4A77-93FF-F8162337FD42}"/>
   </bookViews>
   <sheets>
     <sheet name="New York Fed Nowcast" sheetId="3" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="62">
   <si>
     <t>Forecast Date</t>
   </si>
@@ -1841,7 +1841,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1670CA3-538E-42E7-9E1F-A6A72E94A86A}">
-  <dimension ref="A1:Q207"/>
+  <dimension ref="A1:Q208"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="27.1796875" customWidth="1"/>
@@ -4268,6 +4268,17 @@
       </c>
       <c r="Q207">
         <v>2.54</v>
+      </c>
+    </row>
+    <row r="208" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A208" s="2">
+        <v>46304</v>
+      </c>
+      <c r="P208">
+        <v>2.65</v>
+      </c>
+      <c r="Q208">
+        <v>2.83</v>
       </c>
     </row>
   </sheetData>
@@ -4291,7 +4302,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{596092BD-1EF6-4EC0-96F0-3BB4B0DA037F}">
-  <dimension ref="A1:I207"/>
+  <dimension ref="A1:I208"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="23.453125" customWidth="1"/>
@@ -7140,6 +7151,20 @@
       </c>
       <c r="E207">
         <v>2.54</v>
+      </c>
+    </row>
+    <row r="208" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A208" s="2">
+        <v>46304</v>
+      </c>
+      <c r="B208" t="s">
+        <v>61</v>
+      </c>
+      <c r="D208">
+        <v>2.65</v>
+      </c>
+      <c r="E208">
+        <v>2.83</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data): daily ingest 2026-10-17
NORMAL/SLOWING · GDPNow 3.64 · NY 2.67
</commit_message>
<xml_diff>
--- a/data/cache/nyfed_nowcast_raw.xlsx
+++ b/data/cache/nyfed_nowcast_raw.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\SHARE\drf\TimeSeries\products\Nowcast\automated_nowcast\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70247AE9-CD4B-4378-91C4-F2EA8132CF27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1E1B6F6-094A-48EB-A5DA-DC74401985E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{ABCE1506-5AF9-4A77-93FF-F8162337FD42}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="62">
   <si>
     <t>Forecast Date</t>
   </si>
@@ -1841,7 +1841,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1670CA3-538E-42E7-9E1F-A6A72E94A86A}">
-  <dimension ref="A1:Q208"/>
+  <dimension ref="A1:Q209"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="27.1796875" customWidth="1"/>
@@ -4279,6 +4279,17 @@
       </c>
       <c r="Q208">
         <v>2.83</v>
+      </c>
+    </row>
+    <row r="209" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A209" s="2">
+        <v>46311</v>
+      </c>
+      <c r="P209">
+        <v>2.67</v>
+      </c>
+      <c r="Q209">
+        <v>2.82</v>
       </c>
     </row>
   </sheetData>
@@ -4302,7 +4313,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{596092BD-1EF6-4EC0-96F0-3BB4B0DA037F}">
-  <dimension ref="A1:I208"/>
+  <dimension ref="A1:I209"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="23.453125" customWidth="1"/>
@@ -7165,6 +7176,20 @@
       </c>
       <c r="E208">
         <v>2.83</v>
+      </c>
+    </row>
+    <row r="209" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A209" s="2">
+        <v>46311</v>
+      </c>
+      <c r="B209" t="s">
+        <v>61</v>
+      </c>
+      <c r="D209">
+        <v>2.67</v>
+      </c>
+      <c r="E209">
+        <v>2.82</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data): daily ingest 2026-10-24
NORMAL/SLOWING · GDPNow 3.50 · NY 2.67
</commit_message>
<xml_diff>
--- a/data/cache/nyfed_nowcast_raw.xlsx
+++ b/data/cache/nyfed_nowcast_raw.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\SHARE\drf\TimeSeries\products\Nowcast\automated_nowcast\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1E1B6F6-094A-48EB-A5DA-DC74401985E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D76BF4ED-E00C-435A-A463-511C73781D0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{ABCE1506-5AF9-4A77-93FF-F8162337FD42}"/>
+    <workbookView xWindow="9400" yWindow="10690" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{ABCE1506-5AF9-4A77-93FF-F8162337FD42}"/>
   </bookViews>
   <sheets>
     <sheet name="New York Fed Nowcast" sheetId="3" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="62">
   <si>
     <t>Forecast Date</t>
   </si>
@@ -1604,15 +1604,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4E1EDB4-3E22-4B96-9108-06AEDE165285}">
   <dimension ref="B1:I42"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.81640625" style="5" customWidth="1"/>
-    <col min="2" max="2" width="129.453125" style="5" customWidth="1"/>
-    <col min="3" max="16384" width="9.1796875" style="5"/>
+    <col min="1" max="1" width="24.85546875" style="5" customWidth="1"/>
+    <col min="2" max="2" width="129.42578125" style="5" customWidth="1"/>
+    <col min="3" max="16384" width="9.140625" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="2" spans="2:9" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="2:9" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="33" t="s">
         <v>13</v>
       </c>
@@ -1624,7 +1624,7 @@
       <c r="H2" s="33"/>
       <c r="I2" s="33"/>
     </row>
-    <row r="3" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B3" s="33"/>
       <c r="C3" s="33"/>
       <c r="D3" s="33"/>
@@ -1634,67 +1634,67 @@
       <c r="H3" s="33"/>
       <c r="I3" s="33"/>
     </row>
-    <row r="4" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B4" s="4" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="2:9" ht="31" x14ac:dyDescent="0.7">
+    <row r="8" spans="2:9" ht="31.5" x14ac:dyDescent="0.5">
       <c r="B8" s="24" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="2:9" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="9" spans="2:9" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B9" s="25" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B10" s="6"/>
     </row>
-    <row r="11" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B11" s="20" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="12" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B12" s="7" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="13" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B13" s="9" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="14" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B14" s="9" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="15" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="17" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B17" s="22" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="18" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B18" s="23" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="19" spans="2:7" ht="10.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:7" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C19" s="16"/>
       <c r="D19" s="16"/>
       <c r="E19" s="16"/>
       <c r="F19" s="16"/>
       <c r="G19" s="16"/>
     </row>
-    <row r="20" spans="2:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:7" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="19" t="s">
         <v>27</v>
       </c>
@@ -1703,7 +1703,7 @@
       <c r="E20" s="8"/>
       <c r="F20" s="8"/>
     </row>
-    <row r="21" spans="2:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:7" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="10" t="s">
         <v>28</v>
       </c>
@@ -1712,14 +1712,14 @@
       <c r="E21" s="8"/>
       <c r="F21" s="8"/>
     </row>
-    <row r="22" spans="2:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:7" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="10"/>
       <c r="C22" s="8"/>
       <c r="D22" s="8"/>
       <c r="E22" s="8"/>
       <c r="F22" s="8"/>
     </row>
-    <row r="23" spans="2:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:7" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="19" t="s">
         <v>29</v>
       </c>
@@ -1728,7 +1728,7 @@
       <c r="E23" s="8"/>
       <c r="F23" s="8"/>
     </row>
-    <row r="24" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B24" s="10" t="s">
         <v>36</v>
       </c>
@@ -1737,55 +1737,55 @@
       <c r="E24" s="8"/>
       <c r="F24" s="8"/>
     </row>
-    <row r="25" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="10"/>
       <c r="C25" s="8"/>
       <c r="D25" s="8"/>
       <c r="E25" s="8"/>
       <c r="F25" s="8"/>
     </row>
-    <row r="26" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B26" s="19" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="27" spans="2:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:7" ht="30" x14ac:dyDescent="0.25">
       <c r="B27" s="21" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="28" spans="2:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:7" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28" s="21"/>
     </row>
-    <row r="29" spans="2:7" ht="19" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:7" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B29" s="11" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="30" spans="2:7" ht="19" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:7" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B30" s="13" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="31" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B31" s="18" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="32" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B32" s="18" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="33" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B33" s="17" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="34" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B34" s="13"/>
     </row>
-    <row r="35" spans="2:6" ht="13" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:6" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B35" s="14" t="s">
         <v>23</v>
       </c>
@@ -1794,7 +1794,7 @@
       <c r="E35" s="11"/>
       <c r="F35" s="11"/>
     </row>
-    <row r="36" spans="2:6" ht="16.399999999999999" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:6" ht="16.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B36" s="6" t="s">
         <v>24</v>
       </c>
@@ -1803,13 +1803,13 @@
       <c r="E36" s="12"/>
       <c r="F36" s="12"/>
     </row>
-    <row r="38" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C38" s="11"/>
       <c r="D38" s="11"/>
       <c r="E38" s="11"/>
       <c r="F38" s="11"/>
     </row>
-    <row r="42" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="42" spans="2:6" x14ac:dyDescent="0.25">
       <c r="C42" s="15"/>
       <c r="D42" s="15"/>
     </row>
@@ -1841,14 +1841,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1670CA3-538E-42E7-9E1F-A6A72E94A86A}">
-  <dimension ref="A1:Q209"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:Q210"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="27.1796875" customWidth="1"/>
+    <col min="1" max="1" width="27.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="2" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B2" s="29"/>
       <c r="C2" s="29"/>
       <c r="D2" s="29"/>
@@ -1857,7 +1857,7 @@
       <c r="G2" s="29"/>
       <c r="H2" s="29"/>
     </row>
-    <row r="3" spans="1:16" s="3" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:16" s="3" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B3" s="30" t="s">
         <v>25</v>
       </c>
@@ -1869,16 +1869,16 @@
       <c r="H3" s="31"/>
       <c r="I3" s="31"/>
     </row>
-    <row r="4" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C4" s="32" t="s">
         <v>14</v>
       </c>
       <c r="D4" s="32"/>
     </row>
-    <row r="5" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5"/>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>0</v>
       </c>
@@ -1928,7 +1928,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>44897</v>
       </c>
@@ -1936,7 +1936,7 @@
         <v>1.79</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>44904</v>
       </c>
@@ -1944,7 +1944,7 @@
         <v>1.76</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>44911</v>
       </c>
@@ -1952,7 +1952,7 @@
         <v>1.58</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>44918</v>
       </c>
@@ -1960,7 +1960,7 @@
         <v>1.33</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>44925</v>
       </c>
@@ -1968,7 +1968,7 @@
         <v>1.31</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>44932</v>
       </c>
@@ -1976,7 +1976,7 @@
         <v>1.57</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>44939</v>
       </c>
@@ -1984,7 +1984,7 @@
         <v>1.64</v>
       </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>44946</v>
       </c>
@@ -1992,7 +1992,7 @@
         <v>0.79</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>44953</v>
       </c>
@@ -2000,7 +2000,7 @@
         <v>1.2</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>44960</v>
       </c>
@@ -2008,7 +2008,7 @@
         <v>1.59</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
         <v>44967</v>
       </c>
@@ -2016,7 +2016,7 @@
         <v>1.48</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="2">
         <v>44974</v>
       </c>
@@ -2024,7 +2024,7 @@
         <v>1.1399999999999999</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="2">
         <v>44981</v>
       </c>
@@ -2035,7 +2035,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
         <v>44988</v>
       </c>
@@ -2046,7 +2046,7 @@
         <v>1.45</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="2">
         <v>44995</v>
       </c>
@@ -2057,7 +2057,7 @@
         <v>1.53</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="2">
         <v>45002</v>
       </c>
@@ -2068,7 +2068,7 @@
         <v>1.3</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="2">
         <v>45009</v>
       </c>
@@ -2079,7 +2079,7 @@
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="2">
         <v>45016</v>
       </c>
@@ -2090,7 +2090,7 @@
         <v>1.08</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="2">
         <v>45023</v>
       </c>
@@ -2101,7 +2101,7 @@
         <v>0.67</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="2">
         <v>45030</v>
       </c>
@@ -2112,7 +2112,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="2">
         <v>45037</v>
       </c>
@@ -2123,7 +2123,7 @@
         <v>1.1200000000000001</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="2">
         <v>45044</v>
       </c>
@@ -2134,7 +2134,7 @@
         <v>0.52</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="2">
         <v>45051</v>
       </c>
@@ -2142,7 +2142,7 @@
         <v>1.28</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="2">
         <v>45058</v>
       </c>
@@ -2150,7 +2150,7 @@
         <v>1.19</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="2">
         <v>45065</v>
       </c>
@@ -2158,7 +2158,7 @@
         <v>1.44</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="2">
         <v>45072</v>
       </c>
@@ -2169,7 +2169,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="2">
         <v>45079</v>
       </c>
@@ -2180,7 +2180,7 @@
         <v>1.96</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="2">
         <v>45086</v>
       </c>
@@ -2191,7 +2191,7 @@
         <v>1.9</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="2">
         <v>45093</v>
       </c>
@@ -2202,7 +2202,7 @@
         <v>1.81</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="2">
         <v>45100</v>
       </c>
@@ -2213,7 +2213,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="2">
         <v>45107</v>
       </c>
@@ -2224,7 +2224,7 @@
         <v>2.0699999999999998</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="2">
         <v>45114</v>
       </c>
@@ -2235,7 +2235,7 @@
         <v>1.53</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="2">
         <v>45121</v>
       </c>
@@ -2246,7 +2246,7 @@
         <v>1.51</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="2">
         <v>45128</v>
       </c>
@@ -2257,7 +2257,7 @@
         <v>1.25</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="2">
         <v>45135</v>
       </c>
@@ -2268,7 +2268,7 @@
         <v>1.93</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="2">
         <v>45142</v>
       </c>
@@ -2276,7 +2276,7 @@
         <v>1.81</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="2">
         <v>45149</v>
       </c>
@@ -2284,7 +2284,7 @@
         <v>1.7</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="2">
         <v>45156</v>
       </c>
@@ -2292,7 +2292,7 @@
         <v>2.34</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="2">
         <v>45163</v>
       </c>
@@ -2300,7 +2300,7 @@
         <v>2.12</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="2">
         <v>45170</v>
       </c>
@@ -2311,7 +2311,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="2">
         <v>45177</v>
       </c>
@@ -2322,7 +2322,7 @@
         <v>2.29</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="2">
         <v>45184</v>
       </c>
@@ -2333,7 +2333,7 @@
         <v>2.35</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" s="2">
         <v>45191</v>
       </c>
@@ -2344,7 +2344,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" s="2">
         <v>45198</v>
       </c>
@@ -2355,7 +2355,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" s="2">
         <v>45205</v>
       </c>
@@ -2366,7 +2366,7 @@
         <v>2.4039999999999999</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" s="2">
         <v>45212</v>
       </c>
@@ -2377,7 +2377,7 @@
         <v>2.34</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" s="2">
         <v>45219</v>
       </c>
@@ -2388,7 +2388,7 @@
         <v>2.27</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" s="2">
         <v>45226</v>
       </c>
@@ -2399,7 +2399,7 @@
         <v>2.79</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" s="2">
         <v>45233</v>
       </c>
@@ -2407,7 +2407,7 @@
         <v>2.41</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" s="2">
         <v>45240</v>
       </c>
@@ -2415,7 +2415,7 @@
         <v>2.5099999999999998</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" s="2">
         <v>45247</v>
       </c>
@@ -2423,7 +2423,7 @@
         <v>2.4500000000000002</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" s="2">
         <v>45254</v>
       </c>
@@ -2431,7 +2431,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" s="2">
         <v>45261</v>
       </c>
@@ -2442,7 +2442,7 @@
         <v>2.0499999999999998</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" s="2">
         <v>45268</v>
       </c>
@@ -2453,7 +2453,7 @@
         <v>2.13</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" s="2">
         <v>45275</v>
       </c>
@@ -2464,7 +2464,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" s="2">
         <v>45282</v>
       </c>
@@ -2475,7 +2475,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" s="2">
         <v>45289</v>
       </c>
@@ -2486,7 +2486,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" s="2">
         <v>45296</v>
       </c>
@@ -2497,7 +2497,7 @@
         <v>2.68</v>
       </c>
     </row>
-    <row r="65" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A65" s="2">
         <v>45303</v>
       </c>
@@ -2508,7 +2508,7 @@
         <v>2.4500000000000002</v>
       </c>
     </row>
-    <row r="66" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A66" s="2">
         <v>45310</v>
       </c>
@@ -2529,7 +2529,7 @@
       <c r="O66" s="26"/>
       <c r="P66" s="26"/>
     </row>
-    <row r="67" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A67" s="2">
         <v>45317</v>
       </c>
@@ -2550,7 +2550,7 @@
       <c r="O67" s="26"/>
       <c r="P67" s="26"/>
     </row>
-    <row r="68" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A68" s="2">
         <v>45324</v>
       </c>
@@ -2569,7 +2569,7 @@
       <c r="O68" s="26"/>
       <c r="P68" s="26"/>
     </row>
-    <row r="69" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A69" s="2">
         <v>45331</v>
       </c>
@@ -2588,7 +2588,7 @@
       <c r="O69" s="26"/>
       <c r="P69" s="26"/>
     </row>
-    <row r="70" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A70" s="2">
         <v>45338</v>
       </c>
@@ -2607,7 +2607,7 @@
       <c r="O70" s="26"/>
       <c r="P70" s="26"/>
     </row>
-    <row r="71" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A71" s="2">
         <v>45345</v>
       </c>
@@ -2626,7 +2626,7 @@
       <c r="O71" s="26"/>
       <c r="P71" s="26"/>
     </row>
-    <row r="72" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A72" s="2">
         <v>45352</v>
       </c>
@@ -2647,7 +2647,7 @@
       <c r="O72" s="26"/>
       <c r="P72" s="26"/>
     </row>
-    <row r="73" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A73" s="2">
         <v>45359</v>
       </c>
@@ -2668,7 +2668,7 @@
       <c r="O73" s="26"/>
       <c r="P73" s="26"/>
     </row>
-    <row r="74" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A74" s="2">
         <v>45366</v>
       </c>
@@ -2689,7 +2689,7 @@
       <c r="O74" s="26"/>
       <c r="P74" s="26"/>
     </row>
-    <row r="75" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A75" s="2">
         <v>45373</v>
       </c>
@@ -2710,7 +2710,7 @@
       <c r="O75" s="26"/>
       <c r="P75" s="26"/>
     </row>
-    <row r="76" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A76" s="2">
         <v>45380</v>
       </c>
@@ -2731,7 +2731,7 @@
       <c r="O76" s="26"/>
       <c r="P76" s="26"/>
     </row>
-    <row r="77" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A77" s="2">
         <v>45387</v>
       </c>
@@ -2752,7 +2752,7 @@
       <c r="O77" s="26"/>
       <c r="P77" s="26"/>
     </row>
-    <row r="78" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A78" s="2">
         <v>45394</v>
       </c>
@@ -2773,7 +2773,7 @@
       <c r="O78" s="26"/>
       <c r="P78" s="26"/>
     </row>
-    <row r="79" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A79" s="2">
         <v>45401</v>
       </c>
@@ -2794,7 +2794,7 @@
       <c r="O79" s="26"/>
       <c r="P79" s="26"/>
     </row>
-    <row r="80" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A80" s="2">
         <v>45408</v>
       </c>
@@ -2815,7 +2815,7 @@
       <c r="O80" s="26"/>
       <c r="P80" s="26"/>
     </row>
-    <row r="81" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A81" s="2">
         <v>45415</v>
       </c>
@@ -2834,7 +2834,7 @@
       <c r="O81" s="26"/>
       <c r="P81" s="26"/>
     </row>
-    <row r="82" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A82" s="2">
         <v>45422</v>
       </c>
@@ -2853,7 +2853,7 @@
       <c r="O82" s="26"/>
       <c r="P82" s="26"/>
     </row>
-    <row r="83" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A83" s="2">
         <v>45429</v>
       </c>
@@ -2872,7 +2872,7 @@
       <c r="O83" s="26"/>
       <c r="P83" s="26"/>
     </row>
-    <row r="84" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A84" s="2">
         <v>45436</v>
       </c>
@@ -2891,7 +2891,7 @@
       <c r="O84" s="26"/>
       <c r="P84" s="26"/>
     </row>
-    <row r="85" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A85" s="2">
         <v>45443</v>
       </c>
@@ -2912,7 +2912,7 @@
       <c r="O85" s="26"/>
       <c r="P85" s="26"/>
     </row>
-    <row r="86" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A86" s="2">
         <v>45450</v>
       </c>
@@ -2933,7 +2933,7 @@
       <c r="O86" s="26"/>
       <c r="P86" s="26"/>
     </row>
-    <row r="87" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A87" s="2">
         <v>45457</v>
       </c>
@@ -2954,7 +2954,7 @@
       <c r="O87" s="26"/>
       <c r="P87" s="26"/>
     </row>
-    <row r="88" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A88" s="2">
         <v>45464</v>
       </c>
@@ -2975,7 +2975,7 @@
       <c r="O88" s="26"/>
       <c r="P88" s="26"/>
     </row>
-    <row r="89" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A89" s="2">
         <v>45471</v>
       </c>
@@ -2996,7 +2996,7 @@
       <c r="O89" s="26"/>
       <c r="P89" s="26"/>
     </row>
-    <row r="90" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A90" s="2">
         <v>45478</v>
       </c>
@@ -3017,7 +3017,7 @@
       <c r="O90" s="26"/>
       <c r="P90" s="26"/>
     </row>
-    <row r="91" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A91" s="2">
         <v>45485</v>
       </c>
@@ -3038,7 +3038,7 @@
       <c r="O91" s="26"/>
       <c r="P91" s="26"/>
     </row>
-    <row r="92" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A92" s="2">
         <v>45492</v>
       </c>
@@ -3059,7 +3059,7 @@
       <c r="O92" s="26"/>
       <c r="P92" s="26"/>
     </row>
-    <row r="93" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A93" s="2">
         <v>45499</v>
       </c>
@@ -3080,7 +3080,7 @@
       <c r="O93" s="26"/>
       <c r="P93" s="26"/>
     </row>
-    <row r="94" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A94" s="2">
         <v>45506</v>
       </c>
@@ -3099,7 +3099,7 @@
       <c r="O94" s="26"/>
       <c r="P94" s="26"/>
     </row>
-    <row r="95" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A95" s="2">
         <v>45513</v>
       </c>
@@ -3107,7 +3107,7 @@
         <v>2.238</v>
       </c>
     </row>
-    <row r="96" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A96" s="2">
         <v>45520</v>
       </c>
@@ -3115,7 +3115,7 @@
         <v>1.84</v>
       </c>
     </row>
-    <row r="97" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A97" s="2">
         <v>45527</v>
       </c>
@@ -3123,7 +3123,7 @@
         <v>1.9410000000000001</v>
       </c>
     </row>
-    <row r="98" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A98" s="2">
         <v>45534</v>
       </c>
@@ -3134,7 +3134,7 @@
         <v>2.1160000000000001</v>
       </c>
     </row>
-    <row r="99" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A99" s="2">
         <v>45541</v>
       </c>
@@ -3145,7 +3145,7 @@
         <v>2.2130000000000001</v>
       </c>
     </row>
-    <row r="100" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A100" s="2">
         <v>45548</v>
       </c>
@@ -3156,7 +3156,7 @@
         <v>2.1749999999999998</v>
       </c>
     </row>
-    <row r="101" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A101" s="2">
         <v>45555</v>
       </c>
@@ -3167,7 +3167,7 @@
         <v>2.74</v>
       </c>
     </row>
-    <row r="102" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A102" s="2">
         <v>45562</v>
       </c>
@@ -3178,7 +3178,7 @@
         <v>2.7970000000000002</v>
       </c>
     </row>
-    <row r="103" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A103" s="2">
         <v>45569</v>
       </c>
@@ -3189,7 +3189,7 @@
         <v>2.7629999999999999</v>
       </c>
     </row>
-    <row r="104" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A104" s="2">
         <v>45576</v>
       </c>
@@ -3200,7 +3200,7 @@
         <v>2.7530000000000001</v>
       </c>
     </row>
-    <row r="105" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A105" s="2">
         <v>45583</v>
       </c>
@@ -3211,7 +3211,7 @@
         <v>2.6070000000000002</v>
       </c>
     </row>
-    <row r="106" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A106" s="2">
         <v>45590</v>
       </c>
@@ -3222,7 +3222,7 @@
         <v>2.4649999999999999</v>
       </c>
     </row>
-    <row r="107" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A107" s="2">
         <v>45597</v>
       </c>
@@ -3233,7 +3233,7 @@
         <v>2.0070000000000001</v>
       </c>
     </row>
-    <row r="108" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A108" s="2">
         <v>45604</v>
       </c>
@@ -3241,7 +3241,7 @@
         <v>2.0590000000000002</v>
       </c>
     </row>
-    <row r="109" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A109" s="2">
         <v>45611</v>
       </c>
@@ -3249,7 +3249,7 @@
         <v>2.0640000000000001</v>
       </c>
     </row>
-    <row r="110" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A110" s="2">
         <v>45618</v>
       </c>
@@ -3257,7 +3257,7 @@
         <v>1.909</v>
       </c>
     </row>
-    <row r="111" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A111" s="2">
         <v>45625</v>
       </c>
@@ -3265,7 +3265,7 @@
         <v>1.8049999999999999</v>
       </c>
     </row>
-    <row r="112" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A112" s="2">
         <v>45632</v>
       </c>
@@ -3276,7 +3276,7 @@
         <v>2.3769999999999998</v>
       </c>
     </row>
-    <row r="113" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A113" s="2">
         <v>45639</v>
       </c>
@@ -3287,7 +3287,7 @@
         <v>2.2909999999999999</v>
       </c>
     </row>
-    <row r="114" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A114" s="2">
         <v>45646</v>
       </c>
@@ -3298,7 +3298,7 @@
         <v>2.1269999999999998</v>
       </c>
     </row>
-    <row r="115" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A115" s="2">
         <v>45653</v>
       </c>
@@ -3309,7 +3309,7 @@
         <v>2.0819999999999999</v>
       </c>
     </row>
-    <row r="116" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A116" s="2">
         <v>45660</v>
       </c>
@@ -3320,7 +3320,7 @@
         <v>2.2080000000000002</v>
       </c>
     </row>
-    <row r="117" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A117" s="2">
         <v>45667</v>
       </c>
@@ -3331,7 +3331,7 @@
         <v>2.738</v>
       </c>
     </row>
-    <row r="118" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A118" s="2">
         <v>45674</v>
       </c>
@@ -3342,7 +3342,7 @@
         <v>2.9994999999999998</v>
       </c>
     </row>
-    <row r="119" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A119" s="2">
         <v>45681</v>
       </c>
@@ -3353,7 +3353,7 @@
         <v>2.9994999999999998</v>
       </c>
     </row>
-    <row r="120" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A120" s="2">
         <v>45688</v>
       </c>
@@ -3364,7 +3364,7 @@
         <v>2.915</v>
       </c>
     </row>
-    <row r="121" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A121" s="2">
         <v>45695</v>
       </c>
@@ -3372,7 +3372,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="122" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A122" s="2">
         <v>45702</v>
       </c>
@@ -3380,7 +3380,7 @@
         <v>3.0150000000000001</v>
       </c>
     </row>
-    <row r="123" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A123" s="2">
         <v>45709</v>
       </c>
@@ -3388,7 +3388,7 @@
         <v>2.9460000000000002</v>
       </c>
     </row>
-    <row r="124" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A124" s="2">
         <v>45716</v>
       </c>
@@ -3399,7 +3399,7 @@
         <v>2.8490000000000002</v>
       </c>
     </row>
-    <row r="125" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A125" s="2">
         <v>45723</v>
       </c>
@@ -3410,7 +3410,7 @@
         <v>2.5750000000000002</v>
       </c>
     </row>
-    <row r="126" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A126" s="2">
         <v>45730</v>
       </c>
@@ -3421,7 +3421,7 @@
         <v>2.6579999999999999</v>
       </c>
     </row>
-    <row r="127" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A127" s="2">
         <v>45737</v>
       </c>
@@ -3432,7 +3432,7 @@
         <v>2.641</v>
       </c>
     </row>
-    <row r="128" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A128" s="2">
         <v>45744</v>
       </c>
@@ -3443,7 +3443,7 @@
         <v>2.629</v>
       </c>
     </row>
-    <row r="129" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A129" s="2">
         <v>45751</v>
       </c>
@@ -3454,7 +3454,7 @@
         <v>2.4380000000000002</v>
       </c>
     </row>
-    <row r="130" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A130" s="2">
         <v>45758</v>
       </c>
@@ -3465,7 +3465,7 @@
         <v>2.6179999999999999</v>
       </c>
     </row>
-    <row r="131" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A131" s="2">
         <v>45765</v>
       </c>
@@ -3476,7 +3476,7 @@
         <v>2.605</v>
       </c>
     </row>
-    <row r="132" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A132" s="2">
         <v>45772</v>
       </c>
@@ -3487,7 +3487,7 @@
         <v>2.7149999999999999</v>
       </c>
     </row>
-    <row r="133" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A133" s="2">
         <v>45779</v>
       </c>
@@ -3498,7 +3498,7 @@
         <v>2.335</v>
       </c>
     </row>
-    <row r="134" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A134" s="2">
         <v>45786</v>
       </c>
@@ -3506,7 +3506,7 @@
         <v>2.4249999999999998</v>
       </c>
     </row>
-    <row r="135" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A135" s="2">
         <v>45793</v>
       </c>
@@ -3514,7 +3514,7 @@
         <v>2.3460000000000001</v>
       </c>
     </row>
-    <row r="136" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A136" s="2">
         <v>45800</v>
       </c>
@@ -3522,7 +3522,7 @@
         <v>2.4289999999999998</v>
       </c>
     </row>
-    <row r="137" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A137" s="2">
         <v>45807</v>
       </c>
@@ -3533,7 +3533,7 @@
         <v>2.5379999999999998</v>
       </c>
     </row>
-    <row r="138" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A138" s="2">
         <v>45814</v>
       </c>
@@ -3544,7 +3544,7 @@
         <v>2.3980000000000001</v>
       </c>
     </row>
-    <row r="139" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A139" s="2">
         <v>45821</v>
       </c>
@@ -3555,7 +3555,7 @@
         <v>2.504</v>
       </c>
     </row>
-    <row r="140" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A140" s="2">
         <v>45828</v>
       </c>
@@ -3566,7 +3566,7 @@
         <v>2.0609999999999999</v>
       </c>
     </row>
-    <row r="141" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A141" s="2">
         <v>45835</v>
       </c>
@@ -3577,7 +3577,7 @@
         <v>1.917</v>
       </c>
     </row>
-    <row r="142" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A142" s="2">
         <v>45842</v>
       </c>
@@ -3588,7 +3588,7 @@
         <v>1.7809999999999999</v>
       </c>
     </row>
-    <row r="143" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A143" s="2">
         <v>45849</v>
       </c>
@@ -3599,7 +3599,7 @@
         <v>1.78</v>
       </c>
     </row>
-    <row r="144" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A144" s="2">
         <v>45856</v>
       </c>
@@ -3610,7 +3610,7 @@
         <v>2.44</v>
       </c>
     </row>
-    <row r="145" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A145" s="2">
         <v>45863</v>
       </c>
@@ -3621,7 +3621,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="146" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A146" s="2">
         <v>45870</v>
       </c>
@@ -3632,7 +3632,7 @@
         <v>2.12</v>
       </c>
     </row>
-    <row r="147" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A147" s="2">
         <v>45877</v>
       </c>
@@ -3640,7 +3640,7 @@
         <v>2.02</v>
       </c>
     </row>
-    <row r="148" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A148" s="2">
         <v>45884</v>
       </c>
@@ -3648,7 +3648,7 @@
         <v>2.06</v>
       </c>
     </row>
-    <row r="149" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A149" s="2">
         <v>45891</v>
       </c>
@@ -3656,7 +3656,7 @@
         <v>2.0099999999999998</v>
       </c>
     </row>
-    <row r="150" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A150" s="2">
         <v>45898</v>
       </c>
@@ -3667,7 +3667,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="151" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A151" s="2">
         <v>45905</v>
       </c>
@@ -3678,7 +3678,7 @@
         <v>2.2799999999999998</v>
       </c>
     </row>
-    <row r="152" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A152" s="2">
         <v>45912</v>
       </c>
@@ -3689,7 +3689,7 @@
         <v>2.16</v>
       </c>
     </row>
-    <row r="153" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A153" s="2">
         <v>45919</v>
       </c>
@@ -3700,7 +3700,7 @@
         <v>2.1800000000000002</v>
       </c>
     </row>
-    <row r="154" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A154" s="2">
         <v>45926</v>
       </c>
@@ -3711,7 +3711,7 @@
         <v>2.46</v>
       </c>
     </row>
-    <row r="155" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A155" s="2">
         <v>45933</v>
       </c>
@@ -3722,7 +3722,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="156" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A156" s="2">
         <v>45940</v>
       </c>
@@ -3733,7 +3733,7 @@
         <v>2.23</v>
       </c>
     </row>
-    <row r="157" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A157" s="2">
         <v>45947</v>
       </c>
@@ -3744,7 +3744,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="158" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A158" s="2">
         <v>45954</v>
       </c>
@@ -3755,7 +3755,7 @@
         <v>2.2599999999999998</v>
       </c>
     </row>
-    <row r="159" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A159" s="2">
         <v>45961</v>
       </c>
@@ -3766,7 +3766,7 @@
         <v>2.2599999999999998</v>
       </c>
     </row>
-    <row r="160" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A160" s="2">
         <v>45968</v>
       </c>
@@ -3777,7 +3777,7 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="161" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A161" s="2">
         <v>45975</v>
       </c>
@@ -3788,7 +3788,7 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="162" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A162" s="2">
         <v>45982</v>
       </c>
@@ -3799,7 +3799,7 @@
         <v>2.31</v>
       </c>
     </row>
-    <row r="163" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A163" s="2">
         <v>45989</v>
       </c>
@@ -3813,7 +3813,7 @@
         <v>2.66</v>
       </c>
     </row>
-    <row r="164" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A164" s="2">
         <v>45996</v>
       </c>
@@ -3824,7 +3824,7 @@
         <v>2.2200000000000002</v>
       </c>
     </row>
-    <row r="165" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A165" s="2">
         <v>46003</v>
       </c>
@@ -3835,7 +3835,7 @@
         <v>2.2400000000000002</v>
       </c>
     </row>
-    <row r="166" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A166" s="2">
         <v>46010</v>
       </c>
@@ -3846,7 +3846,7 @@
         <v>2.11</v>
       </c>
     </row>
-    <row r="167" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A167" s="2">
         <v>46017</v>
       </c>
@@ -3857,7 +3857,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="168" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A168" s="2">
         <v>46024</v>
       </c>
@@ -3868,7 +3868,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="169" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A169" s="2">
         <v>46031</v>
       </c>
@@ -3879,7 +3879,7 @@
         <v>2.61</v>
       </c>
     </row>
-    <row r="170" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A170" s="2">
         <v>46038</v>
       </c>
@@ -3890,7 +3890,7 @@
         <v>2.75</v>
       </c>
     </row>
-    <row r="171" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A171" s="2">
         <v>46045</v>
       </c>
@@ -3901,7 +3901,7 @@
         <v>2.73</v>
       </c>
     </row>
-    <row r="172" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A172" s="2">
         <v>46052</v>
       </c>
@@ -3912,7 +3912,7 @@
         <v>2.73</v>
       </c>
     </row>
-    <row r="173" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A173" s="2">
         <v>46059</v>
       </c>
@@ -3923,7 +3923,7 @@
         <v>2.59</v>
       </c>
     </row>
-    <row r="174" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A174" s="2">
         <v>46066</v>
       </c>
@@ -3934,7 +3934,7 @@
         <v>2.63</v>
       </c>
     </row>
-    <row r="175" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A175" s="2">
         <v>46073</v>
       </c>
@@ -3945,7 +3945,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="176" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A176" s="2">
         <v>46080</v>
       </c>
@@ -3953,7 +3953,7 @@
         <v>2.38</v>
       </c>
     </row>
-    <row r="177" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A177" s="2">
         <v>46087</v>
       </c>
@@ -3961,7 +3961,7 @@
         <v>2.23</v>
       </c>
     </row>
-    <row r="178" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A178" s="2">
         <v>46094</v>
       </c>
@@ -3972,7 +3972,7 @@
         <v>2.68</v>
       </c>
     </row>
-    <row r="179" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A179" s="2">
         <v>46101</v>
       </c>
@@ -3983,7 +3983,7 @@
         <v>2.67</v>
       </c>
     </row>
-    <row r="180" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A180" s="2">
         <v>46108</v>
       </c>
@@ -3994,7 +3994,7 @@
         <v>2.68</v>
       </c>
     </row>
-    <row r="181" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A181" s="2">
         <v>46115</v>
       </c>
@@ -4005,7 +4005,7 @@
         <v>2.82</v>
       </c>
     </row>
-    <row r="182" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A182" s="2">
         <v>46122</v>
       </c>
@@ -4016,7 +4016,7 @@
         <v>2.6</v>
       </c>
     </row>
-    <row r="183" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A183" s="2">
         <v>46129</v>
       </c>
@@ -4027,7 +4027,7 @@
         <v>2.75</v>
       </c>
     </row>
-    <row r="184" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A184" s="2">
         <v>46136</v>
       </c>
@@ -4038,7 +4038,7 @@
         <v>2.81</v>
       </c>
     </row>
-    <row r="185" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A185" s="2">
         <v>46143</v>
       </c>
@@ -4049,7 +4049,7 @@
         <v>2.52</v>
       </c>
     </row>
-    <row r="186" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A186" s="2">
         <v>46150</v>
       </c>
@@ -4057,7 +4057,7 @@
         <v>2.59</v>
       </c>
     </row>
-    <row r="187" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A187" s="2">
         <v>46157</v>
       </c>
@@ -4065,7 +4065,7 @@
         <v>2.61</v>
       </c>
     </row>
-    <row r="188" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A188" s="2">
         <v>46164</v>
       </c>
@@ -4073,7 +4073,7 @@
         <v>2.61</v>
       </c>
     </row>
-    <row r="189" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A189" s="2">
         <v>46171</v>
       </c>
@@ -4084,7 +4084,7 @@
         <v>2.36</v>
       </c>
     </row>
-    <row r="190" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A190" s="2">
         <v>46178</v>
       </c>
@@ -4095,7 +4095,7 @@
         <v>2.4700000000000002</v>
       </c>
     </row>
-    <row r="191" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A191" s="2">
         <v>46185</v>
       </c>
@@ -4106,7 +4106,7 @@
         <v>2.46</v>
       </c>
     </row>
-    <row r="192" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A192" s="2">
         <v>46192</v>
       </c>
@@ -4117,7 +4117,7 @@
         <v>2.4500000000000002</v>
       </c>
     </row>
-    <row r="193" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A193" s="2">
         <v>46199</v>
       </c>
@@ -4128,7 +4128,7 @@
         <v>2.42</v>
       </c>
     </row>
-    <row r="194" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A194" s="2">
         <v>46206</v>
       </c>
@@ -4139,7 +4139,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="195" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A195" s="2">
         <v>46213</v>
       </c>
@@ -4150,7 +4150,7 @@
         <v>2.36</v>
       </c>
     </row>
-    <row r="196" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A196" s="2">
         <v>46220</v>
       </c>
@@ -4161,7 +4161,7 @@
         <v>2.6</v>
       </c>
     </row>
-    <row r="197" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A197" s="2">
         <v>46227</v>
       </c>
@@ -4172,7 +4172,7 @@
         <v>2.62</v>
       </c>
     </row>
-    <row r="198" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A198" s="2">
         <v>46234</v>
       </c>
@@ -4183,7 +4183,7 @@
         <v>2.52</v>
       </c>
     </row>
-    <row r="199" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A199" s="2">
         <v>46241</v>
       </c>
@@ -4191,7 +4191,7 @@
         <v>2.2400000000000002</v>
       </c>
     </row>
-    <row r="200" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A200" s="2">
         <v>46248</v>
       </c>
@@ -4199,7 +4199,7 @@
         <v>2.14</v>
       </c>
     </row>
-    <row r="201" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A201" s="2">
         <v>46255</v>
       </c>
@@ -4207,7 +4207,7 @@
         <v>2.27</v>
       </c>
     </row>
-    <row r="202" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A202" s="2">
         <v>46262</v>
       </c>
@@ -4215,7 +4215,7 @@
         <v>2.2200000000000002</v>
       </c>
     </row>
-    <row r="203" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A203" s="2">
         <v>46269</v>
       </c>
@@ -4226,7 +4226,7 @@
         <v>2.5099999999999998</v>
       </c>
     </row>
-    <row r="204" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A204" s="2">
         <v>46276</v>
       </c>
@@ -4237,7 +4237,7 @@
         <v>2.5099999999999998</v>
       </c>
     </row>
-    <row r="205" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A205" s="2">
         <v>46283</v>
       </c>
@@ -4248,7 +4248,7 @@
         <v>2.6</v>
       </c>
     </row>
-    <row r="206" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A206" s="2">
         <v>46290</v>
       </c>
@@ -4259,7 +4259,7 @@
         <v>2.6</v>
       </c>
     </row>
-    <row r="207" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A207" s="2">
         <v>46297</v>
       </c>
@@ -4270,7 +4270,7 @@
         <v>2.54</v>
       </c>
     </row>
-    <row r="208" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A208" s="2">
         <v>46304</v>
       </c>
@@ -4281,7 +4281,7 @@
         <v>2.83</v>
       </c>
     </row>
-    <row r="209" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A209" s="2">
         <v>46311</v>
       </c>
@@ -4290,6 +4290,17 @@
       </c>
       <c r="Q209">
         <v>2.82</v>
+      </c>
+    </row>
+    <row r="210" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A210" s="2">
+        <v>46318</v>
+      </c>
+      <c r="P210">
+        <v>2.67</v>
+      </c>
+      <c r="Q210">
+        <v>2.81</v>
       </c>
     </row>
   </sheetData>
@@ -4313,18 +4324,18 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{596092BD-1EF6-4EC0-96F0-3BB4B0DA037F}">
-  <dimension ref="A1:I209"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:I210"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.453125" customWidth="1"/>
-    <col min="2" max="2" width="18.81640625" customWidth="1"/>
-    <col min="3" max="3" width="24.81640625" customWidth="1"/>
-    <col min="4" max="4" width="25.1796875" customWidth="1"/>
-    <col min="5" max="5" width="23.453125" customWidth="1"/>
+    <col min="1" max="1" width="23.42578125" customWidth="1"/>
+    <col min="2" max="2" width="18.85546875" customWidth="1"/>
+    <col min="3" max="3" width="24.85546875" customWidth="1"/>
+    <col min="4" max="4" width="25.140625" customWidth="1"/>
+    <col min="5" max="5" width="23.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="2" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B2" s="29"/>
       <c r="C2" s="29"/>
       <c r="D2" s="29"/>
@@ -4333,7 +4344,7 @@
       <c r="G2" s="29"/>
       <c r="H2" s="29"/>
     </row>
-    <row r="3" spans="1:9" s="3" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" s="3" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B3" s="30" t="s">
         <v>25</v>
       </c>
@@ -4345,16 +4356,16 @@
       <c r="H3" s="31"/>
       <c r="I3" s="31"/>
     </row>
-    <row r="4" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C4" s="32" t="s">
         <v>14</v>
       </c>
       <c r="D4" s="32"/>
     </row>
-    <row r="5" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5"/>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -4371,7 +4382,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>44897</v>
       </c>
@@ -4382,7 +4393,7 @@
         <v>1.79</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>44904</v>
       </c>
@@ -4393,7 +4404,7 @@
         <v>1.76</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>44911</v>
       </c>
@@ -4404,7 +4415,7 @@
         <v>1.58</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>44918</v>
       </c>
@@ -4415,7 +4426,7 @@
         <v>1.33</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>44925</v>
       </c>
@@ -4426,7 +4437,7 @@
         <v>1.31</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>44932</v>
       </c>
@@ -4437,7 +4448,7 @@
         <v>1.57</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>44939</v>
       </c>
@@ -4448,7 +4459,7 @@
         <v>1.64</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>44946</v>
       </c>
@@ -4459,7 +4470,7 @@
         <v>0.79</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>44953</v>
       </c>
@@ -4470,7 +4481,7 @@
         <v>1.2</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>44960</v>
       </c>
@@ -4481,7 +4492,7 @@
         <v>1.59</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
         <v>44967</v>
       </c>
@@ -4492,7 +4503,7 @@
         <v>1.48</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="2">
         <v>44974</v>
       </c>
@@ -4503,7 +4514,7 @@
         <v>1.1399999999999999</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="2">
         <v>44981</v>
       </c>
@@ -4517,7 +4528,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
         <v>44988</v>
       </c>
@@ -4531,7 +4542,7 @@
         <v>1.45</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="2">
         <v>44995</v>
       </c>
@@ -4545,7 +4556,7 @@
         <v>1.53</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="2">
         <v>45002</v>
       </c>
@@ -4559,7 +4570,7 @@
         <v>1.3</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="2">
         <v>45009</v>
       </c>
@@ -4573,7 +4584,7 @@
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="2">
         <v>45016</v>
       </c>
@@ -4587,7 +4598,7 @@
         <v>1.08</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="2">
         <v>45023</v>
       </c>
@@ -4601,7 +4612,7 @@
         <v>0.67</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="2">
         <v>45030</v>
       </c>
@@ -4615,7 +4626,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="2">
         <v>45037</v>
       </c>
@@ -4629,7 +4640,7 @@
         <v>1.1200000000000001</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="2">
         <v>45044</v>
       </c>
@@ -4643,7 +4654,7 @@
         <v>0.52</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="2">
         <v>45051</v>
       </c>
@@ -4654,7 +4665,7 @@
         <v>1.28</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="2">
         <v>45058</v>
       </c>
@@ -4665,7 +4676,7 @@
         <v>1.19</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="2">
         <v>45065</v>
       </c>
@@ -4676,7 +4687,7 @@
         <v>1.44</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="2">
         <v>45072</v>
       </c>
@@ -4690,7 +4701,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="2">
         <v>45079</v>
       </c>
@@ -4704,7 +4715,7 @@
         <v>1.96</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="2">
         <v>45086</v>
       </c>
@@ -4718,7 +4729,7 @@
         <v>1.9</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="2">
         <v>45093</v>
       </c>
@@ -4732,7 +4743,7 @@
         <v>1.81</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="2">
         <v>45100</v>
       </c>
@@ -4746,7 +4757,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="2">
         <v>45107</v>
       </c>
@@ -4760,7 +4771,7 @@
         <v>2.0699999999999998</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="2">
         <v>45114</v>
       </c>
@@ -4774,7 +4785,7 @@
         <v>1.53</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="2">
         <v>45121</v>
       </c>
@@ -4788,7 +4799,7 @@
         <v>1.51</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="2">
         <v>45128</v>
       </c>
@@ -4802,7 +4813,7 @@
         <v>1.25</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="2">
         <v>45135</v>
       </c>
@@ -4816,7 +4827,7 @@
         <v>1.93</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="2">
         <v>45142</v>
       </c>
@@ -4827,7 +4838,7 @@
         <v>1.81</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="2">
         <v>45149</v>
       </c>
@@ -4838,7 +4849,7 @@
         <v>1.7</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="2">
         <v>45156</v>
       </c>
@@ -4849,7 +4860,7 @@
         <v>2.34</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="2">
         <v>45163</v>
       </c>
@@ -4860,7 +4871,7 @@
         <v>2.12</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="2">
         <v>45170</v>
       </c>
@@ -4874,7 +4885,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="2">
         <v>45177</v>
       </c>
@@ -4888,7 +4899,7 @@
         <v>2.29</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="2">
         <v>45184</v>
       </c>
@@ -4902,7 +4913,7 @@
         <v>2.35</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="2">
         <v>45191</v>
       </c>
@@ -4916,7 +4927,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="2">
         <v>45198</v>
       </c>
@@ -4930,7 +4941,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="2">
         <v>45205</v>
       </c>
@@ -4944,7 +4955,7 @@
         <v>2.4039999999999999</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="2">
         <v>45212</v>
       </c>
@@ -4958,7 +4969,7 @@
         <v>2.34</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" s="2">
         <v>45219</v>
       </c>
@@ -4972,7 +4983,7 @@
         <v>2.27</v>
       </c>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" s="2">
         <v>45226</v>
       </c>
@@ -4986,7 +4997,7 @@
         <v>2.79</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="2">
         <v>45233</v>
       </c>
@@ -4997,7 +5008,7 @@
         <v>2.41</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="2">
         <v>45240</v>
       </c>
@@ -5008,7 +5019,7 @@
         <v>2.5099999999999998</v>
       </c>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="2">
         <v>45247</v>
       </c>
@@ -5019,7 +5030,7 @@
         <v>2.4500000000000002</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="2">
         <v>45254</v>
       </c>
@@ -5030,7 +5041,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="2">
         <v>45261</v>
       </c>
@@ -5044,7 +5055,7 @@
         <v>2.0499999999999998</v>
       </c>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="2">
         <v>45268</v>
       </c>
@@ -5058,7 +5069,7 @@
         <v>2.13</v>
       </c>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="2">
         <v>45275</v>
       </c>
@@ -5072,7 +5083,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="2">
         <v>45282</v>
       </c>
@@ -5086,7 +5097,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="2">
         <v>45289</v>
       </c>
@@ -5100,7 +5111,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="2">
         <v>45296</v>
       </c>
@@ -5117,7 +5128,7 @@
       <c r="F64" s="26"/>
       <c r="G64" s="26"/>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A65" s="2">
         <v>45303</v>
       </c>
@@ -5134,7 +5145,7 @@
       <c r="F65" s="26"/>
       <c r="G65" s="26"/>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A66" s="2">
         <v>45310</v>
       </c>
@@ -5151,7 +5162,7 @@
       <c r="F66" s="26"/>
       <c r="G66" s="26"/>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A67" s="2">
         <v>45317</v>
       </c>
@@ -5168,7 +5179,7 @@
       <c r="F67" s="26"/>
       <c r="G67" s="26"/>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A68" s="2">
         <v>45324</v>
       </c>
@@ -5183,7 +5194,7 @@
       <c r="F68" s="26"/>
       <c r="G68" s="26"/>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A69" s="2">
         <v>45331</v>
       </c>
@@ -5198,7 +5209,7 @@
       <c r="F69" s="26"/>
       <c r="G69" s="26"/>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A70" s="2">
         <v>45338</v>
       </c>
@@ -5213,7 +5224,7 @@
       <c r="F70" s="26"/>
       <c r="G70" s="26"/>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A71" s="2">
         <v>45345</v>
       </c>
@@ -5228,7 +5239,7 @@
       <c r="F71" s="26"/>
       <c r="G71" s="26"/>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A72" s="2">
         <v>45352</v>
       </c>
@@ -5245,7 +5256,7 @@
       <c r="F72" s="26"/>
       <c r="G72" s="26"/>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A73" s="2">
         <v>45359</v>
       </c>
@@ -5262,7 +5273,7 @@
       <c r="F73" s="26"/>
       <c r="G73" s="26"/>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A74" s="2">
         <v>45366</v>
       </c>
@@ -5276,7 +5287,7 @@
         <v>2.09</v>
       </c>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A75" s="2">
         <v>45373</v>
       </c>
@@ -5290,7 +5301,7 @@
         <v>2.19</v>
       </c>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A76" s="2">
         <v>45380</v>
       </c>
@@ -5307,7 +5318,7 @@
       <c r="F76" s="26"/>
       <c r="G76" s="26"/>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A77" s="2">
         <v>45387</v>
       </c>
@@ -5324,7 +5335,7 @@
       <c r="F77" s="26"/>
       <c r="G77" s="26"/>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A78" s="2">
         <v>45394</v>
       </c>
@@ -5341,7 +5352,7 @@
       <c r="F78" s="26"/>
       <c r="G78" s="26"/>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A79" s="2">
         <v>45401</v>
       </c>
@@ -5358,7 +5369,7 @@
       <c r="F79" s="26"/>
       <c r="G79" s="26"/>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A80" s="2">
         <v>45408</v>
       </c>
@@ -5375,7 +5386,7 @@
       <c r="F80" s="26"/>
       <c r="G80" s="26"/>
     </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A81" s="2">
         <v>45415</v>
       </c>
@@ -5390,7 +5401,7 @@
       <c r="F81" s="26"/>
       <c r="G81" s="26"/>
     </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A82" s="2">
         <v>45422</v>
       </c>
@@ -5405,7 +5416,7 @@
       <c r="F82" s="26"/>
       <c r="G82" s="26"/>
     </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A83" s="2">
         <v>45429</v>
       </c>
@@ -5420,7 +5431,7 @@
       <c r="F83" s="26"/>
       <c r="G83" s="26"/>
     </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A84" s="2">
         <v>45436</v>
       </c>
@@ -5435,7 +5446,7 @@
       <c r="F84" s="26"/>
       <c r="G84" s="26"/>
     </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A85" s="2">
         <v>45443</v>
       </c>
@@ -5452,7 +5463,7 @@
       <c r="F85" s="26"/>
       <c r="G85" s="26"/>
     </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A86" s="2">
         <v>45450</v>
       </c>
@@ -5469,7 +5480,7 @@
       <c r="F86" s="26"/>
       <c r="G86" s="26"/>
     </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A87" s="2">
         <v>45457</v>
       </c>
@@ -5486,7 +5497,7 @@
       <c r="F87" s="26"/>
       <c r="G87" s="26"/>
     </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A88" s="2">
         <v>45464</v>
       </c>
@@ -5503,7 +5514,7 @@
       <c r="F88" s="26"/>
       <c r="G88" s="26"/>
     </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A89" s="2">
         <v>45471</v>
       </c>
@@ -5520,7 +5531,7 @@
       <c r="F89" s="26"/>
       <c r="G89" s="26"/>
     </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A90" s="2">
         <v>45478</v>
       </c>
@@ -5537,7 +5548,7 @@
       <c r="F90" s="26"/>
       <c r="G90" s="26"/>
     </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A91" s="2">
         <v>45485</v>
       </c>
@@ -5554,7 +5565,7 @@
       <c r="F91" s="26"/>
       <c r="G91" s="26"/>
     </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A92" s="2">
         <v>45492</v>
       </c>
@@ -5571,7 +5582,7 @@
       <c r="F92" s="26"/>
       <c r="G92" s="26"/>
     </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A93" s="2">
         <v>45499</v>
       </c>
@@ -5588,7 +5599,7 @@
       <c r="F93" s="26"/>
       <c r="G93" s="26"/>
     </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A94" s="2">
         <v>45506</v>
       </c>
@@ -5603,7 +5614,7 @@
       <c r="F94" s="26"/>
       <c r="G94" s="26"/>
     </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A95" s="2">
         <v>45513</v>
       </c>
@@ -5618,7 +5629,7 @@
       <c r="F95" s="26"/>
       <c r="G95" s="26"/>
     </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A96" s="2">
         <v>45520</v>
       </c>
@@ -5633,7 +5644,7 @@
       <c r="F96" s="26"/>
       <c r="G96" s="26"/>
     </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A97" s="2">
         <v>45527</v>
       </c>
@@ -5648,7 +5659,7 @@
       <c r="F97" s="26"/>
       <c r="G97" s="26"/>
     </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A98" s="2">
         <v>45534</v>
       </c>
@@ -5665,7 +5676,7 @@
       <c r="F98" s="26"/>
       <c r="G98" s="26"/>
     </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A99" s="2">
         <v>45541</v>
       </c>
@@ -5682,7 +5693,7 @@
       <c r="F99" s="26"/>
       <c r="G99" s="26"/>
     </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A100" s="2">
         <v>45548</v>
       </c>
@@ -5699,7 +5710,7 @@
       <c r="F100" s="26"/>
       <c r="G100" s="26"/>
     </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A101" s="2">
         <v>45555</v>
       </c>
@@ -5713,7 +5724,7 @@
         <v>2.74</v>
       </c>
     </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A102" s="2">
         <v>45562</v>
       </c>
@@ -5727,7 +5738,7 @@
         <v>2.7970000000000002</v>
       </c>
     </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A103" s="2">
         <v>45569</v>
       </c>
@@ -5741,7 +5752,7 @@
         <v>2.7629999999999999</v>
       </c>
     </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A104" s="2">
         <v>45576</v>
       </c>
@@ -5755,7 +5766,7 @@
         <v>2.7530000000000001</v>
       </c>
     </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A105" s="2">
         <v>45583</v>
       </c>
@@ -5770,7 +5781,7 @@
       </c>
       <c r="E105" s="26"/>
     </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A106" s="2">
         <v>45590</v>
       </c>
@@ -5785,7 +5796,7 @@
       </c>
       <c r="E106" s="26"/>
     </row>
-    <row r="107" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A107" s="2">
         <v>45597</v>
       </c>
@@ -5800,7 +5811,7 @@
       </c>
       <c r="E107" s="26"/>
     </row>
-    <row r="108" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A108" s="2">
         <v>45604</v>
       </c>
@@ -5813,7 +5824,7 @@
       </c>
       <c r="E108" s="26"/>
     </row>
-    <row r="109" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A109" s="2">
         <v>45611</v>
       </c>
@@ -5826,7 +5837,7 @@
       </c>
       <c r="E109" s="26"/>
     </row>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A110" s="2">
         <v>45618</v>
       </c>
@@ -5839,7 +5850,7 @@
       </c>
       <c r="E110" s="26"/>
     </row>
-    <row r="111" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A111" s="2">
         <v>45625</v>
       </c>
@@ -5852,7 +5863,7 @@
       </c>
       <c r="E111" s="26"/>
     </row>
-    <row r="112" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A112" s="2">
         <v>45632</v>
       </c>
@@ -5867,7 +5878,7 @@
         <v>2.3769999999999998</v>
       </c>
     </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A113" s="2">
         <v>45639</v>
       </c>
@@ -5882,7 +5893,7 @@
         <v>2.2909999999999999</v>
       </c>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A114" s="2">
         <v>45646</v>
       </c>
@@ -5897,7 +5908,7 @@
         <v>2.1269999999999998</v>
       </c>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A115" s="2">
         <v>45653</v>
       </c>
@@ -5912,7 +5923,7 @@
         <v>2.0819999999999999</v>
       </c>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A116" s="2">
         <v>45660</v>
       </c>
@@ -5926,7 +5937,7 @@
         <v>2.2080000000000002</v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A117" s="2">
         <v>45667</v>
       </c>
@@ -5940,7 +5951,7 @@
         <v>2.738</v>
       </c>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A118" s="2">
         <v>45674</v>
       </c>
@@ -5954,7 +5965,7 @@
         <v>2.9994999999999998</v>
       </c>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A119" s="2">
         <v>45681</v>
       </c>
@@ -5968,7 +5979,7 @@
         <v>2.9994999999999998</v>
       </c>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A120" s="2">
         <v>45688</v>
       </c>
@@ -5982,7 +5993,7 @@
         <v>2.915</v>
       </c>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A121" s="2">
         <v>45695</v>
       </c>
@@ -5993,7 +6004,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A122" s="2">
         <v>45702</v>
       </c>
@@ -6004,7 +6015,7 @@
         <v>3.0150000000000001</v>
       </c>
     </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A123" s="2">
         <v>45709</v>
       </c>
@@ -6015,7 +6026,7 @@
         <v>2.9460000000000002</v>
       </c>
     </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A124" s="2">
         <v>45716</v>
       </c>
@@ -6029,7 +6040,7 @@
         <v>2.8490000000000002</v>
       </c>
     </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A125" s="2">
         <v>45723</v>
       </c>
@@ -6043,7 +6054,7 @@
         <v>2.5750000000000002</v>
       </c>
     </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A126" s="2">
         <v>45730</v>
       </c>
@@ -6057,7 +6068,7 @@
         <v>2.6579999999999999</v>
       </c>
     </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A127" s="2">
         <v>45737</v>
       </c>
@@ -6071,7 +6082,7 @@
         <v>2.641</v>
       </c>
     </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A128" s="2">
         <v>45744</v>
       </c>
@@ -6085,7 +6096,7 @@
         <v>2.629</v>
       </c>
     </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A129" s="2">
         <v>45751</v>
       </c>
@@ -6099,7 +6110,7 @@
         <v>2.4380000000000002</v>
       </c>
     </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A130" s="2">
         <v>45758</v>
       </c>
@@ -6113,7 +6124,7 @@
         <v>2.6179999999999999</v>
       </c>
     </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A131" s="2">
         <v>45765</v>
       </c>
@@ -6127,7 +6138,7 @@
         <v>2.605</v>
       </c>
     </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A132" s="2">
         <v>45772</v>
       </c>
@@ -6141,7 +6152,7 @@
         <v>2.7149999999999999</v>
       </c>
     </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A133" s="2">
         <v>45779</v>
       </c>
@@ -6155,7 +6166,7 @@
         <v>2.335</v>
       </c>
     </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A134" s="2">
         <v>45786</v>
       </c>
@@ -6166,7 +6177,7 @@
         <v>2.4249999999999998</v>
       </c>
     </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A135" s="2">
         <v>45793</v>
       </c>
@@ -6177,7 +6188,7 @@
         <v>2.3460000000000001</v>
       </c>
     </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A136" s="2">
         <v>45800</v>
       </c>
@@ -6188,7 +6199,7 @@
         <v>2.4289999999999998</v>
       </c>
     </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A137" s="2">
         <v>45807</v>
       </c>
@@ -6202,7 +6213,7 @@
         <v>2.5379999999999998</v>
       </c>
     </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A138" s="2">
         <v>45814</v>
       </c>
@@ -6216,7 +6227,7 @@
         <v>2.3980000000000001</v>
       </c>
     </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A139" s="2">
         <v>45821</v>
       </c>
@@ -6230,7 +6241,7 @@
         <v>2.504</v>
       </c>
     </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A140" s="2">
         <v>45828</v>
       </c>
@@ -6245,7 +6256,7 @@
         <v>2.0609999999999999</v>
       </c>
     </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A141" s="2">
         <v>45835</v>
       </c>
@@ -6260,7 +6271,7 @@
         <v>1.917</v>
       </c>
     </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A142" s="2">
         <v>45842</v>
       </c>
@@ -6274,7 +6285,7 @@
         <v>1.7809999999999999</v>
       </c>
     </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A143" s="2">
         <v>45849</v>
       </c>
@@ -6289,7 +6300,7 @@
       </c>
       <c r="E143" s="26"/>
     </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A144" s="2">
         <v>45856</v>
       </c>
@@ -6304,7 +6315,7 @@
       </c>
       <c r="E144" s="26"/>
     </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A145" s="2">
         <v>45863</v>
       </c>
@@ -6319,7 +6330,7 @@
       </c>
       <c r="E145" s="26"/>
     </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A146" s="2">
         <v>45870</v>
       </c>
@@ -6334,7 +6345,7 @@
       </c>
       <c r="E146" s="26"/>
     </row>
-    <row r="147" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A147" s="2">
         <v>45877</v>
       </c>
@@ -6347,7 +6358,7 @@
       </c>
       <c r="E147" s="26"/>
     </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A148" s="2">
         <v>45884</v>
       </c>
@@ -6360,7 +6371,7 @@
       </c>
       <c r="E148" s="26"/>
     </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A149" s="2">
         <v>45891</v>
       </c>
@@ -6373,7 +6384,7 @@
       </c>
       <c r="E149" s="26"/>
     </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A150" s="2">
         <v>45898</v>
       </c>
@@ -6388,7 +6399,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A151" s="2">
         <v>45905</v>
       </c>
@@ -6403,7 +6414,7 @@
         <v>2.2799999999999998</v>
       </c>
     </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A152" s="2">
         <v>45912</v>
       </c>
@@ -6418,7 +6429,7 @@
         <v>2.16</v>
       </c>
     </row>
-    <row r="153" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A153" s="2">
         <v>45919</v>
       </c>
@@ -6432,7 +6443,7 @@
         <v>2.1800000000000002</v>
       </c>
     </row>
-    <row r="154" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A154" s="2">
         <v>45926</v>
       </c>
@@ -6446,7 +6457,7 @@
         <v>2.46</v>
       </c>
     </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A155" s="2">
         <v>45933</v>
       </c>
@@ -6460,7 +6471,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A156" s="2">
         <v>45940</v>
       </c>
@@ -6474,7 +6485,7 @@
         <v>2.23</v>
       </c>
     </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A157" s="2">
         <v>45947</v>
       </c>
@@ -6488,7 +6499,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A158" s="2">
         <v>45954</v>
       </c>
@@ -6502,7 +6513,7 @@
         <v>2.2599999999999998</v>
       </c>
     </row>
-    <row r="159" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A159" s="2">
         <v>45961</v>
       </c>
@@ -6516,7 +6527,7 @@
         <v>2.2599999999999998</v>
       </c>
     </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A160" s="2">
         <v>45968</v>
       </c>
@@ -6530,7 +6541,7 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="161" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A161" s="2">
         <v>45975</v>
       </c>
@@ -6544,7 +6555,7 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A162" s="2">
         <v>45982</v>
       </c>
@@ -6558,7 +6569,7 @@
         <v>2.31</v>
       </c>
     </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A163" s="2">
         <v>45989</v>
       </c>
@@ -6575,7 +6586,7 @@
         <v>2.66</v>
       </c>
     </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A164" s="2">
         <v>45996</v>
       </c>
@@ -6589,7 +6600,7 @@
         <v>2.2200000000000002</v>
       </c>
     </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A165" s="2">
         <v>46003</v>
       </c>
@@ -6603,7 +6614,7 @@
         <v>2.2400000000000002</v>
       </c>
     </row>
-    <row r="166" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A166" s="2">
         <v>46010</v>
       </c>
@@ -6617,7 +6628,7 @@
         <v>2.11</v>
       </c>
     </row>
-    <row r="167" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A167" s="2">
         <v>46017</v>
       </c>
@@ -6631,7 +6642,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="168" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A168" s="2">
         <v>46024</v>
       </c>
@@ -6645,7 +6656,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="169" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A169" s="2">
         <v>46031</v>
       </c>
@@ -6659,7 +6670,7 @@
         <v>2.61</v>
       </c>
     </row>
-    <row r="170" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A170" s="2">
         <v>46038</v>
       </c>
@@ -6673,7 +6684,7 @@
         <v>2.75</v>
       </c>
     </row>
-    <row r="171" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A171" s="2">
         <v>46045</v>
       </c>
@@ -6687,7 +6698,7 @@
         <v>2.73</v>
       </c>
     </row>
-    <row r="172" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A172" s="2">
         <v>46052</v>
       </c>
@@ -6701,7 +6712,7 @@
         <v>2.73</v>
       </c>
     </row>
-    <row r="173" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A173" s="2">
         <v>46059</v>
       </c>
@@ -6715,7 +6726,7 @@
         <v>2.59</v>
       </c>
     </row>
-    <row r="174" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A174" s="2">
         <v>46066</v>
       </c>
@@ -6729,7 +6740,7 @@
         <v>2.63</v>
       </c>
     </row>
-    <row r="175" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A175" s="2">
         <v>46073</v>
       </c>
@@ -6743,7 +6754,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="176" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A176" s="2">
         <v>46080</v>
       </c>
@@ -6754,7 +6765,7 @@
         <v>2.38</v>
       </c>
     </row>
-    <row r="177" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A177" s="2">
         <v>46087</v>
       </c>
@@ -6765,7 +6776,7 @@
         <v>2.23</v>
       </c>
     </row>
-    <row r="178" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A178" s="2">
         <v>46094</v>
       </c>
@@ -6779,7 +6790,7 @@
         <v>2.68</v>
       </c>
     </row>
-    <row r="179" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A179" s="2">
         <v>46101</v>
       </c>
@@ -6793,7 +6804,7 @@
         <v>2.67</v>
       </c>
     </row>
-    <row r="180" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A180" s="2">
         <v>46108</v>
       </c>
@@ -6807,7 +6818,7 @@
         <v>2.68</v>
       </c>
     </row>
-    <row r="181" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A181" s="2">
         <v>46115</v>
       </c>
@@ -6821,7 +6832,7 @@
         <v>2.82</v>
       </c>
     </row>
-    <row r="182" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A182" s="2">
         <v>46122</v>
       </c>
@@ -6835,7 +6846,7 @@
         <v>2.6</v>
       </c>
     </row>
-    <row r="183" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A183" s="2">
         <v>46129</v>
       </c>
@@ -6849,7 +6860,7 @@
         <v>2.75</v>
       </c>
     </row>
-    <row r="184" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A184" s="2">
         <v>46136</v>
       </c>
@@ -6863,7 +6874,7 @@
         <v>2.81</v>
       </c>
     </row>
-    <row r="185" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A185" s="2">
         <v>46143</v>
       </c>
@@ -6877,7 +6888,7 @@
         <v>2.52</v>
       </c>
     </row>
-    <row r="186" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A186" s="2">
         <v>46150</v>
       </c>
@@ -6888,7 +6899,7 @@
         <v>2.59</v>
       </c>
     </row>
-    <row r="187" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A187" s="2">
         <v>46157</v>
       </c>
@@ -6899,7 +6910,7 @@
         <v>2.61</v>
       </c>
     </row>
-    <row r="188" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A188" s="2">
         <v>46164</v>
       </c>
@@ -6910,7 +6921,7 @@
         <v>2.61</v>
       </c>
     </row>
-    <row r="189" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A189" s="2">
         <v>46171</v>
       </c>
@@ -6924,7 +6935,7 @@
         <v>2.36</v>
       </c>
     </row>
-    <row r="190" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A190" s="2">
         <v>46178</v>
       </c>
@@ -6938,7 +6949,7 @@
         <v>2.4700000000000002</v>
       </c>
     </row>
-    <row r="191" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A191" s="2">
         <v>46185</v>
       </c>
@@ -6952,7 +6963,7 @@
         <v>2.46</v>
       </c>
     </row>
-    <row r="192" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A192" s="2">
         <v>46192</v>
       </c>
@@ -6966,7 +6977,7 @@
         <v>2.4500000000000002</v>
       </c>
     </row>
-    <row r="193" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A193" s="2">
         <v>46199</v>
       </c>
@@ -6980,7 +6991,7 @@
         <v>2.42</v>
       </c>
     </row>
-    <row r="194" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A194" s="2">
         <v>46206</v>
       </c>
@@ -6994,7 +7005,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="195" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A195" s="2">
         <v>46213</v>
       </c>
@@ -7008,7 +7019,7 @@
         <v>2.36</v>
       </c>
     </row>
-    <row r="196" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A196" s="2">
         <v>46220</v>
       </c>
@@ -7022,7 +7033,7 @@
         <v>2.6</v>
       </c>
     </row>
-    <row r="197" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A197" s="2">
         <v>46227</v>
       </c>
@@ -7036,7 +7047,7 @@
         <v>2.62</v>
       </c>
     </row>
-    <row r="198" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A198" s="2">
         <v>46234</v>
       </c>
@@ -7050,7 +7061,7 @@
         <v>2.52</v>
       </c>
     </row>
-    <row r="199" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A199" s="2">
         <v>46241</v>
       </c>
@@ -7061,7 +7072,7 @@
         <v>2.2400000000000002</v>
       </c>
     </row>
-    <row r="200" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A200" s="2">
         <v>46248</v>
       </c>
@@ -7072,7 +7083,7 @@
         <v>2.14</v>
       </c>
     </row>
-    <row r="201" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A201" s="2">
         <v>46255</v>
       </c>
@@ -7083,7 +7094,7 @@
         <v>2.27</v>
       </c>
     </row>
-    <row r="202" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A202" s="2">
         <v>46262</v>
       </c>
@@ -7094,7 +7105,7 @@
         <v>2.2200000000000002</v>
       </c>
     </row>
-    <row r="203" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A203" s="2">
         <v>46269</v>
       </c>
@@ -7108,7 +7119,7 @@
         <v>2.5099999999999998</v>
       </c>
     </row>
-    <row r="204" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A204" s="2">
         <v>46276</v>
       </c>
@@ -7122,7 +7133,7 @@
         <v>2.5099999999999998</v>
       </c>
     </row>
-    <row r="205" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A205" s="2">
         <v>46283</v>
       </c>
@@ -7136,7 +7147,7 @@
         <v>2.6</v>
       </c>
     </row>
-    <row r="206" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A206" s="2">
         <v>46290</v>
       </c>
@@ -7150,7 +7161,7 @@
         <v>2.6</v>
       </c>
     </row>
-    <row r="207" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A207" s="2">
         <v>46297</v>
       </c>
@@ -7164,7 +7175,7 @@
         <v>2.54</v>
       </c>
     </row>
-    <row r="208" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A208" s="2">
         <v>46304</v>
       </c>
@@ -7178,7 +7189,7 @@
         <v>2.83</v>
       </c>
     </row>
-    <row r="209" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A209" s="2">
         <v>46311</v>
       </c>
@@ -7190,6 +7201,20 @@
       </c>
       <c r="E209">
         <v>2.82</v>
+      </c>
+    </row>
+    <row r="210" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A210" s="2">
+        <v>46318</v>
+      </c>
+      <c r="B210" t="s">
+        <v>61</v>
+      </c>
+      <c r="D210">
+        <v>2.67</v>
+      </c>
+      <c r="E210">
+        <v>2.81</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data): daily ingest 2026-10-31
NORMAL/SLOWING · GDPNow 3.22 · NY 2.67
</commit_message>
<xml_diff>
--- a/data/cache/nyfed_nowcast_raw.xlsx
+++ b/data/cache/nyfed_nowcast_raw.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\SHARE\drf\TimeSeries\products\Nowcast\automated_nowcast\output\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Nowcast Emergency Port\automated_nowcast\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D76BF4ED-E00C-435A-A463-511C73781D0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A396B063-7EF3-4BF8-A2B1-48E1D9931CC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9400" yWindow="10690" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{ABCE1506-5AF9-4A77-93FF-F8162337FD42}"/>
+    <workbookView xWindow="51090" yWindow="510" windowWidth="18105" windowHeight="19470" activeTab="2" xr2:uid="{ABCE1506-5AF9-4A77-93FF-F8162337FD42}"/>
   </bookViews>
   <sheets>
     <sheet name="New York Fed Nowcast" sheetId="3" r:id="rId1"/>
@@ -33,12 +33,15 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="62">
   <si>
     <t>Forecast Date</t>
   </si>
@@ -1006,6 +1009,9 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="21" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="28" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -1017,9 +1023,6 @@
     </xf>
     <xf numFmtId="0" fontId="24" fillId="34" borderId="0" xfId="44" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="46">
@@ -1604,97 +1607,97 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4E1EDB4-3E22-4B96-9108-06AEDE165285}">
   <dimension ref="B1:I42"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="24.85546875" style="5" customWidth="1"/>
-    <col min="2" max="2" width="129.42578125" style="5" customWidth="1"/>
-    <col min="3" max="16384" width="9.140625" style="5"/>
+    <col min="1" max="1" width="24.81640625" style="5" customWidth="1"/>
+    <col min="2" max="2" width="129.453125" style="5" customWidth="1"/>
+    <col min="3" max="16384" width="9.1796875" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="2:9" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="33" t="s">
+    <row r="1" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="2" spans="2:9" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B2" s="29" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="33"/>
-      <c r="D2" s="33"/>
-      <c r="E2" s="33"/>
-      <c r="F2" s="33"/>
-      <c r="G2" s="33"/>
-      <c r="H2" s="33"/>
-      <c r="I2" s="33"/>
-    </row>
-    <row r="3" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="33"/>
-      <c r="C3" s="33"/>
-      <c r="D3" s="33"/>
-      <c r="E3" s="33"/>
-      <c r="F3" s="33"/>
-      <c r="G3" s="33"/>
-      <c r="H3" s="33"/>
-      <c r="I3" s="33"/>
-    </row>
-    <row r="4" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
+      <c r="F2" s="29"/>
+      <c r="G2" s="29"/>
+      <c r="H2" s="29"/>
+      <c r="I2" s="29"/>
+    </row>
+    <row r="3" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B3" s="29"/>
+      <c r="C3" s="29"/>
+      <c r="D3" s="29"/>
+      <c r="E3" s="29"/>
+      <c r="F3" s="29"/>
+      <c r="G3" s="29"/>
+      <c r="H3" s="29"/>
+      <c r="I3" s="29"/>
+    </row>
+    <row r="4" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B4" s="4" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="2:9" ht="31.5" x14ac:dyDescent="0.5">
+    <row r="8" spans="2:9" ht="31" x14ac:dyDescent="0.7">
       <c r="B8" s="24" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="2:9" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:9" ht="18.5" x14ac:dyDescent="0.45">
       <c r="B9" s="25" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B10" s="6"/>
     </row>
-    <row r="11" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B11" s="20" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="12" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B12" s="7" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="13" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B13" s="9" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="14" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B14" s="9" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="15" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B15" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B17" s="22" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B18" s="23" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="19" spans="2:7" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:7" ht="10.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C19" s="16"/>
       <c r="D19" s="16"/>
       <c r="E19" s="16"/>
       <c r="F19" s="16"/>
       <c r="G19" s="16"/>
     </row>
-    <row r="20" spans="2:7" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B20" s="19" t="s">
         <v>27</v>
       </c>
@@ -1703,7 +1706,7 @@
       <c r="E20" s="8"/>
       <c r="F20" s="8"/>
     </row>
-    <row r="21" spans="2:7" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B21" s="10" t="s">
         <v>28</v>
       </c>
@@ -1712,14 +1715,14 @@
       <c r="E21" s="8"/>
       <c r="F21" s="8"/>
     </row>
-    <row r="22" spans="2:7" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B22" s="10"/>
       <c r="C22" s="8"/>
       <c r="D22" s="8"/>
       <c r="E22" s="8"/>
       <c r="F22" s="8"/>
     </row>
-    <row r="23" spans="2:7" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B23" s="19" t="s">
         <v>29</v>
       </c>
@@ -1728,7 +1731,7 @@
       <c r="E23" s="8"/>
       <c r="F23" s="8"/>
     </row>
-    <row r="24" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B24" s="10" t="s">
         <v>36</v>
       </c>
@@ -1737,55 +1740,55 @@
       <c r="E24" s="8"/>
       <c r="F24" s="8"/>
     </row>
-    <row r="25" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B25" s="10"/>
       <c r="C25" s="8"/>
       <c r="D25" s="8"/>
       <c r="E25" s="8"/>
       <c r="F25" s="8"/>
     </row>
-    <row r="26" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B26" s="19" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="27" spans="2:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:7" ht="29" x14ac:dyDescent="0.35">
       <c r="B27" s="21" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="28" spans="2:7" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B28" s="21"/>
     </row>
-    <row r="29" spans="2:7" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:7" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B29" s="11" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="30" spans="2:7" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:7" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B30" s="13" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="31" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B31" s="18" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="32" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B32" s="18" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="33" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B33" s="17" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="34" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B34" s="13"/>
     </row>
-    <row r="35" spans="2:6" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:6" ht="13" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B35" s="14" t="s">
         <v>23</v>
       </c>
@@ -1794,7 +1797,7 @@
       <c r="E35" s="11"/>
       <c r="F35" s="11"/>
     </row>
-    <row r="36" spans="2:6" ht="16.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:6" ht="16.399999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B36" s="6" t="s">
         <v>24</v>
       </c>
@@ -1803,13 +1806,13 @@
       <c r="E36" s="12"/>
       <c r="F36" s="12"/>
     </row>
-    <row r="38" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C38" s="11"/>
       <c r="D38" s="11"/>
       <c r="E38" s="11"/>
       <c r="F38" s="11"/>
     </row>
-    <row r="42" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:6" x14ac:dyDescent="0.35">
       <c r="C42" s="15"/>
       <c r="D42" s="15"/>
     </row>
@@ -1841,44 +1844,44 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1670CA3-538E-42E7-9E1F-A6A72E94A86A}">
-  <dimension ref="A1:Q210"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:Q211"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="27.140625" customWidth="1"/>
+    <col min="1" max="1" width="27.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-      <c r="H2" s="29"/>
-    </row>
-    <row r="3" spans="1:16" s="3" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B3" s="30" t="s">
+    <row r="1" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="2" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="30"/>
+      <c r="H2" s="30"/>
+    </row>
+    <row r="3" spans="1:16" s="3" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="B3" s="31" t="s">
         <v>25</v>
       </c>
-      <c r="C3" s="31"/>
-      <c r="D3" s="31"/>
-      <c r="E3" s="31"/>
-      <c r="F3" s="31"/>
-      <c r="G3" s="31"/>
-      <c r="H3" s="31"/>
-      <c r="I3" s="31"/>
-    </row>
-    <row r="4" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C4" s="32" t="s">
+      <c r="C3" s="32"/>
+      <c r="D3" s="32"/>
+      <c r="E3" s="32"/>
+      <c r="F3" s="32"/>
+      <c r="G3" s="32"/>
+      <c r="H3" s="32"/>
+      <c r="I3" s="32"/>
+    </row>
+    <row r="4" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="C4" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="32"/>
-    </row>
-    <row r="5" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="D4" s="33"/>
+    </row>
+    <row r="5" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A5"/>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>0</v>
       </c>
@@ -1928,7 +1931,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A7" s="2">
         <v>44897</v>
       </c>
@@ -1936,7 +1939,7 @@
         <v>1.79</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A8" s="2">
         <v>44904</v>
       </c>
@@ -1944,7 +1947,7 @@
         <v>1.76</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A9" s="2">
         <v>44911</v>
       </c>
@@ -1952,7 +1955,7 @@
         <v>1.58</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A10" s="2">
         <v>44918</v>
       </c>
@@ -1960,7 +1963,7 @@
         <v>1.33</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A11" s="2">
         <v>44925</v>
       </c>
@@ -1968,7 +1971,7 @@
         <v>1.31</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A12" s="2">
         <v>44932</v>
       </c>
@@ -1976,7 +1979,7 @@
         <v>1.57</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A13" s="2">
         <v>44939</v>
       </c>
@@ -1984,7 +1987,7 @@
         <v>1.64</v>
       </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A14" s="2">
         <v>44946</v>
       </c>
@@ -1992,7 +1995,7 @@
         <v>0.79</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A15" s="2">
         <v>44953</v>
       </c>
@@ -2000,7 +2003,7 @@
         <v>1.2</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A16" s="2">
         <v>44960</v>
       </c>
@@ -2008,7 +2011,7 @@
         <v>1.59</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" s="2">
         <v>44967</v>
       </c>
@@ -2016,7 +2019,7 @@
         <v>1.48</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" s="2">
         <v>44974</v>
       </c>
@@ -2024,7 +2027,7 @@
         <v>1.1399999999999999</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" s="2">
         <v>44981</v>
       </c>
@@ -2035,7 +2038,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" s="2">
         <v>44988</v>
       </c>
@@ -2046,7 +2049,7 @@
         <v>1.45</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" s="2">
         <v>44995</v>
       </c>
@@ -2057,7 +2060,7 @@
         <v>1.53</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" s="2">
         <v>45002</v>
       </c>
@@ -2068,7 +2071,7 @@
         <v>1.3</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" s="2">
         <v>45009</v>
       </c>
@@ -2079,7 +2082,7 @@
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A24" s="2">
         <v>45016</v>
       </c>
@@ -2090,7 +2093,7 @@
         <v>1.08</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A25" s="2">
         <v>45023</v>
       </c>
@@ -2101,7 +2104,7 @@
         <v>0.67</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A26" s="2">
         <v>45030</v>
       </c>
@@ -2112,7 +2115,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A27" s="2">
         <v>45037</v>
       </c>
@@ -2123,7 +2126,7 @@
         <v>1.1200000000000001</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A28" s="2">
         <v>45044</v>
       </c>
@@ -2134,7 +2137,7 @@
         <v>0.52</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A29" s="2">
         <v>45051</v>
       </c>
@@ -2142,7 +2145,7 @@
         <v>1.28</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A30" s="2">
         <v>45058</v>
       </c>
@@ -2150,7 +2153,7 @@
         <v>1.19</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A31" s="2">
         <v>45065</v>
       </c>
@@ -2158,7 +2161,7 @@
         <v>1.44</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A32" s="2">
         <v>45072</v>
       </c>
@@ -2169,7 +2172,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" s="2">
         <v>45079</v>
       </c>
@@ -2180,7 +2183,7 @@
         <v>1.96</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" s="2">
         <v>45086</v>
       </c>
@@ -2191,7 +2194,7 @@
         <v>1.9</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" s="2">
         <v>45093</v>
       </c>
@@ -2202,7 +2205,7 @@
         <v>1.81</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" s="2">
         <v>45100</v>
       </c>
@@ -2213,7 +2216,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" s="2">
         <v>45107</v>
       </c>
@@ -2224,7 +2227,7 @@
         <v>2.0699999999999998</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" s="2">
         <v>45114</v>
       </c>
@@ -2235,7 +2238,7 @@
         <v>1.53</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" s="2">
         <v>45121</v>
       </c>
@@ -2246,7 +2249,7 @@
         <v>1.51</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" s="2">
         <v>45128</v>
       </c>
@@ -2257,7 +2260,7 @@
         <v>1.25</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" s="2">
         <v>45135</v>
       </c>
@@ -2268,7 +2271,7 @@
         <v>1.93</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" s="2">
         <v>45142</v>
       </c>
@@ -2276,7 +2279,7 @@
         <v>1.81</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43" s="2">
         <v>45149</v>
       </c>
@@ -2284,7 +2287,7 @@
         <v>1.7</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" s="2">
         <v>45156</v>
       </c>
@@ -2292,7 +2295,7 @@
         <v>2.34</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" s="2">
         <v>45163</v>
       </c>
@@ -2300,7 +2303,7 @@
         <v>2.12</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A46" s="2">
         <v>45170</v>
       </c>
@@ -2311,7 +2314,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" s="2">
         <v>45177</v>
       </c>
@@ -2322,7 +2325,7 @@
         <v>2.29</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48" s="2">
         <v>45184</v>
       </c>
@@ -2333,7 +2336,7 @@
         <v>2.35</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A49" s="2">
         <v>45191</v>
       </c>
@@ -2344,7 +2347,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A50" s="2">
         <v>45198</v>
       </c>
@@ -2355,7 +2358,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A51" s="2">
         <v>45205</v>
       </c>
@@ -2366,7 +2369,7 @@
         <v>2.4039999999999999</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A52" s="2">
         <v>45212</v>
       </c>
@@ -2377,7 +2380,7 @@
         <v>2.34</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A53" s="2">
         <v>45219</v>
       </c>
@@ -2388,7 +2391,7 @@
         <v>2.27</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A54" s="2">
         <v>45226</v>
       </c>
@@ -2399,7 +2402,7 @@
         <v>2.79</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A55" s="2">
         <v>45233</v>
       </c>
@@ -2407,7 +2410,7 @@
         <v>2.41</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A56" s="2">
         <v>45240</v>
       </c>
@@ -2415,7 +2418,7 @@
         <v>2.5099999999999998</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A57" s="2">
         <v>45247</v>
       </c>
@@ -2423,7 +2426,7 @@
         <v>2.4500000000000002</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A58" s="2">
         <v>45254</v>
       </c>
@@ -2431,7 +2434,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A59" s="2">
         <v>45261</v>
       </c>
@@ -2442,7 +2445,7 @@
         <v>2.0499999999999998</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A60" s="2">
         <v>45268</v>
       </c>
@@ -2453,7 +2456,7 @@
         <v>2.13</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A61" s="2">
         <v>45275</v>
       </c>
@@ -2464,7 +2467,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A62" s="2">
         <v>45282</v>
       </c>
@@ -2475,7 +2478,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A63" s="2">
         <v>45289</v>
       </c>
@@ -2486,7 +2489,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A64" s="2">
         <v>45296</v>
       </c>
@@ -2497,7 +2500,7 @@
         <v>2.68</v>
       </c>
     </row>
-    <row r="65" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A65" s="2">
         <v>45303</v>
       </c>
@@ -2508,7 +2511,7 @@
         <v>2.4500000000000002</v>
       </c>
     </row>
-    <row r="66" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A66" s="2">
         <v>45310</v>
       </c>
@@ -2529,7 +2532,7 @@
       <c r="O66" s="26"/>
       <c r="P66" s="26"/>
     </row>
-    <row r="67" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A67" s="2">
         <v>45317</v>
       </c>
@@ -2550,7 +2553,7 @@
       <c r="O67" s="26"/>
       <c r="P67" s="26"/>
     </row>
-    <row r="68" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A68" s="2">
         <v>45324</v>
       </c>
@@ -2569,7 +2572,7 @@
       <c r="O68" s="26"/>
       <c r="P68" s="26"/>
     </row>
-    <row r="69" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A69" s="2">
         <v>45331</v>
       </c>
@@ -2588,7 +2591,7 @@
       <c r="O69" s="26"/>
       <c r="P69" s="26"/>
     </row>
-    <row r="70" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A70" s="2">
         <v>45338</v>
       </c>
@@ -2607,7 +2610,7 @@
       <c r="O70" s="26"/>
       <c r="P70" s="26"/>
     </row>
-    <row r="71" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A71" s="2">
         <v>45345</v>
       </c>
@@ -2626,7 +2629,7 @@
       <c r="O71" s="26"/>
       <c r="P71" s="26"/>
     </row>
-    <row r="72" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A72" s="2">
         <v>45352</v>
       </c>
@@ -2647,7 +2650,7 @@
       <c r="O72" s="26"/>
       <c r="P72" s="26"/>
     </row>
-    <row r="73" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A73" s="2">
         <v>45359</v>
       </c>
@@ -2668,7 +2671,7 @@
       <c r="O73" s="26"/>
       <c r="P73" s="26"/>
     </row>
-    <row r="74" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A74" s="2">
         <v>45366</v>
       </c>
@@ -2689,7 +2692,7 @@
       <c r="O74" s="26"/>
       <c r="P74" s="26"/>
     </row>
-    <row r="75" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A75" s="2">
         <v>45373</v>
       </c>
@@ -2710,7 +2713,7 @@
       <c r="O75" s="26"/>
       <c r="P75" s="26"/>
     </row>
-    <row r="76" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A76" s="2">
         <v>45380</v>
       </c>
@@ -2731,7 +2734,7 @@
       <c r="O76" s="26"/>
       <c r="P76" s="26"/>
     </row>
-    <row r="77" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A77" s="2">
         <v>45387</v>
       </c>
@@ -2752,7 +2755,7 @@
       <c r="O77" s="26"/>
       <c r="P77" s="26"/>
     </row>
-    <row r="78" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A78" s="2">
         <v>45394</v>
       </c>
@@ -2773,7 +2776,7 @@
       <c r="O78" s="26"/>
       <c r="P78" s="26"/>
     </row>
-    <row r="79" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A79" s="2">
         <v>45401</v>
       </c>
@@ -2794,7 +2797,7 @@
       <c r="O79" s="26"/>
       <c r="P79" s="26"/>
     </row>
-    <row r="80" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A80" s="2">
         <v>45408</v>
       </c>
@@ -2815,7 +2818,7 @@
       <c r="O80" s="26"/>
       <c r="P80" s="26"/>
     </row>
-    <row r="81" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A81" s="2">
         <v>45415</v>
       </c>
@@ -2834,7 +2837,7 @@
       <c r="O81" s="26"/>
       <c r="P81" s="26"/>
     </row>
-    <row r="82" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A82" s="2">
         <v>45422</v>
       </c>
@@ -2853,7 +2856,7 @@
       <c r="O82" s="26"/>
       <c r="P82" s="26"/>
     </row>
-    <row r="83" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A83" s="2">
         <v>45429</v>
       </c>
@@ -2872,7 +2875,7 @@
       <c r="O83" s="26"/>
       <c r="P83" s="26"/>
     </row>
-    <row r="84" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A84" s="2">
         <v>45436</v>
       </c>
@@ -2891,7 +2894,7 @@
       <c r="O84" s="26"/>
       <c r="P84" s="26"/>
     </row>
-    <row r="85" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A85" s="2">
         <v>45443</v>
       </c>
@@ -2912,7 +2915,7 @@
       <c r="O85" s="26"/>
       <c r="P85" s="26"/>
     </row>
-    <row r="86" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A86" s="2">
         <v>45450</v>
       </c>
@@ -2933,7 +2936,7 @@
       <c r="O86" s="26"/>
       <c r="P86" s="26"/>
     </row>
-    <row r="87" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A87" s="2">
         <v>45457</v>
       </c>
@@ -2954,7 +2957,7 @@
       <c r="O87" s="26"/>
       <c r="P87" s="26"/>
     </row>
-    <row r="88" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A88" s="2">
         <v>45464</v>
       </c>
@@ -2975,7 +2978,7 @@
       <c r="O88" s="26"/>
       <c r="P88" s="26"/>
     </row>
-    <row r="89" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A89" s="2">
         <v>45471</v>
       </c>
@@ -2996,7 +2999,7 @@
       <c r="O89" s="26"/>
       <c r="P89" s="26"/>
     </row>
-    <row r="90" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A90" s="2">
         <v>45478</v>
       </c>
@@ -3017,7 +3020,7 @@
       <c r="O90" s="26"/>
       <c r="P90" s="26"/>
     </row>
-    <row r="91" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A91" s="2">
         <v>45485</v>
       </c>
@@ -3038,7 +3041,7 @@
       <c r="O91" s="26"/>
       <c r="P91" s="26"/>
     </row>
-    <row r="92" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A92" s="2">
         <v>45492</v>
       </c>
@@ -3059,7 +3062,7 @@
       <c r="O92" s="26"/>
       <c r="P92" s="26"/>
     </row>
-    <row r="93" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A93" s="2">
         <v>45499</v>
       </c>
@@ -3080,7 +3083,7 @@
       <c r="O93" s="26"/>
       <c r="P93" s="26"/>
     </row>
-    <row r="94" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A94" s="2">
         <v>45506</v>
       </c>
@@ -3099,7 +3102,7 @@
       <c r="O94" s="26"/>
       <c r="P94" s="26"/>
     </row>
-    <row r="95" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A95" s="2">
         <v>45513</v>
       </c>
@@ -3107,7 +3110,7 @@
         <v>2.238</v>
       </c>
     </row>
-    <row r="96" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A96" s="2">
         <v>45520</v>
       </c>
@@ -3115,7 +3118,7 @@
         <v>1.84</v>
       </c>
     </row>
-    <row r="97" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A97" s="2">
         <v>45527</v>
       </c>
@@ -3123,7 +3126,7 @@
         <v>1.9410000000000001</v>
       </c>
     </row>
-    <row r="98" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A98" s="2">
         <v>45534</v>
       </c>
@@ -3134,7 +3137,7 @@
         <v>2.1160000000000001</v>
       </c>
     </row>
-    <row r="99" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A99" s="2">
         <v>45541</v>
       </c>
@@ -3145,7 +3148,7 @@
         <v>2.2130000000000001</v>
       </c>
     </row>
-    <row r="100" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A100" s="2">
         <v>45548</v>
       </c>
@@ -3156,7 +3159,7 @@
         <v>2.1749999999999998</v>
       </c>
     </row>
-    <row r="101" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A101" s="2">
         <v>45555</v>
       </c>
@@ -3167,7 +3170,7 @@
         <v>2.74</v>
       </c>
     </row>
-    <row r="102" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A102" s="2">
         <v>45562</v>
       </c>
@@ -3178,7 +3181,7 @@
         <v>2.7970000000000002</v>
       </c>
     </row>
-    <row r="103" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A103" s="2">
         <v>45569</v>
       </c>
@@ -3189,7 +3192,7 @@
         <v>2.7629999999999999</v>
       </c>
     </row>
-    <row r="104" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A104" s="2">
         <v>45576</v>
       </c>
@@ -3200,7 +3203,7 @@
         <v>2.7530000000000001</v>
       </c>
     </row>
-    <row r="105" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A105" s="2">
         <v>45583</v>
       </c>
@@ -3211,7 +3214,7 @@
         <v>2.6070000000000002</v>
       </c>
     </row>
-    <row r="106" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A106" s="2">
         <v>45590</v>
       </c>
@@ -3222,7 +3225,7 @@
         <v>2.4649999999999999</v>
       </c>
     </row>
-    <row r="107" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A107" s="2">
         <v>45597</v>
       </c>
@@ -3233,7 +3236,7 @@
         <v>2.0070000000000001</v>
       </c>
     </row>
-    <row r="108" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A108" s="2">
         <v>45604</v>
       </c>
@@ -3241,7 +3244,7 @@
         <v>2.0590000000000002</v>
       </c>
     </row>
-    <row r="109" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A109" s="2">
         <v>45611</v>
       </c>
@@ -3249,7 +3252,7 @@
         <v>2.0640000000000001</v>
       </c>
     </row>
-    <row r="110" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A110" s="2">
         <v>45618</v>
       </c>
@@ -3257,7 +3260,7 @@
         <v>1.909</v>
       </c>
     </row>
-    <row r="111" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A111" s="2">
         <v>45625</v>
       </c>
@@ -3265,7 +3268,7 @@
         <v>1.8049999999999999</v>
       </c>
     </row>
-    <row r="112" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A112" s="2">
         <v>45632</v>
       </c>
@@ -3276,7 +3279,7 @@
         <v>2.3769999999999998</v>
       </c>
     </row>
-    <row r="113" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A113" s="2">
         <v>45639</v>
       </c>
@@ -3287,7 +3290,7 @@
         <v>2.2909999999999999</v>
       </c>
     </row>
-    <row r="114" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A114" s="2">
         <v>45646</v>
       </c>
@@ -3298,7 +3301,7 @@
         <v>2.1269999999999998</v>
       </c>
     </row>
-    <row r="115" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A115" s="2">
         <v>45653</v>
       </c>
@@ -3309,7 +3312,7 @@
         <v>2.0819999999999999</v>
       </c>
     </row>
-    <row r="116" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A116" s="2">
         <v>45660</v>
       </c>
@@ -3320,7 +3323,7 @@
         <v>2.2080000000000002</v>
       </c>
     </row>
-    <row r="117" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A117" s="2">
         <v>45667</v>
       </c>
@@ -3331,7 +3334,7 @@
         <v>2.738</v>
       </c>
     </row>
-    <row r="118" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A118" s="2">
         <v>45674</v>
       </c>
@@ -3342,7 +3345,7 @@
         <v>2.9994999999999998</v>
       </c>
     </row>
-    <row r="119" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A119" s="2">
         <v>45681</v>
       </c>
@@ -3353,7 +3356,7 @@
         <v>2.9994999999999998</v>
       </c>
     </row>
-    <row r="120" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A120" s="2">
         <v>45688</v>
       </c>
@@ -3364,7 +3367,7 @@
         <v>2.915</v>
       </c>
     </row>
-    <row r="121" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A121" s="2">
         <v>45695</v>
       </c>
@@ -3372,7 +3375,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="122" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A122" s="2">
         <v>45702</v>
       </c>
@@ -3380,7 +3383,7 @@
         <v>3.0150000000000001</v>
       </c>
     </row>
-    <row r="123" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A123" s="2">
         <v>45709</v>
       </c>
@@ -3388,7 +3391,7 @@
         <v>2.9460000000000002</v>
       </c>
     </row>
-    <row r="124" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A124" s="2">
         <v>45716</v>
       </c>
@@ -3399,7 +3402,7 @@
         <v>2.8490000000000002</v>
       </c>
     </row>
-    <row r="125" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A125" s="2">
         <v>45723</v>
       </c>
@@ -3410,7 +3413,7 @@
         <v>2.5750000000000002</v>
       </c>
     </row>
-    <row r="126" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A126" s="2">
         <v>45730</v>
       </c>
@@ -3421,7 +3424,7 @@
         <v>2.6579999999999999</v>
       </c>
     </row>
-    <row r="127" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A127" s="2">
         <v>45737</v>
       </c>
@@ -3432,7 +3435,7 @@
         <v>2.641</v>
       </c>
     </row>
-    <row r="128" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A128" s="2">
         <v>45744</v>
       </c>
@@ -3443,7 +3446,7 @@
         <v>2.629</v>
       </c>
     </row>
-    <row r="129" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A129" s="2">
         <v>45751</v>
       </c>
@@ -3454,7 +3457,7 @@
         <v>2.4380000000000002</v>
       </c>
     </row>
-    <row r="130" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A130" s="2">
         <v>45758</v>
       </c>
@@ -3465,7 +3468,7 @@
         <v>2.6179999999999999</v>
       </c>
     </row>
-    <row r="131" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A131" s="2">
         <v>45765</v>
       </c>
@@ -3476,7 +3479,7 @@
         <v>2.605</v>
       </c>
     </row>
-    <row r="132" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A132" s="2">
         <v>45772</v>
       </c>
@@ -3487,7 +3490,7 @@
         <v>2.7149999999999999</v>
       </c>
     </row>
-    <row r="133" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A133" s="2">
         <v>45779</v>
       </c>
@@ -3498,7 +3501,7 @@
         <v>2.335</v>
       </c>
     </row>
-    <row r="134" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A134" s="2">
         <v>45786</v>
       </c>
@@ -3506,7 +3509,7 @@
         <v>2.4249999999999998</v>
       </c>
     </row>
-    <row r="135" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A135" s="2">
         <v>45793</v>
       </c>
@@ -3514,7 +3517,7 @@
         <v>2.3460000000000001</v>
       </c>
     </row>
-    <row r="136" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A136" s="2">
         <v>45800</v>
       </c>
@@ -3522,7 +3525,7 @@
         <v>2.4289999999999998</v>
       </c>
     </row>
-    <row r="137" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A137" s="2">
         <v>45807</v>
       </c>
@@ -3533,7 +3536,7 @@
         <v>2.5379999999999998</v>
       </c>
     </row>
-    <row r="138" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A138" s="2">
         <v>45814</v>
       </c>
@@ -3544,7 +3547,7 @@
         <v>2.3980000000000001</v>
       </c>
     </row>
-    <row r="139" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A139" s="2">
         <v>45821</v>
       </c>
@@ -3555,7 +3558,7 @@
         <v>2.504</v>
       </c>
     </row>
-    <row r="140" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A140" s="2">
         <v>45828</v>
       </c>
@@ -3566,7 +3569,7 @@
         <v>2.0609999999999999</v>
       </c>
     </row>
-    <row r="141" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A141" s="2">
         <v>45835</v>
       </c>
@@ -3577,7 +3580,7 @@
         <v>1.917</v>
       </c>
     </row>
-    <row r="142" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A142" s="2">
         <v>45842</v>
       </c>
@@ -3588,7 +3591,7 @@
         <v>1.7809999999999999</v>
       </c>
     </row>
-    <row r="143" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A143" s="2">
         <v>45849</v>
       </c>
@@ -3599,7 +3602,7 @@
         <v>1.78</v>
       </c>
     </row>
-    <row r="144" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A144" s="2">
         <v>45856</v>
       </c>
@@ -3610,7 +3613,7 @@
         <v>2.44</v>
       </c>
     </row>
-    <row r="145" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A145" s="2">
         <v>45863</v>
       </c>
@@ -3621,7 +3624,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="146" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A146" s="2">
         <v>45870</v>
       </c>
@@ -3632,7 +3635,7 @@
         <v>2.12</v>
       </c>
     </row>
-    <row r="147" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A147" s="2">
         <v>45877</v>
       </c>
@@ -3640,7 +3643,7 @@
         <v>2.02</v>
       </c>
     </row>
-    <row r="148" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A148" s="2">
         <v>45884</v>
       </c>
@@ -3648,7 +3651,7 @@
         <v>2.06</v>
       </c>
     </row>
-    <row r="149" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A149" s="2">
         <v>45891</v>
       </c>
@@ -3656,7 +3659,7 @@
         <v>2.0099999999999998</v>
       </c>
     </row>
-    <row r="150" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A150" s="2">
         <v>45898</v>
       </c>
@@ -3667,7 +3670,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="151" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A151" s="2">
         <v>45905</v>
       </c>
@@ -3678,7 +3681,7 @@
         <v>2.2799999999999998</v>
       </c>
     </row>
-    <row r="152" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A152" s="2">
         <v>45912</v>
       </c>
@@ -3689,7 +3692,7 @@
         <v>2.16</v>
       </c>
     </row>
-    <row r="153" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A153" s="2">
         <v>45919</v>
       </c>
@@ -3700,7 +3703,7 @@
         <v>2.1800000000000002</v>
       </c>
     </row>
-    <row r="154" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A154" s="2">
         <v>45926</v>
       </c>
@@ -3711,7 +3714,7 @@
         <v>2.46</v>
       </c>
     </row>
-    <row r="155" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A155" s="2">
         <v>45933</v>
       </c>
@@ -3722,7 +3725,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="156" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A156" s="2">
         <v>45940</v>
       </c>
@@ -3733,7 +3736,7 @@
         <v>2.23</v>
       </c>
     </row>
-    <row r="157" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A157" s="2">
         <v>45947</v>
       </c>
@@ -3744,7 +3747,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="158" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A158" s="2">
         <v>45954</v>
       </c>
@@ -3755,7 +3758,7 @@
         <v>2.2599999999999998</v>
       </c>
     </row>
-    <row r="159" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A159" s="2">
         <v>45961</v>
       </c>
@@ -3766,7 +3769,7 @@
         <v>2.2599999999999998</v>
       </c>
     </row>
-    <row r="160" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A160" s="2">
         <v>45968</v>
       </c>
@@ -3777,7 +3780,7 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="161" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A161" s="2">
         <v>45975</v>
       </c>
@@ -3788,7 +3791,7 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="162" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A162" s="2">
         <v>45982</v>
       </c>
@@ -3799,7 +3802,7 @@
         <v>2.31</v>
       </c>
     </row>
-    <row r="163" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A163" s="2">
         <v>45989</v>
       </c>
@@ -3813,7 +3816,7 @@
         <v>2.66</v>
       </c>
     </row>
-    <row r="164" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A164" s="2">
         <v>45996</v>
       </c>
@@ -3824,7 +3827,7 @@
         <v>2.2200000000000002</v>
       </c>
     </row>
-    <row r="165" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A165" s="2">
         <v>46003</v>
       </c>
@@ -3835,7 +3838,7 @@
         <v>2.2400000000000002</v>
       </c>
     </row>
-    <row r="166" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A166" s="2">
         <v>46010</v>
       </c>
@@ -3846,7 +3849,7 @@
         <v>2.11</v>
       </c>
     </row>
-    <row r="167" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A167" s="2">
         <v>46017</v>
       </c>
@@ -3857,7 +3860,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="168" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A168" s="2">
         <v>46024</v>
       </c>
@@ -3868,7 +3871,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="169" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A169" s="2">
         <v>46031</v>
       </c>
@@ -3879,7 +3882,7 @@
         <v>2.61</v>
       </c>
     </row>
-    <row r="170" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A170" s="2">
         <v>46038</v>
       </c>
@@ -3890,7 +3893,7 @@
         <v>2.75</v>
       </c>
     </row>
-    <row r="171" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A171" s="2">
         <v>46045</v>
       </c>
@@ -3901,7 +3904,7 @@
         <v>2.73</v>
       </c>
     </row>
-    <row r="172" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A172" s="2">
         <v>46052</v>
       </c>
@@ -3912,7 +3915,7 @@
         <v>2.73</v>
       </c>
     </row>
-    <row r="173" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A173" s="2">
         <v>46059</v>
       </c>
@@ -3923,7 +3926,7 @@
         <v>2.59</v>
       </c>
     </row>
-    <row r="174" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A174" s="2">
         <v>46066</v>
       </c>
@@ -3934,7 +3937,7 @@
         <v>2.63</v>
       </c>
     </row>
-    <row r="175" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A175" s="2">
         <v>46073</v>
       </c>
@@ -3945,7 +3948,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="176" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A176" s="2">
         <v>46080</v>
       </c>
@@ -3953,7 +3956,7 @@
         <v>2.38</v>
       </c>
     </row>
-    <row r="177" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A177" s="2">
         <v>46087</v>
       </c>
@@ -3961,7 +3964,7 @@
         <v>2.23</v>
       </c>
     </row>
-    <row r="178" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A178" s="2">
         <v>46094</v>
       </c>
@@ -3972,7 +3975,7 @@
         <v>2.68</v>
       </c>
     </row>
-    <row r="179" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A179" s="2">
         <v>46101</v>
       </c>
@@ -3983,7 +3986,7 @@
         <v>2.67</v>
       </c>
     </row>
-    <row r="180" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A180" s="2">
         <v>46108</v>
       </c>
@@ -3994,7 +3997,7 @@
         <v>2.68</v>
       </c>
     </row>
-    <row r="181" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A181" s="2">
         <v>46115</v>
       </c>
@@ -4005,7 +4008,7 @@
         <v>2.82</v>
       </c>
     </row>
-    <row r="182" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A182" s="2">
         <v>46122</v>
       </c>
@@ -4016,7 +4019,7 @@
         <v>2.6</v>
       </c>
     </row>
-    <row r="183" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A183" s="2">
         <v>46129</v>
       </c>
@@ -4027,7 +4030,7 @@
         <v>2.75</v>
       </c>
     </row>
-    <row r="184" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A184" s="2">
         <v>46136</v>
       </c>
@@ -4038,7 +4041,7 @@
         <v>2.81</v>
       </c>
     </row>
-    <row r="185" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A185" s="2">
         <v>46143</v>
       </c>
@@ -4049,7 +4052,7 @@
         <v>2.52</v>
       </c>
     </row>
-    <row r="186" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A186" s="2">
         <v>46150</v>
       </c>
@@ -4057,7 +4060,7 @@
         <v>2.59</v>
       </c>
     </row>
-    <row r="187" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A187" s="2">
         <v>46157</v>
       </c>
@@ -4065,7 +4068,7 @@
         <v>2.61</v>
       </c>
     </row>
-    <row r="188" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A188" s="2">
         <v>46164</v>
       </c>
@@ -4073,7 +4076,7 @@
         <v>2.61</v>
       </c>
     </row>
-    <row r="189" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A189" s="2">
         <v>46171</v>
       </c>
@@ -4084,7 +4087,7 @@
         <v>2.36</v>
       </c>
     </row>
-    <row r="190" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A190" s="2">
         <v>46178</v>
       </c>
@@ -4095,7 +4098,7 @@
         <v>2.4700000000000002</v>
       </c>
     </row>
-    <row r="191" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A191" s="2">
         <v>46185</v>
       </c>
@@ -4106,7 +4109,7 @@
         <v>2.46</v>
       </c>
     </row>
-    <row r="192" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A192" s="2">
         <v>46192</v>
       </c>
@@ -4117,7 +4120,7 @@
         <v>2.4500000000000002</v>
       </c>
     </row>
-    <row r="193" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A193" s="2">
         <v>46199</v>
       </c>
@@ -4128,7 +4131,7 @@
         <v>2.42</v>
       </c>
     </row>
-    <row r="194" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A194" s="2">
         <v>46206</v>
       </c>
@@ -4139,7 +4142,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="195" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A195" s="2">
         <v>46213</v>
       </c>
@@ -4150,7 +4153,7 @@
         <v>2.36</v>
       </c>
     </row>
-    <row r="196" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A196" s="2">
         <v>46220</v>
       </c>
@@ -4161,7 +4164,7 @@
         <v>2.6</v>
       </c>
     </row>
-    <row r="197" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A197" s="2">
         <v>46227</v>
       </c>
@@ -4172,7 +4175,7 @@
         <v>2.62</v>
       </c>
     </row>
-    <row r="198" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A198" s="2">
         <v>46234</v>
       </c>
@@ -4183,7 +4186,7 @@
         <v>2.52</v>
       </c>
     </row>
-    <row r="199" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A199" s="2">
         <v>46241</v>
       </c>
@@ -4191,7 +4194,7 @@
         <v>2.2400000000000002</v>
       </c>
     </row>
-    <row r="200" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A200" s="2">
         <v>46248</v>
       </c>
@@ -4199,7 +4202,7 @@
         <v>2.14</v>
       </c>
     </row>
-    <row r="201" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A201" s="2">
         <v>46255</v>
       </c>
@@ -4207,7 +4210,7 @@
         <v>2.27</v>
       </c>
     </row>
-    <row r="202" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A202" s="2">
         <v>46262</v>
       </c>
@@ -4215,7 +4218,7 @@
         <v>2.2200000000000002</v>
       </c>
     </row>
-    <row r="203" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A203" s="2">
         <v>46269</v>
       </c>
@@ -4226,7 +4229,7 @@
         <v>2.5099999999999998</v>
       </c>
     </row>
-    <row r="204" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A204" s="2">
         <v>46276</v>
       </c>
@@ -4237,7 +4240,7 @@
         <v>2.5099999999999998</v>
       </c>
     </row>
-    <row r="205" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A205" s="2">
         <v>46283</v>
       </c>
@@ -4248,7 +4251,7 @@
         <v>2.6</v>
       </c>
     </row>
-    <row r="206" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A206" s="2">
         <v>46290</v>
       </c>
@@ -4259,7 +4262,7 @@
         <v>2.6</v>
       </c>
     </row>
-    <row r="207" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A207" s="2">
         <v>46297</v>
       </c>
@@ -4270,7 +4273,7 @@
         <v>2.54</v>
       </c>
     </row>
-    <row r="208" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A208" s="2">
         <v>46304</v>
       </c>
@@ -4281,7 +4284,7 @@
         <v>2.83</v>
       </c>
     </row>
-    <row r="209" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A209" s="2">
         <v>46311</v>
       </c>
@@ -4292,7 +4295,7 @@
         <v>2.82</v>
       </c>
     </row>
-    <row r="210" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A210" s="2">
         <v>46318</v>
       </c>
@@ -4301,6 +4304,17 @@
       </c>
       <c r="Q210">
         <v>2.81</v>
+      </c>
+    </row>
+    <row r="211" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A211" s="2">
+        <v>46325</v>
+      </c>
+      <c r="P211">
+        <v>2.67</v>
+      </c>
+      <c r="Q211">
+        <v>2.9</v>
       </c>
     </row>
   </sheetData>
@@ -4324,48 +4338,48 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{596092BD-1EF6-4EC0-96F0-3BB4B0DA037F}">
-  <dimension ref="A1:I210"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:I211"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="23.42578125" customWidth="1"/>
-    <col min="2" max="2" width="18.85546875" customWidth="1"/>
-    <col min="3" max="3" width="24.85546875" customWidth="1"/>
-    <col min="4" max="4" width="25.140625" customWidth="1"/>
-    <col min="5" max="5" width="23.42578125" customWidth="1"/>
+    <col min="1" max="1" width="23.453125" customWidth="1"/>
+    <col min="2" max="2" width="18.81640625" customWidth="1"/>
+    <col min="3" max="3" width="24.81640625" customWidth="1"/>
+    <col min="4" max="4" width="25.1796875" customWidth="1"/>
+    <col min="5" max="5" width="23.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-      <c r="H2" s="29"/>
-    </row>
-    <row r="3" spans="1:9" s="3" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B3" s="30" t="s">
+    <row r="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="2" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="30"/>
+      <c r="H2" s="30"/>
+    </row>
+    <row r="3" spans="1:9" s="3" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="B3" s="31" t="s">
         <v>25</v>
       </c>
-      <c r="C3" s="31"/>
-      <c r="D3" s="31"/>
-      <c r="E3" s="31"/>
-      <c r="F3" s="31"/>
-      <c r="G3" s="31"/>
-      <c r="H3" s="31"/>
-      <c r="I3" s="31"/>
-    </row>
-    <row r="4" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C4" s="32" t="s">
+      <c r="C3" s="32"/>
+      <c r="D3" s="32"/>
+      <c r="E3" s="32"/>
+      <c r="F3" s="32"/>
+      <c r="G3" s="32"/>
+      <c r="H3" s="32"/>
+      <c r="I3" s="32"/>
+    </row>
+    <row r="4" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="C4" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="32"/>
-    </row>
-    <row r="5" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="D4" s="33"/>
+    </row>
+    <row r="5" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A5"/>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -4382,7 +4396,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" s="2">
         <v>44897</v>
       </c>
@@ -4393,7 +4407,7 @@
         <v>1.79</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" s="2">
         <v>44904</v>
       </c>
@@ -4404,7 +4418,7 @@
         <v>1.76</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" s="2">
         <v>44911</v>
       </c>
@@ -4415,7 +4429,7 @@
         <v>1.58</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" s="2">
         <v>44918</v>
       </c>
@@ -4426,7 +4440,7 @@
         <v>1.33</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" s="2">
         <v>44925</v>
       </c>
@@ -4437,7 +4451,7 @@
         <v>1.31</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" s="2">
         <v>44932</v>
       </c>
@@ -4448,7 +4462,7 @@
         <v>1.57</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" s="2">
         <v>44939</v>
       </c>
@@ -4459,7 +4473,7 @@
         <v>1.64</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" s="2">
         <v>44946</v>
       </c>
@@ -4470,7 +4484,7 @@
         <v>0.79</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" s="2">
         <v>44953</v>
       </c>
@@ -4481,7 +4495,7 @@
         <v>1.2</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" s="2">
         <v>44960</v>
       </c>
@@ -4492,7 +4506,7 @@
         <v>1.59</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" s="2">
         <v>44967</v>
       </c>
@@ -4503,7 +4517,7 @@
         <v>1.48</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" s="2">
         <v>44974</v>
       </c>
@@ -4514,7 +4528,7 @@
         <v>1.1399999999999999</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" s="2">
         <v>44981</v>
       </c>
@@ -4528,7 +4542,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" s="2">
         <v>44988</v>
       </c>
@@ -4542,7 +4556,7 @@
         <v>1.45</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" s="2">
         <v>44995</v>
       </c>
@@ -4556,7 +4570,7 @@
         <v>1.53</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" s="2">
         <v>45002</v>
       </c>
@@ -4570,7 +4584,7 @@
         <v>1.3</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" s="2">
         <v>45009</v>
       </c>
@@ -4584,7 +4598,7 @@
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" s="2">
         <v>45016</v>
       </c>
@@ -4598,7 +4612,7 @@
         <v>1.08</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" s="2">
         <v>45023</v>
       </c>
@@ -4612,7 +4626,7 @@
         <v>0.67</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" s="2">
         <v>45030</v>
       </c>
@@ -4626,7 +4640,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" s="2">
         <v>45037</v>
       </c>
@@ -4640,7 +4654,7 @@
         <v>1.1200000000000001</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" s="2">
         <v>45044</v>
       </c>
@@ -4654,7 +4668,7 @@
         <v>0.52</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" s="2">
         <v>45051</v>
       </c>
@@ -4665,7 +4679,7 @@
         <v>1.28</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" s="2">
         <v>45058</v>
       </c>
@@ -4676,7 +4690,7 @@
         <v>1.19</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" s="2">
         <v>45065</v>
       </c>
@@ -4687,7 +4701,7 @@
         <v>1.44</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" s="2">
         <v>45072</v>
       </c>
@@ -4701,7 +4715,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" s="2">
         <v>45079</v>
       </c>
@@ -4715,7 +4729,7 @@
         <v>1.96</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" s="2">
         <v>45086</v>
       </c>
@@ -4729,7 +4743,7 @@
         <v>1.9</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" s="2">
         <v>45093</v>
       </c>
@@ -4743,7 +4757,7 @@
         <v>1.81</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" s="2">
         <v>45100</v>
       </c>
@@ -4757,7 +4771,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" s="2">
         <v>45107</v>
       </c>
@@ -4771,7 +4785,7 @@
         <v>2.0699999999999998</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" s="2">
         <v>45114</v>
       </c>
@@ -4785,7 +4799,7 @@
         <v>1.53</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" s="2">
         <v>45121</v>
       </c>
@@ -4799,7 +4813,7 @@
         <v>1.51</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" s="2">
         <v>45128</v>
       </c>
@@ -4813,7 +4827,7 @@
         <v>1.25</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" s="2">
         <v>45135</v>
       </c>
@@ -4827,7 +4841,7 @@
         <v>1.93</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" s="2">
         <v>45142</v>
       </c>
@@ -4838,7 +4852,7 @@
         <v>1.81</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43" s="2">
         <v>45149</v>
       </c>
@@ -4849,7 +4863,7 @@
         <v>1.7</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" s="2">
         <v>45156</v>
       </c>
@@ -4860,7 +4874,7 @@
         <v>2.34</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" s="2">
         <v>45163</v>
       </c>
@@ -4871,7 +4885,7 @@
         <v>2.12</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A46" s="2">
         <v>45170</v>
       </c>
@@ -4885,7 +4899,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" s="2">
         <v>45177</v>
       </c>
@@ -4899,7 +4913,7 @@
         <v>2.29</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48" s="2">
         <v>45184</v>
       </c>
@@ -4913,7 +4927,7 @@
         <v>2.35</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A49" s="2">
         <v>45191</v>
       </c>
@@ -4927,7 +4941,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A50" s="2">
         <v>45198</v>
       </c>
@@ -4941,7 +4955,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A51" s="2">
         <v>45205</v>
       </c>
@@ -4955,7 +4969,7 @@
         <v>2.4039999999999999</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A52" s="2">
         <v>45212</v>
       </c>
@@ -4969,7 +4983,7 @@
         <v>2.34</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A53" s="2">
         <v>45219</v>
       </c>
@@ -4983,7 +4997,7 @@
         <v>2.27</v>
       </c>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A54" s="2">
         <v>45226</v>
       </c>
@@ -4997,7 +5011,7 @@
         <v>2.79</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A55" s="2">
         <v>45233</v>
       </c>
@@ -5008,7 +5022,7 @@
         <v>2.41</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A56" s="2">
         <v>45240</v>
       </c>
@@ -5019,7 +5033,7 @@
         <v>2.5099999999999998</v>
       </c>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A57" s="2">
         <v>45247</v>
       </c>
@@ -5030,7 +5044,7 @@
         <v>2.4500000000000002</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A58" s="2">
         <v>45254</v>
       </c>
@@ -5041,7 +5055,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A59" s="2">
         <v>45261</v>
       </c>
@@ -5055,7 +5069,7 @@
         <v>2.0499999999999998</v>
       </c>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A60" s="2">
         <v>45268</v>
       </c>
@@ -5069,7 +5083,7 @@
         <v>2.13</v>
       </c>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A61" s="2">
         <v>45275</v>
       </c>
@@ -5083,7 +5097,7 @@
         <v>1.98</v>
       </c>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A62" s="2">
         <v>45282</v>
       </c>
@@ -5097,7 +5111,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A63" s="2">
         <v>45289</v>
       </c>
@@ -5111,7 +5125,7 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A64" s="2">
         <v>45296</v>
       </c>
@@ -5128,7 +5142,7 @@
       <c r="F64" s="26"/>
       <c r="G64" s="26"/>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A65" s="2">
         <v>45303</v>
       </c>
@@ -5145,7 +5159,7 @@
       <c r="F65" s="26"/>
       <c r="G65" s="26"/>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A66" s="2">
         <v>45310</v>
       </c>
@@ -5162,7 +5176,7 @@
       <c r="F66" s="26"/>
       <c r="G66" s="26"/>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A67" s="2">
         <v>45317</v>
       </c>
@@ -5179,7 +5193,7 @@
       <c r="F67" s="26"/>
       <c r="G67" s="26"/>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A68" s="2">
         <v>45324</v>
       </c>
@@ -5194,7 +5208,7 @@
       <c r="F68" s="26"/>
       <c r="G68" s="26"/>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A69" s="2">
         <v>45331</v>
       </c>
@@ -5209,7 +5223,7 @@
       <c r="F69" s="26"/>
       <c r="G69" s="26"/>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A70" s="2">
         <v>45338</v>
       </c>
@@ -5224,7 +5238,7 @@
       <c r="F70" s="26"/>
       <c r="G70" s="26"/>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A71" s="2">
         <v>45345</v>
       </c>
@@ -5239,7 +5253,7 @@
       <c r="F71" s="26"/>
       <c r="G71" s="26"/>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A72" s="2">
         <v>45352</v>
       </c>
@@ -5256,7 +5270,7 @@
       <c r="F72" s="26"/>
       <c r="G72" s="26"/>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A73" s="2">
         <v>45359</v>
       </c>
@@ -5273,7 +5287,7 @@
       <c r="F73" s="26"/>
       <c r="G73" s="26"/>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A74" s="2">
         <v>45366</v>
       </c>
@@ -5287,7 +5301,7 @@
         <v>2.09</v>
       </c>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A75" s="2">
         <v>45373</v>
       </c>
@@ -5301,7 +5315,7 @@
         <v>2.19</v>
       </c>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A76" s="2">
         <v>45380</v>
       </c>
@@ -5318,7 +5332,7 @@
       <c r="F76" s="26"/>
       <c r="G76" s="26"/>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A77" s="2">
         <v>45387</v>
       </c>
@@ -5335,7 +5349,7 @@
       <c r="F77" s="26"/>
       <c r="G77" s="26"/>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A78" s="2">
         <v>45394</v>
       </c>
@@ -5352,7 +5366,7 @@
       <c r="F78" s="26"/>
       <c r="G78" s="26"/>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A79" s="2">
         <v>45401</v>
       </c>
@@ -5369,7 +5383,7 @@
       <c r="F79" s="26"/>
       <c r="G79" s="26"/>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A80" s="2">
         <v>45408</v>
       </c>
@@ -5386,7 +5400,7 @@
       <c r="F80" s="26"/>
       <c r="G80" s="26"/>
     </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A81" s="2">
         <v>45415</v>
       </c>
@@ -5401,7 +5415,7 @@
       <c r="F81" s="26"/>
       <c r="G81" s="26"/>
     </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A82" s="2">
         <v>45422</v>
       </c>
@@ -5416,7 +5430,7 @@
       <c r="F82" s="26"/>
       <c r="G82" s="26"/>
     </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A83" s="2">
         <v>45429</v>
       </c>
@@ -5431,7 +5445,7 @@
       <c r="F83" s="26"/>
       <c r="G83" s="26"/>
     </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A84" s="2">
         <v>45436</v>
       </c>
@@ -5446,7 +5460,7 @@
       <c r="F84" s="26"/>
       <c r="G84" s="26"/>
     </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A85" s="2">
         <v>45443</v>
       </c>
@@ -5463,7 +5477,7 @@
       <c r="F85" s="26"/>
       <c r="G85" s="26"/>
     </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A86" s="2">
         <v>45450</v>
       </c>
@@ -5480,7 +5494,7 @@
       <c r="F86" s="26"/>
       <c r="G86" s="26"/>
     </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A87" s="2">
         <v>45457</v>
       </c>
@@ -5497,7 +5511,7 @@
       <c r="F87" s="26"/>
       <c r="G87" s="26"/>
     </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A88" s="2">
         <v>45464</v>
       </c>
@@ -5514,7 +5528,7 @@
       <c r="F88" s="26"/>
       <c r="G88" s="26"/>
     </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A89" s="2">
         <v>45471</v>
       </c>
@@ -5531,7 +5545,7 @@
       <c r="F89" s="26"/>
       <c r="G89" s="26"/>
     </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A90" s="2">
         <v>45478</v>
       </c>
@@ -5548,7 +5562,7 @@
       <c r="F90" s="26"/>
       <c r="G90" s="26"/>
     </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A91" s="2">
         <v>45485</v>
       </c>
@@ -5565,7 +5579,7 @@
       <c r="F91" s="26"/>
       <c r="G91" s="26"/>
     </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A92" s="2">
         <v>45492</v>
       </c>
@@ -5582,7 +5596,7 @@
       <c r="F92" s="26"/>
       <c r="G92" s="26"/>
     </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A93" s="2">
         <v>45499</v>
       </c>
@@ -5599,7 +5613,7 @@
       <c r="F93" s="26"/>
       <c r="G93" s="26"/>
     </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A94" s="2">
         <v>45506</v>
       </c>
@@ -5614,7 +5628,7 @@
       <c r="F94" s="26"/>
       <c r="G94" s="26"/>
     </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A95" s="2">
         <v>45513</v>
       </c>
@@ -5629,7 +5643,7 @@
       <c r="F95" s="26"/>
       <c r="G95" s="26"/>
     </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A96" s="2">
         <v>45520</v>
       </c>
@@ -5644,7 +5658,7 @@
       <c r="F96" s="26"/>
       <c r="G96" s="26"/>
     </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A97" s="2">
         <v>45527</v>
       </c>
@@ -5659,7 +5673,7 @@
       <c r="F97" s="26"/>
       <c r="G97" s="26"/>
     </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A98" s="2">
         <v>45534</v>
       </c>
@@ -5676,7 +5690,7 @@
       <c r="F98" s="26"/>
       <c r="G98" s="26"/>
     </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A99" s="2">
         <v>45541</v>
       </c>
@@ -5693,7 +5707,7 @@
       <c r="F99" s="26"/>
       <c r="G99" s="26"/>
     </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A100" s="2">
         <v>45548</v>
       </c>
@@ -5710,7 +5724,7 @@
       <c r="F100" s="26"/>
       <c r="G100" s="26"/>
     </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A101" s="2">
         <v>45555</v>
       </c>
@@ -5724,7 +5738,7 @@
         <v>2.74</v>
       </c>
     </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A102" s="2">
         <v>45562</v>
       </c>
@@ -5738,7 +5752,7 @@
         <v>2.7970000000000002</v>
       </c>
     </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A103" s="2">
         <v>45569</v>
       </c>
@@ -5752,7 +5766,7 @@
         <v>2.7629999999999999</v>
       </c>
     </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A104" s="2">
         <v>45576</v>
       </c>
@@ -5766,7 +5780,7 @@
         <v>2.7530000000000001</v>
       </c>
     </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A105" s="2">
         <v>45583</v>
       </c>
@@ -5781,7 +5795,7 @@
       </c>
       <c r="E105" s="26"/>
     </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A106" s="2">
         <v>45590</v>
       </c>
@@ -5796,7 +5810,7 @@
       </c>
       <c r="E106" s="26"/>
     </row>
-    <row r="107" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A107" s="2">
         <v>45597</v>
       </c>
@@ -5811,7 +5825,7 @@
       </c>
       <c r="E107" s="26"/>
     </row>
-    <row r="108" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A108" s="2">
         <v>45604</v>
       </c>
@@ -5824,7 +5838,7 @@
       </c>
       <c r="E108" s="26"/>
     </row>
-    <row r="109" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A109" s="2">
         <v>45611</v>
       </c>
@@ -5837,7 +5851,7 @@
       </c>
       <c r="E109" s="26"/>
     </row>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A110" s="2">
         <v>45618</v>
       </c>
@@ -5850,7 +5864,7 @@
       </c>
       <c r="E110" s="26"/>
     </row>
-    <row r="111" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A111" s="2">
         <v>45625</v>
       </c>
@@ -5863,7 +5877,7 @@
       </c>
       <c r="E111" s="26"/>
     </row>
-    <row r="112" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A112" s="2">
         <v>45632</v>
       </c>
@@ -5878,7 +5892,7 @@
         <v>2.3769999999999998</v>
       </c>
     </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A113" s="2">
         <v>45639</v>
       </c>
@@ -5893,7 +5907,7 @@
         <v>2.2909999999999999</v>
       </c>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A114" s="2">
         <v>45646</v>
       </c>
@@ -5908,7 +5922,7 @@
         <v>2.1269999999999998</v>
       </c>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A115" s="2">
         <v>45653</v>
       </c>
@@ -5923,7 +5937,7 @@
         <v>2.0819999999999999</v>
       </c>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A116" s="2">
         <v>45660</v>
       </c>
@@ -5937,7 +5951,7 @@
         <v>2.2080000000000002</v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A117" s="2">
         <v>45667</v>
       </c>
@@ -5951,7 +5965,7 @@
         <v>2.738</v>
       </c>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A118" s="2">
         <v>45674</v>
       </c>
@@ -5965,7 +5979,7 @@
         <v>2.9994999999999998</v>
       </c>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A119" s="2">
         <v>45681</v>
       </c>
@@ -5979,7 +5993,7 @@
         <v>2.9994999999999998</v>
       </c>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A120" s="2">
         <v>45688</v>
       </c>
@@ -5993,7 +6007,7 @@
         <v>2.915</v>
       </c>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A121" s="2">
         <v>45695</v>
       </c>
@@ -6004,7 +6018,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A122" s="2">
         <v>45702</v>
       </c>
@@ -6015,7 +6029,7 @@
         <v>3.0150000000000001</v>
       </c>
     </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A123" s="2">
         <v>45709</v>
       </c>
@@ -6026,7 +6040,7 @@
         <v>2.9460000000000002</v>
       </c>
     </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A124" s="2">
         <v>45716</v>
       </c>
@@ -6040,7 +6054,7 @@
         <v>2.8490000000000002</v>
       </c>
     </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A125" s="2">
         <v>45723</v>
       </c>
@@ -6054,7 +6068,7 @@
         <v>2.5750000000000002</v>
       </c>
     </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A126" s="2">
         <v>45730</v>
       </c>
@@ -6068,7 +6082,7 @@
         <v>2.6579999999999999</v>
       </c>
     </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A127" s="2">
         <v>45737</v>
       </c>
@@ -6082,7 +6096,7 @@
         <v>2.641</v>
       </c>
     </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A128" s="2">
         <v>45744</v>
       </c>
@@ -6096,7 +6110,7 @@
         <v>2.629</v>
       </c>
     </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A129" s="2">
         <v>45751</v>
       </c>
@@ -6110,7 +6124,7 @@
         <v>2.4380000000000002</v>
       </c>
     </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A130" s="2">
         <v>45758</v>
       </c>
@@ -6124,7 +6138,7 @@
         <v>2.6179999999999999</v>
       </c>
     </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A131" s="2">
         <v>45765</v>
       </c>
@@ -6138,7 +6152,7 @@
         <v>2.605</v>
       </c>
     </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A132" s="2">
         <v>45772</v>
       </c>
@@ -6152,7 +6166,7 @@
         <v>2.7149999999999999</v>
       </c>
     </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A133" s="2">
         <v>45779</v>
       </c>
@@ -6166,7 +6180,7 @@
         <v>2.335</v>
       </c>
     </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A134" s="2">
         <v>45786</v>
       </c>
@@ -6177,7 +6191,7 @@
         <v>2.4249999999999998</v>
       </c>
     </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A135" s="2">
         <v>45793</v>
       </c>
@@ -6188,7 +6202,7 @@
         <v>2.3460000000000001</v>
       </c>
     </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A136" s="2">
         <v>45800</v>
       </c>
@@ -6199,7 +6213,7 @@
         <v>2.4289999999999998</v>
       </c>
     </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A137" s="2">
         <v>45807</v>
       </c>
@@ -6213,7 +6227,7 @@
         <v>2.5379999999999998</v>
       </c>
     </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A138" s="2">
         <v>45814</v>
       </c>
@@ -6227,7 +6241,7 @@
         <v>2.3980000000000001</v>
       </c>
     </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A139" s="2">
         <v>45821</v>
       </c>
@@ -6241,7 +6255,7 @@
         <v>2.504</v>
       </c>
     </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A140" s="2">
         <v>45828</v>
       </c>
@@ -6256,7 +6270,7 @@
         <v>2.0609999999999999</v>
       </c>
     </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A141" s="2">
         <v>45835</v>
       </c>
@@ -6271,7 +6285,7 @@
         <v>1.917</v>
       </c>
     </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A142" s="2">
         <v>45842</v>
       </c>
@@ -6285,7 +6299,7 @@
         <v>1.7809999999999999</v>
       </c>
     </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A143" s="2">
         <v>45849</v>
       </c>
@@ -6300,7 +6314,7 @@
       </c>
       <c r="E143" s="26"/>
     </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A144" s="2">
         <v>45856</v>
       </c>
@@ -6315,7 +6329,7 @@
       </c>
       <c r="E144" s="26"/>
     </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A145" s="2">
         <v>45863</v>
       </c>
@@ -6330,7 +6344,7 @@
       </c>
       <c r="E145" s="26"/>
     </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A146" s="2">
         <v>45870</v>
       </c>
@@ -6345,7 +6359,7 @@
       </c>
       <c r="E146" s="26"/>
     </row>
-    <row r="147" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A147" s="2">
         <v>45877</v>
       </c>
@@ -6358,7 +6372,7 @@
       </c>
       <c r="E147" s="26"/>
     </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A148" s="2">
         <v>45884</v>
       </c>
@@ -6371,7 +6385,7 @@
       </c>
       <c r="E148" s="26"/>
     </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A149" s="2">
         <v>45891</v>
       </c>
@@ -6384,7 +6398,7 @@
       </c>
       <c r="E149" s="26"/>
     </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A150" s="2">
         <v>45898</v>
       </c>
@@ -6399,7 +6413,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A151" s="2">
         <v>45905</v>
       </c>
@@ -6414,7 +6428,7 @@
         <v>2.2799999999999998</v>
       </c>
     </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A152" s="2">
         <v>45912</v>
       </c>
@@ -6429,7 +6443,7 @@
         <v>2.16</v>
       </c>
     </row>
-    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A153" s="2">
         <v>45919</v>
       </c>
@@ -6443,7 +6457,7 @@
         <v>2.1800000000000002</v>
       </c>
     </row>
-    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A154" s="2">
         <v>45926</v>
       </c>
@@ -6457,7 +6471,7 @@
         <v>2.46</v>
       </c>
     </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A155" s="2">
         <v>45933</v>
       </c>
@@ -6471,7 +6485,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A156" s="2">
         <v>45940</v>
       </c>
@@ -6485,7 +6499,7 @@
         <v>2.23</v>
       </c>
     </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A157" s="2">
         <v>45947</v>
       </c>
@@ -6499,7 +6513,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A158" s="2">
         <v>45954</v>
       </c>
@@ -6513,7 +6527,7 @@
         <v>2.2599999999999998</v>
       </c>
     </row>
-    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A159" s="2">
         <v>45961</v>
       </c>
@@ -6527,7 +6541,7 @@
         <v>2.2599999999999998</v>
       </c>
     </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A160" s="2">
         <v>45968</v>
       </c>
@@ -6541,7 +6555,7 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A161" s="2">
         <v>45975</v>
       </c>
@@ -6555,7 +6569,7 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A162" s="2">
         <v>45982</v>
       </c>
@@ -6569,7 +6583,7 @@
         <v>2.31</v>
       </c>
     </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A163" s="2">
         <v>45989</v>
       </c>
@@ -6586,7 +6600,7 @@
         <v>2.66</v>
       </c>
     </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A164" s="2">
         <v>45996</v>
       </c>
@@ -6600,7 +6614,7 @@
         <v>2.2200000000000002</v>
       </c>
     </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A165" s="2">
         <v>46003</v>
       </c>
@@ -6614,7 +6628,7 @@
         <v>2.2400000000000002</v>
       </c>
     </row>
-    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A166" s="2">
         <v>46010</v>
       </c>
@@ -6628,7 +6642,7 @@
         <v>2.11</v>
       </c>
     </row>
-    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A167" s="2">
         <v>46017</v>
       </c>
@@ -6642,7 +6656,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A168" s="2">
         <v>46024</v>
       </c>
@@ -6656,7 +6670,7 @@
         <v>2.17</v>
       </c>
     </row>
-    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A169" s="2">
         <v>46031</v>
       </c>
@@ -6670,7 +6684,7 @@
         <v>2.61</v>
       </c>
     </row>
-    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A170" s="2">
         <v>46038</v>
       </c>
@@ -6684,7 +6698,7 @@
         <v>2.75</v>
       </c>
     </row>
-    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A171" s="2">
         <v>46045</v>
       </c>
@@ -6698,7 +6712,7 @@
         <v>2.73</v>
       </c>
     </row>
-    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A172" s="2">
         <v>46052</v>
       </c>
@@ -6712,7 +6726,7 @@
         <v>2.73</v>
       </c>
     </row>
-    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A173" s="2">
         <v>46059</v>
       </c>
@@ -6726,7 +6740,7 @@
         <v>2.59</v>
       </c>
     </row>
-    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A174" s="2">
         <v>46066</v>
       </c>
@@ -6740,7 +6754,7 @@
         <v>2.63</v>
       </c>
     </row>
-    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A175" s="2">
         <v>46073</v>
       </c>
@@ -6754,7 +6768,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="176" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A176" s="2">
         <v>46080</v>
       </c>
@@ -6765,7 +6779,7 @@
         <v>2.38</v>
       </c>
     </row>
-    <row r="177" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A177" s="2">
         <v>46087</v>
       </c>
@@ -6776,7 +6790,7 @@
         <v>2.23</v>
       </c>
     </row>
-    <row r="178" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A178" s="2">
         <v>46094</v>
       </c>
@@ -6790,7 +6804,7 @@
         <v>2.68</v>
       </c>
     </row>
-    <row r="179" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A179" s="2">
         <v>46101</v>
       </c>
@@ -6804,7 +6818,7 @@
         <v>2.67</v>
       </c>
     </row>
-    <row r="180" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A180" s="2">
         <v>46108</v>
       </c>
@@ -6818,7 +6832,7 @@
         <v>2.68</v>
       </c>
     </row>
-    <row r="181" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A181" s="2">
         <v>46115</v>
       </c>
@@ -6832,7 +6846,7 @@
         <v>2.82</v>
       </c>
     </row>
-    <row r="182" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A182" s="2">
         <v>46122</v>
       </c>
@@ -6846,7 +6860,7 @@
         <v>2.6</v>
       </c>
     </row>
-    <row r="183" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A183" s="2">
         <v>46129</v>
       </c>
@@ -6860,7 +6874,7 @@
         <v>2.75</v>
       </c>
     </row>
-    <row r="184" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A184" s="2">
         <v>46136</v>
       </c>
@@ -6874,7 +6888,7 @@
         <v>2.81</v>
       </c>
     </row>
-    <row r="185" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A185" s="2">
         <v>46143</v>
       </c>
@@ -6888,7 +6902,7 @@
         <v>2.52</v>
       </c>
     </row>
-    <row r="186" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A186" s="2">
         <v>46150</v>
       </c>
@@ -6899,7 +6913,7 @@
         <v>2.59</v>
       </c>
     </row>
-    <row r="187" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A187" s="2">
         <v>46157</v>
       </c>
@@ -6910,7 +6924,7 @@
         <v>2.61</v>
       </c>
     </row>
-    <row r="188" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A188" s="2">
         <v>46164</v>
       </c>
@@ -6921,7 +6935,7 @@
         <v>2.61</v>
       </c>
     </row>
-    <row r="189" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A189" s="2">
         <v>46171</v>
       </c>
@@ -6935,7 +6949,7 @@
         <v>2.36</v>
       </c>
     </row>
-    <row r="190" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A190" s="2">
         <v>46178</v>
       </c>
@@ -6949,7 +6963,7 @@
         <v>2.4700000000000002</v>
       </c>
     </row>
-    <row r="191" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A191" s="2">
         <v>46185</v>
       </c>
@@ -6963,7 +6977,7 @@
         <v>2.46</v>
       </c>
     </row>
-    <row r="192" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A192" s="2">
         <v>46192</v>
       </c>
@@ -6977,7 +6991,7 @@
         <v>2.4500000000000002</v>
       </c>
     </row>
-    <row r="193" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A193" s="2">
         <v>46199</v>
       </c>
@@ -6991,7 +7005,7 @@
         <v>2.42</v>
       </c>
     </row>
-    <row r="194" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A194" s="2">
         <v>46206</v>
       </c>
@@ -7005,7 +7019,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="195" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A195" s="2">
         <v>46213</v>
       </c>
@@ -7019,7 +7033,7 @@
         <v>2.36</v>
       </c>
     </row>
-    <row r="196" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A196" s="2">
         <v>46220</v>
       </c>
@@ -7033,7 +7047,7 @@
         <v>2.6</v>
       </c>
     </row>
-    <row r="197" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A197" s="2">
         <v>46227</v>
       </c>
@@ -7047,7 +7061,7 @@
         <v>2.62</v>
       </c>
     </row>
-    <row r="198" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A198" s="2">
         <v>46234</v>
       </c>
@@ -7061,7 +7075,7 @@
         <v>2.52</v>
       </c>
     </row>
-    <row r="199" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A199" s="2">
         <v>46241</v>
       </c>
@@ -7072,7 +7086,7 @@
         <v>2.2400000000000002</v>
       </c>
     </row>
-    <row r="200" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A200" s="2">
         <v>46248</v>
       </c>
@@ -7083,7 +7097,7 @@
         <v>2.14</v>
       </c>
     </row>
-    <row r="201" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A201" s="2">
         <v>46255</v>
       </c>
@@ -7094,7 +7108,7 @@
         <v>2.27</v>
       </c>
     </row>
-    <row r="202" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A202" s="2">
         <v>46262</v>
       </c>
@@ -7105,7 +7119,7 @@
         <v>2.2200000000000002</v>
       </c>
     </row>
-    <row r="203" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A203" s="2">
         <v>46269</v>
       </c>
@@ -7119,7 +7133,7 @@
         <v>2.5099999999999998</v>
       </c>
     </row>
-    <row r="204" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A204" s="2">
         <v>46276</v>
       </c>
@@ -7133,7 +7147,7 @@
         <v>2.5099999999999998</v>
       </c>
     </row>
-    <row r="205" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A205" s="2">
         <v>46283</v>
       </c>
@@ -7147,7 +7161,7 @@
         <v>2.6</v>
       </c>
     </row>
-    <row r="206" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A206" s="2">
         <v>46290</v>
       </c>
@@ -7161,7 +7175,7 @@
         <v>2.6</v>
       </c>
     </row>
-    <row r="207" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A207" s="2">
         <v>46297</v>
       </c>
@@ -7175,7 +7189,7 @@
         <v>2.54</v>
       </c>
     </row>
-    <row r="208" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A208" s="2">
         <v>46304</v>
       </c>
@@ -7189,7 +7203,7 @@
         <v>2.83</v>
       </c>
     </row>
-    <row r="209" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A209" s="2">
         <v>46311</v>
       </c>
@@ -7203,7 +7217,7 @@
         <v>2.82</v>
       </c>
     </row>
-    <row r="210" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A210" s="2">
         <v>46318</v>
       </c>
@@ -7215,6 +7229,20 @@
       </c>
       <c r="E210">
         <v>2.81</v>
+      </c>
+    </row>
+    <row r="211" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A211" s="2">
+        <v>46325</v>
+      </c>
+      <c r="B211" t="s">
+        <v>61</v>
+      </c>
+      <c r="D211">
+        <v>2.67</v>
+      </c>
+      <c r="E211">
+        <v>2.9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>